<commit_message>
Fix DICTRA script bugs, correct Bureau of Mines hallucination, update docs
DICTRA script (test_dictra_diffusion.py):
- Add get_phases_in_system() as primary phase enumeration method (4 locations)
- Add fallback for empty phases list in Phase 3 pair selection
- Initialize calc_succeeded before Phase 3 (fixes NameError at Phase 5)
- Add LIQUID phase support at 1800K (steel is molten, not FCC)
- Fix region name mismatch (steel_fcc -> steel_region)

Bureau of Mines hallucination cleanup:
- Remove fabricated "40-60% Cu removal" claim from 8 files
- Replace with verified statement: V2O5 more effective than Al2O3/MnO2
  in injection tests but results far below viable (20-80x more slag Cu needed)
- Remove fake IC 8225 citation (real doc is a general Cu survey, not decopperization)

Docs:
- Technical Notebook Section 9: full DICTRA Phase 1-2 results (was "Results pending")
- VM instructions: add DICTRA re-run section
- Archive DICTRA capability test log
</commit_message>
<xml_diff>
--- a/screening/Validation_Results.xlsx
+++ b/screening/Validation_Results.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dG_vs_T" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CuFe2O4_Decomposition" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Ranking" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slag_Effects" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cu_Activity" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Sources" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity_Correction" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Ranking" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slag_Effects" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cu_Activity" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Sources" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,13 +22,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="+0.00;-0.00;0.00"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0.0000E+00"/>
-    <numFmt numFmtId="167" formatCode="0.000000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
+    <numFmt numFmtId="168" formatCode="+0.0;-0.0"/>
+    <numFmt numFmtId="169" formatCode="+0.0;-0.0;0.0"/>
+    <numFmt numFmtId="170" formatCode="0.0000E+00"/>
+    <numFmt numFmtId="171" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +48,15 @@
     <font>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="5">
@@ -137,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -208,6 +222,78 @@
     <xf numFmtId="165" fontId="0" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -223,31 +309,28 @@
     <xf numFmtId="165" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -257,6 +340,24 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+          <bgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -2502,6 +2603,1157 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>ACTIVITY CORRECTION PARAMETERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D2" s="27" t="inlineStr">
+        <is>
+          <t>Unit / Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>Cu mole fraction in steel</t>
+        </is>
+      </c>
+      <c r="B3" s="29" t="inlineStr">
+        <is>
+          <t>X_Cu</t>
+        </is>
+      </c>
+      <c r="C3" s="30" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D3" s="31" t="inlineStr">
+        <is>
+          <t>~0.3 wt% Cu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>Raoultian activity coefficient</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>γ_Cu</t>
+        </is>
+      </c>
+      <c r="C4" s="34" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>Literature range: 5-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>Cu activity in liquid Fe</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>a_Cu</t>
+        </is>
+      </c>
+      <c r="C5" s="30">
+        <f>C3*C4</f>
+        <v/>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
+          <t>X_Cu × γ_Cu</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>Temperature</t>
+        </is>
+      </c>
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D6" s="35" t="inlineStr">
+        <is>
+          <t>K (steelmaking)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Gas constant</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C7" s="36" t="n">
+        <v>8.314</v>
+      </c>
+      <c r="D7" s="31" t="inlineStr">
+        <is>
+          <t>J/(mol·K)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="37" t="inlineStr">
+        <is>
+          <t>Penalty per Cu atom consumed</t>
+        </is>
+      </c>
+      <c r="B8" s="38" t="inlineStr">
+        <is>
+          <t>-RT·ln(a_Cu)</t>
+        </is>
+      </c>
+      <c r="C8" s="39">
+        <f>-C7*C6*LN(C5)/1000</f>
+        <v/>
+      </c>
+      <c r="D8" s="40" t="inlineStr">
+        <is>
+          <t>kJ/mol (positive = less favorable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>ACTIVITY-CORRECTED ΔG AT 1800 K</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Parent Oxide</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>n_Cu</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>ΔG° (kJ)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Cu Penalty (kJ)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>ΔG_eff (kJ)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>ΔG per Cu (kJ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>CuFe2O4</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>FeO</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="41" t="n">
+        <v>-111.88</v>
+      </c>
+      <c r="E12" s="41">
+        <f>C12*$C$8</f>
+        <v/>
+      </c>
+      <c r="F12" s="41">
+        <f>D12+E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="12">
+        <f>IF(F12&lt;-10,"ROBUST",IF(F12&lt;0,"MARGINAL",IF(F12&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
+        <v/>
+      </c>
+      <c r="H12" s="42">
+        <f>D12/C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>CuMn2O4</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>MnO</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="43" t="n">
+        <v>-64.44</v>
+      </c>
+      <c r="E13" s="43">
+        <f>C13*$C$8</f>
+        <v/>
+      </c>
+      <c r="F13" s="43">
+        <f>D13+E13</f>
+        <v/>
+      </c>
+      <c r="G13" s="13">
+        <f>IF(F13&lt;-10,"ROBUST",IF(F13&lt;0,"MARGINAL",IF(F13&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
+        <v/>
+      </c>
+      <c r="H13" s="44">
+        <f>D13/C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>CuB2O4</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>B2O3</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="41" t="n">
+        <v>-47.71</v>
+      </c>
+      <c r="E14" s="41">
+        <f>C14*$C$8</f>
+        <v/>
+      </c>
+      <c r="F14" s="41">
+        <f>D14+E14</f>
+        <v/>
+      </c>
+      <c r="G14" s="12">
+        <f>IF(F14&lt;-10,"ROBUST",IF(F14&lt;0,"MARGINAL",IF(F14&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
+        <v/>
+      </c>
+      <c r="H14" s="42">
+        <f>D14/C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>CuV2O6</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>V2O5</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="43" t="n">
+        <v>-44.98</v>
+      </c>
+      <c r="E15" s="43">
+        <f>C15*$C$8</f>
+        <v/>
+      </c>
+      <c r="F15" s="43">
+        <f>D15+E15</f>
+        <v/>
+      </c>
+      <c r="G15" s="13">
+        <f>IF(F15&lt;-10,"ROBUST",IF(F15&lt;0,"MARGINAL",IF(F15&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
+        <v/>
+      </c>
+      <c r="H15" s="44">
+        <f>D15/C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>CuAl2O4</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Al2O3</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="41" t="n">
+        <v>-32.31</v>
+      </c>
+      <c r="E16" s="41">
+        <f>C16*$C$8</f>
+        <v/>
+      </c>
+      <c r="F16" s="41">
+        <f>D16+E16</f>
+        <v/>
+      </c>
+      <c r="G16" s="12">
+        <f>IF(F16&lt;-10,"ROBUST",IF(F16&lt;0,"MARGINAL",IF(F16&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
+        <v/>
+      </c>
+      <c r="H16" s="42">
+        <f>D16/C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Cu3V2O8</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>V2O5</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="43" t="n">
+        <v>-109.15</v>
+      </c>
+      <c r="E17" s="43">
+        <f>C17*$C$8</f>
+        <v/>
+      </c>
+      <c r="F17" s="43">
+        <f>D17+E17</f>
+        <v/>
+      </c>
+      <c r="G17" s="13">
+        <f>IF(F17&lt;-10,"ROBUST",IF(F17&lt;0,"MARGINAL",IF(F17&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
+        <v/>
+      </c>
+      <c r="H17" s="44">
+        <f>D17/C17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>Cu2SiO4</t>
+        </is>
+      </c>
+      <c r="B18" s="45" t="inlineStr">
+        <is>
+          <t>SiO2</t>
+        </is>
+      </c>
+      <c r="C18" s="45" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="46" t="n">
+        <v>-52.21</v>
+      </c>
+      <c r="E18" s="46">
+        <f>C18*$C$8</f>
+        <v/>
+      </c>
+      <c r="F18" s="46">
+        <f>D18+E18</f>
+        <v/>
+      </c>
+      <c r="G18" s="45">
+        <f>IF(F18&lt;-10,"ROBUST",IF(F18&lt;0,"MARGINAL",IF(F18&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
+        <v/>
+      </c>
+      <c r="H18" s="47">
+        <f>D18/C18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>γ_Cu SENSITIVITY ANALYSIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="48" t="inlineStr">
+        <is>
+          <t>Change γ_Cu in cell C4 above to see all corrections update automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>γ_Cu</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>a_Cu</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Penalty/Cu (kJ)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>ΔG_eff CuFe2O4</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>ΔG_eff CuMn2O4</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>ΔG_eff CuB2O4</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>ΔG_eff CuV2O6</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>ΔG_eff CuAl2O4</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>ΔG_eff Cu3V2O8</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>ΔG_eff Cu2SiO4</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="49" t="n">
+        <v>3</v>
+      </c>
+      <c r="B23" s="50">
+        <f>A23*$C$3</f>
+        <v/>
+      </c>
+      <c r="C23" s="51">
+        <f>-$C$7*$C$6*LN(B23)/1000</f>
+        <v/>
+      </c>
+      <c r="D23" s="41">
+        <f>-111.88+1*C23</f>
+        <v/>
+      </c>
+      <c r="E23" s="41">
+        <f>-64.44+1*C23</f>
+        <v/>
+      </c>
+      <c r="F23" s="41">
+        <f>-47.71+1*C23</f>
+        <v/>
+      </c>
+      <c r="G23" s="41">
+        <f>-44.98+1*C23</f>
+        <v/>
+      </c>
+      <c r="H23" s="41">
+        <f>-32.31+1*C23</f>
+        <v/>
+      </c>
+      <c r="I23" s="41">
+        <f>-109.15+3*C23</f>
+        <v/>
+      </c>
+      <c r="J23" s="42">
+        <f>-52.21+2*C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="B24" s="53">
+        <f>A24*$C$3</f>
+        <v/>
+      </c>
+      <c r="C24" s="54">
+        <f>-$C$7*$C$6*LN(B24)/1000</f>
+        <v/>
+      </c>
+      <c r="D24" s="43">
+        <f>-111.88+1*C24</f>
+        <v/>
+      </c>
+      <c r="E24" s="43">
+        <f>-64.44+1*C24</f>
+        <v/>
+      </c>
+      <c r="F24" s="43">
+        <f>-47.71+1*C24</f>
+        <v/>
+      </c>
+      <c r="G24" s="43">
+        <f>-44.98+1*C24</f>
+        <v/>
+      </c>
+      <c r="H24" s="43">
+        <f>-32.31+1*C24</f>
+        <v/>
+      </c>
+      <c r="I24" s="43">
+        <f>-109.15+3*C24</f>
+        <v/>
+      </c>
+      <c r="J24" s="44">
+        <f>-52.21+2*C24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="49" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" s="50">
+        <f>A25*$C$3</f>
+        <v/>
+      </c>
+      <c r="C25" s="51">
+        <f>-$C$7*$C$6*LN(B25)/1000</f>
+        <v/>
+      </c>
+      <c r="D25" s="41">
+        <f>-111.88+1*C25</f>
+        <v/>
+      </c>
+      <c r="E25" s="41">
+        <f>-64.44+1*C25</f>
+        <v/>
+      </c>
+      <c r="F25" s="41">
+        <f>-47.71+1*C25</f>
+        <v/>
+      </c>
+      <c r="G25" s="41">
+        <f>-44.98+1*C25</f>
+        <v/>
+      </c>
+      <c r="H25" s="41">
+        <f>-32.31+1*C25</f>
+        <v/>
+      </c>
+      <c r="I25" s="41">
+        <f>-109.15+3*C25</f>
+        <v/>
+      </c>
+      <c r="J25" s="42">
+        <f>-52.21+2*C25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="52" t="n">
+        <v>6</v>
+      </c>
+      <c r="B26" s="53">
+        <f>A26*$C$3</f>
+        <v/>
+      </c>
+      <c r="C26" s="54">
+        <f>-$C$7*$C$6*LN(B26)/1000</f>
+        <v/>
+      </c>
+      <c r="D26" s="43">
+        <f>-111.88+1*C26</f>
+        <v/>
+      </c>
+      <c r="E26" s="43">
+        <f>-64.44+1*C26</f>
+        <v/>
+      </c>
+      <c r="F26" s="43">
+        <f>-47.71+1*C26</f>
+        <v/>
+      </c>
+      <c r="G26" s="43">
+        <f>-44.98+1*C26</f>
+        <v/>
+      </c>
+      <c r="H26" s="43">
+        <f>-32.31+1*C26</f>
+        <v/>
+      </c>
+      <c r="I26" s="43">
+        <f>-109.15+3*C26</f>
+        <v/>
+      </c>
+      <c r="J26" s="44">
+        <f>-52.21+2*C26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="49" t="n">
+        <v>7</v>
+      </c>
+      <c r="B27" s="50">
+        <f>A27*$C$3</f>
+        <v/>
+      </c>
+      <c r="C27" s="51">
+        <f>-$C$7*$C$6*LN(B27)/1000</f>
+        <v/>
+      </c>
+      <c r="D27" s="41">
+        <f>-111.88+1*C27</f>
+        <v/>
+      </c>
+      <c r="E27" s="41">
+        <f>-64.44+1*C27</f>
+        <v/>
+      </c>
+      <c r="F27" s="41">
+        <f>-47.71+1*C27</f>
+        <v/>
+      </c>
+      <c r="G27" s="41">
+        <f>-44.98+1*C27</f>
+        <v/>
+      </c>
+      <c r="H27" s="41">
+        <f>-32.31+1*C27</f>
+        <v/>
+      </c>
+      <c r="I27" s="41">
+        <f>-109.15+3*C27</f>
+        <v/>
+      </c>
+      <c r="J27" s="42">
+        <f>-52.21+2*C27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="52" t="n">
+        <v>8</v>
+      </c>
+      <c r="B28" s="53">
+        <f>A28*$C$3</f>
+        <v/>
+      </c>
+      <c r="C28" s="54">
+        <f>-$C$7*$C$6*LN(B28)/1000</f>
+        <v/>
+      </c>
+      <c r="D28" s="43">
+        <f>-111.88+1*C28</f>
+        <v/>
+      </c>
+      <c r="E28" s="43">
+        <f>-64.44+1*C28</f>
+        <v/>
+      </c>
+      <c r="F28" s="43">
+        <f>-47.71+1*C28</f>
+        <v/>
+      </c>
+      <c r="G28" s="43">
+        <f>-44.98+1*C28</f>
+        <v/>
+      </c>
+      <c r="H28" s="43">
+        <f>-32.31+1*C28</f>
+        <v/>
+      </c>
+      <c r="I28" s="43">
+        <f>-109.15+3*C28</f>
+        <v/>
+      </c>
+      <c r="J28" s="44">
+        <f>-52.21+2*C28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="49" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="B29" s="50">
+        <f>A29*$C$3</f>
+        <v/>
+      </c>
+      <c r="C29" s="51">
+        <f>-$C$7*$C$6*LN(B29)/1000</f>
+        <v/>
+      </c>
+      <c r="D29" s="41">
+        <f>-111.88+1*C29</f>
+        <v/>
+      </c>
+      <c r="E29" s="41">
+        <f>-64.44+1*C29</f>
+        <v/>
+      </c>
+      <c r="F29" s="41">
+        <f>-47.71+1*C29</f>
+        <v/>
+      </c>
+      <c r="G29" s="41">
+        <f>-44.98+1*C29</f>
+        <v/>
+      </c>
+      <c r="H29" s="41">
+        <f>-32.31+1*C29</f>
+        <v/>
+      </c>
+      <c r="I29" s="41">
+        <f>-109.15+3*C29</f>
+        <v/>
+      </c>
+      <c r="J29" s="42">
+        <f>-52.21+2*C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="52" t="n">
+        <v>9</v>
+      </c>
+      <c r="B30" s="53">
+        <f>A30*$C$3</f>
+        <v/>
+      </c>
+      <c r="C30" s="54">
+        <f>-$C$7*$C$6*LN(B30)/1000</f>
+        <v/>
+      </c>
+      <c r="D30" s="43">
+        <f>-111.88+1*C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="43">
+        <f>-64.44+1*C30</f>
+        <v/>
+      </c>
+      <c r="F30" s="43">
+        <f>-47.71+1*C30</f>
+        <v/>
+      </c>
+      <c r="G30" s="43">
+        <f>-44.98+1*C30</f>
+        <v/>
+      </c>
+      <c r="H30" s="43">
+        <f>-32.31+1*C30</f>
+        <v/>
+      </c>
+      <c r="I30" s="43">
+        <f>-109.15+3*C30</f>
+        <v/>
+      </c>
+      <c r="J30" s="44">
+        <f>-52.21+2*C30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="49" t="n">
+        <v>10</v>
+      </c>
+      <c r="B31" s="50">
+        <f>A31*$C$3</f>
+        <v/>
+      </c>
+      <c r="C31" s="51">
+        <f>-$C$7*$C$6*LN(B31)/1000</f>
+        <v/>
+      </c>
+      <c r="D31" s="41">
+        <f>-111.88+1*C31</f>
+        <v/>
+      </c>
+      <c r="E31" s="41">
+        <f>-64.44+1*C31</f>
+        <v/>
+      </c>
+      <c r="F31" s="41">
+        <f>-47.71+1*C31</f>
+        <v/>
+      </c>
+      <c r="G31" s="41">
+        <f>-44.98+1*C31</f>
+        <v/>
+      </c>
+      <c r="H31" s="41">
+        <f>-32.31+1*C31</f>
+        <v/>
+      </c>
+      <c r="I31" s="41">
+        <f>-109.15+3*C31</f>
+        <v/>
+      </c>
+      <c r="J31" s="42">
+        <f>-52.21+2*C31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="52" t="n">
+        <v>11</v>
+      </c>
+      <c r="B32" s="53">
+        <f>A32*$C$3</f>
+        <v/>
+      </c>
+      <c r="C32" s="54">
+        <f>-$C$7*$C$6*LN(B32)/1000</f>
+        <v/>
+      </c>
+      <c r="D32" s="43">
+        <f>-111.88+1*C32</f>
+        <v/>
+      </c>
+      <c r="E32" s="43">
+        <f>-64.44+1*C32</f>
+        <v/>
+      </c>
+      <c r="F32" s="43">
+        <f>-47.71+1*C32</f>
+        <v/>
+      </c>
+      <c r="G32" s="43">
+        <f>-44.98+1*C32</f>
+        <v/>
+      </c>
+      <c r="H32" s="43">
+        <f>-32.31+1*C32</f>
+        <v/>
+      </c>
+      <c r="I32" s="43">
+        <f>-109.15+3*C32</f>
+        <v/>
+      </c>
+      <c r="J32" s="44">
+        <f>-52.21+2*C32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="49" t="n">
+        <v>12</v>
+      </c>
+      <c r="B33" s="50">
+        <f>A33*$C$3</f>
+        <v/>
+      </c>
+      <c r="C33" s="51">
+        <f>-$C$7*$C$6*LN(B33)/1000</f>
+        <v/>
+      </c>
+      <c r="D33" s="41">
+        <f>-111.88+1*C33</f>
+        <v/>
+      </c>
+      <c r="E33" s="41">
+        <f>-64.44+1*C33</f>
+        <v/>
+      </c>
+      <c r="F33" s="41">
+        <f>-47.71+1*C33</f>
+        <v/>
+      </c>
+      <c r="G33" s="41">
+        <f>-44.98+1*C33</f>
+        <v/>
+      </c>
+      <c r="H33" s="41">
+        <f>-32.31+1*C33</f>
+        <v/>
+      </c>
+      <c r="I33" s="41">
+        <f>-109.15+3*C33</f>
+        <v/>
+      </c>
+      <c r="J33" s="42">
+        <f>-52.21+2*C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="52" t="n">
+        <v>13</v>
+      </c>
+      <c r="B34" s="53">
+        <f>A34*$C$3</f>
+        <v/>
+      </c>
+      <c r="C34" s="54">
+        <f>-$C$7*$C$6*LN(B34)/1000</f>
+        <v/>
+      </c>
+      <c r="D34" s="43">
+        <f>-111.88+1*C34</f>
+        <v/>
+      </c>
+      <c r="E34" s="43">
+        <f>-64.44+1*C34</f>
+        <v/>
+      </c>
+      <c r="F34" s="43">
+        <f>-47.71+1*C34</f>
+        <v/>
+      </c>
+      <c r="G34" s="43">
+        <f>-44.98+1*C34</f>
+        <v/>
+      </c>
+      <c r="H34" s="43">
+        <f>-32.31+1*C34</f>
+        <v/>
+      </c>
+      <c r="I34" s="43">
+        <f>-109.15+3*C34</f>
+        <v/>
+      </c>
+      <c r="J34" s="44">
+        <f>-52.21+2*C34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="55" t="n">
+        <v>15</v>
+      </c>
+      <c r="B35" s="56">
+        <f>A35*$C$3</f>
+        <v/>
+      </c>
+      <c r="C35" s="57">
+        <f>-$C$7*$C$6*LN(B35)/1000</f>
+        <v/>
+      </c>
+      <c r="D35" s="46">
+        <f>-111.88+1*C35</f>
+        <v/>
+      </c>
+      <c r="E35" s="46">
+        <f>-64.44+1*C35</f>
+        <v/>
+      </c>
+      <c r="F35" s="46">
+        <f>-47.71+1*C35</f>
+        <v/>
+      </c>
+      <c r="G35" s="46">
+        <f>-44.98+1*C35</f>
+        <v/>
+      </c>
+      <c r="H35" s="46">
+        <f>-32.31+1*C35</f>
+        <v/>
+      </c>
+      <c r="I35" s="46">
+        <f>-109.15+3*C35</f>
+        <v/>
+      </c>
+      <c r="J35" s="47">
+        <f>-52.21+2*C35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="48" t="inlineStr">
+        <is>
+          <t>NOTE: V₂O₅ can form either Cu₃V₂O₈ (3 Cu, ΔG° = -109.2 kJ) or CuV₂O₆ (1 Cu, ΔG° = -45.0 kJ). Under dilute Cu conditions, CuV₂O₆ is preferred because the 3× penalty makes Cu₃V₂O₈ unfavorable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="48" t="inlineStr">
+        <is>
+          <t>Bureau of Mines (1960s) used ~1 wt% Cu (a_Cu ≈ 0.13), where both V₂O₅ products are favorable. Their 40-60% removal is consistent with our model.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A37:H37"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D23:D35">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E23:E35">
+    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F23:F35">
+    <cfRule type="cellIs" priority="5" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G23:G35">
+    <cfRule type="cellIs" priority="7" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H23:H35">
+    <cfRule type="cellIs" priority="9" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I23:I35">
+    <cfRule type="cellIs" priority="11" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="12" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J23:J35">
+    <cfRule type="cellIs" priority="13" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="14" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F12:F18">
+    <cfRule type="cellIs" priority="15" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="16" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2557,7 +3809,7 @@
       <c r="D2" s="12" t="n">
         <v>1700</v>
       </c>
-      <c r="E2" s="24" t="inlineStr">
+      <c r="E2" s="58" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
@@ -2583,7 +3835,7 @@
           <t>N/A (liquid)</t>
         </is>
       </c>
-      <c r="E3" s="25" t="inlineStr">
+      <c r="E3" s="59" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
@@ -2607,7 +3859,7 @@
       <c r="D4" s="12" t="n">
         <v>1700</v>
       </c>
-      <c r="E4" s="24" t="inlineStr">
+      <c r="E4" s="58" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
@@ -2633,7 +3885,7 @@
           <t>N/A (liquid)</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="59" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
@@ -2657,14 +3909,14 @@
       <c r="D6" s="12" t="n">
         <v>1300</v>
       </c>
-      <c r="E6" s="24" t="inlineStr">
+      <c r="E6" s="58" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>CuAl2O4</t>
         </is>
@@ -2681,7 +3933,7 @@
       <c r="D7" s="15" t="n">
         <v>1550</v>
       </c>
-      <c r="E7" s="27" t="inlineStr">
+      <c r="E7" s="61" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
@@ -2692,7 +3944,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2752,10 +4004,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C2" s="28" t="n">
+      <c r="C2" s="62" t="n">
         <v>0.2</v>
       </c>
-      <c r="D2" s="29" t="n">
+      <c r="D2" s="63" t="n">
         <v>0.0006024287195135149</v>
       </c>
       <c r="E2" s="12" t="inlineStr">
@@ -2778,10 +4030,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C3" s="28" t="n">
+      <c r="C3" s="62" t="n">
         <v>0.4</v>
       </c>
-      <c r="D3" s="29" t="n">
+      <c r="D3" s="63" t="n">
         <v>0.0005921646682545373</v>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -2805,10 +4057,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C4" s="28" t="n">
+      <c r="C4" s="62" t="n">
         <v>0.6</v>
       </c>
-      <c r="D4" s="29" t="n">
+      <c r="D4" s="63" t="n">
         <v>0.0005849859614188124</v>
       </c>
       <c r="E4" s="12" t="inlineStr">
@@ -2832,10 +4084,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C5" s="28" t="n">
+      <c r="C5" s="62" t="n">
         <v>0.8</v>
       </c>
-      <c r="D5" s="29" t="n">
+      <c r="D5" s="63" t="n">
         <v>0.0005795578709134352</v>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -2859,10 +4111,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C6" s="28" t="n">
+      <c r="C6" s="62" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="29" t="n">
+      <c r="D6" s="63" t="n">
         <v>0.0005747540319710688</v>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -2886,10 +4138,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C7" s="28" t="n">
+      <c r="C7" s="62" t="n">
         <v>1.2</v>
       </c>
-      <c r="D7" s="29" t="n">
+      <c r="D7" s="63" t="n">
         <v>0.0005690086100650586</v>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -2913,10 +4165,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C8" s="28" t="n">
+      <c r="C8" s="62" t="n">
         <v>1.4</v>
       </c>
-      <c r="D8" s="29" t="n">
+      <c r="D8" s="63" t="n">
         <v>0.0005623991726393003</v>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -2940,10 +4192,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="62" t="n">
         <v>1.6</v>
       </c>
-      <c r="D9" s="29" t="n">
+      <c r="D9" s="63" t="n">
         <v>0.0005549646048769486</v>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -2967,10 +4219,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="62" t="n">
         <v>1.8</v>
       </c>
-      <c r="D10" s="29" t="n">
+      <c r="D10" s="63" t="n">
         <v>0.0005469620453455369</v>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -2994,10 +4246,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C11" s="28" t="n">
+      <c r="C11" s="62" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="29" t="n">
+      <c r="D11" s="63" t="n">
         <v>0.0005386374910615401</v>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -3021,10 +4273,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C12" s="28" t="n">
+      <c r="C12" s="62" t="n">
         <v>2.2</v>
       </c>
-      <c r="D12" s="29" t="n">
+      <c r="D12" s="63" t="n">
         <v>0.0005302395956835024</v>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -3048,10 +4300,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C13" s="28" t="n">
+      <c r="C13" s="62" t="n">
         <v>2.4</v>
       </c>
-      <c r="D13" s="29" t="n">
+      <c r="D13" s="63" t="n">
         <v>0.0005220166239764437</v>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -3075,10 +4327,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C14" s="28" t="n">
+      <c r="C14" s="62" t="n">
         <v>2.6</v>
       </c>
-      <c r="D14" s="29" t="n">
+      <c r="D14" s="63" t="n">
         <v>0.0005141731215264483</v>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -3102,10 +4354,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C15" s="28" t="n">
+      <c r="C15" s="62" t="n">
         <v>2.8</v>
       </c>
-      <c r="D15" s="29" t="n">
+      <c r="D15" s="63" t="n">
         <v>0.000506844968432079</v>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -3129,10 +4381,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C16" s="28" t="n">
+      <c r="C16" s="62" t="n">
         <v>3</v>
       </c>
-      <c r="D16" s="29" t="n">
+      <c r="D16" s="63" t="n">
         <v>0.0005001045724686611</v>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -3156,10 +4408,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C17" s="30" t="n">
+      <c r="C17" s="64" t="n">
         <v>0.2</v>
       </c>
-      <c r="D17" s="31" t="n">
+      <c r="D17" s="65" t="n">
         <v>0.0006238595135610499</v>
       </c>
       <c r="E17" s="13" t="inlineStr">
@@ -3182,10 +4434,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C18" s="30" t="n">
+      <c r="C18" s="64" t="n">
         <v>0.4</v>
       </c>
-      <c r="D18" s="31" t="n">
+      <c r="D18" s="65" t="n">
         <v>0.0006238595135610499</v>
       </c>
       <c r="E18" s="13" t="inlineStr">
@@ -3209,10 +4461,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C19" s="30" t="n">
+      <c r="C19" s="64" t="n">
         <v>0.6</v>
       </c>
-      <c r="D19" s="31" t="n">
+      <c r="D19" s="65" t="n">
         <v>0.0006238595135610521</v>
       </c>
       <c r="E19" s="13" t="inlineStr">
@@ -3236,10 +4488,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C20" s="30" t="n">
+      <c r="C20" s="64" t="n">
         <v>0.8</v>
       </c>
-      <c r="D20" s="31" t="n">
+      <c r="D20" s="65" t="n">
         <v>0.0006238595135610521</v>
       </c>
       <c r="E20" s="13" t="inlineStr">
@@ -3263,10 +4515,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C21" s="30" t="n">
+      <c r="C21" s="64" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="31" t="n">
+      <c r="D21" s="65" t="n">
         <v>0.0006238595135610521</v>
       </c>
       <c r="E21" s="13" t="inlineStr">
@@ -3290,10 +4542,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C22" s="30" t="n">
+      <c r="C22" s="64" t="n">
         <v>1.2</v>
       </c>
-      <c r="D22" s="31" t="n">
+      <c r="D22" s="65" t="n">
         <v>0.0006238595135610504</v>
       </c>
       <c r="E22" s="13" t="inlineStr">
@@ -3317,10 +4569,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C23" s="30" t="n">
+      <c r="C23" s="64" t="n">
         <v>1.4</v>
       </c>
-      <c r="D23" s="31" t="n">
+      <c r="D23" s="65" t="n">
         <v>0.0006238595135610504</v>
       </c>
       <c r="E23" s="13" t="inlineStr">
@@ -3344,10 +4596,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C24" s="30" t="n">
+      <c r="C24" s="64" t="n">
         <v>1.6</v>
       </c>
-      <c r="D24" s="31" t="n">
+      <c r="D24" s="65" t="n">
         <v>0.0006240110028708597</v>
       </c>
       <c r="E24" s="13" t="inlineStr">
@@ -3371,10 +4623,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C25" s="30" t="n">
+      <c r="C25" s="64" t="n">
         <v>1.8</v>
       </c>
-      <c r="D25" s="31" t="n">
+      <c r="D25" s="65" t="n">
         <v>0.0006240764395684967</v>
       </c>
       <c r="E25" s="13" t="inlineStr">
@@ -3398,10 +4650,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C26" s="30" t="n">
+      <c r="C26" s="64" t="n">
         <v>2</v>
       </c>
-      <c r="D26" s="31" t="n">
+      <c r="D26" s="65" t="n">
         <v>0.0006240764395684967</v>
       </c>
       <c r="E26" s="13" t="inlineStr">
@@ -3425,10 +4677,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C27" s="30" t="n">
+      <c r="C27" s="64" t="n">
         <v>2.2</v>
       </c>
-      <c r="D27" s="31" t="n">
+      <c r="D27" s="65" t="n">
         <v>0.0006240764395684956</v>
       </c>
       <c r="E27" s="13" t="inlineStr">
@@ -3452,10 +4704,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C28" s="30" t="n">
+      <c r="C28" s="64" t="n">
         <v>2.4</v>
       </c>
-      <c r="D28" s="31" t="n">
+      <c r="D28" s="65" t="n">
         <v>0.0006240764395684967</v>
       </c>
       <c r="E28" s="13" t="inlineStr">
@@ -3479,10 +4731,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C29" s="30" t="n">
+      <c r="C29" s="64" t="n">
         <v>2.6</v>
       </c>
-      <c r="D29" s="31" t="n">
+      <c r="D29" s="65" t="n">
         <v>0.0006240764395684967</v>
       </c>
       <c r="E29" s="13" t="inlineStr">
@@ -3506,10 +4758,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C30" s="30" t="n">
+      <c r="C30" s="64" t="n">
         <v>2.8</v>
       </c>
-      <c r="D30" s="31" t="n">
+      <c r="D30" s="65" t="n">
         <v>0.0006240764395684973</v>
       </c>
       <c r="E30" s="13" t="inlineStr">
@@ -3523,7 +4775,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="26" t="inlineStr">
+      <c r="A31" s="60" t="inlineStr">
         <is>
           <t>Cu-Al-Si-O</t>
         </is>
@@ -3533,10 +4785,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C31" s="32" t="n">
+      <c r="C31" s="66" t="n">
         <v>3</v>
       </c>
-      <c r="D31" s="33" t="n">
+      <c r="D31" s="67" t="n">
         <v>0.0006240764395684973</v>
       </c>
       <c r="E31" s="15" t="inlineStr">
@@ -3554,7 +4806,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3629,19 +4881,19 @@
       <c r="C2" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D2" s="34" t="n">
+      <c r="D2" s="68" t="n">
         <v>0.9</v>
       </c>
-      <c r="E2" s="34" t="n">
+      <c r="E2" s="68" t="n">
         <v>0.04</v>
       </c>
-      <c r="F2" s="34" t="n">
+      <c r="F2" s="68" t="n">
         <v>0.06</v>
       </c>
-      <c r="G2" s="29" t="n">
+      <c r="G2" s="63" t="n">
         <v>0.0006242415932771841</v>
       </c>
-      <c r="H2" s="24" t="inlineStr">
+      <c r="H2" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3661,19 +4913,19 @@
       <c r="C3" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D3" s="34" t="n">
+      <c r="D3" s="68" t="n">
         <v>0.855263</v>
       </c>
-      <c r="E3" s="34" t="n">
+      <c r="E3" s="68" t="n">
         <v>0.057895</v>
       </c>
-      <c r="F3" s="34" t="n">
+      <c r="F3" s="68" t="n">
         <v>0.086842</v>
       </c>
-      <c r="G3" s="29" t="n">
+      <c r="G3" s="63" t="n">
         <v>0.000624241593277183</v>
       </c>
-      <c r="H3" s="24" t="inlineStr">
+      <c r="H3" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3693,19 +4945,19 @@
       <c r="C4" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D4" s="34" t="n">
+      <c r="D4" s="68" t="n">
         <v>0.810526</v>
       </c>
-      <c r="E4" s="34" t="n">
+      <c r="E4" s="68" t="n">
         <v>0.075789</v>
       </c>
-      <c r="F4" s="34" t="n">
+      <c r="F4" s="68" t="n">
         <v>0.113684</v>
       </c>
-      <c r="G4" s="29" t="n">
+      <c r="G4" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H4" s="24" t="inlineStr">
+      <c r="H4" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3725,19 +4977,19 @@
       <c r="C5" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D5" s="34" t="n">
+      <c r="D5" s="68" t="n">
         <v>0.7657890000000001</v>
       </c>
-      <c r="E5" s="34" t="n">
+      <c r="E5" s="68" t="n">
         <v>0.093684</v>
       </c>
-      <c r="F5" s="34" t="n">
+      <c r="F5" s="68" t="n">
         <v>0.140526</v>
       </c>
-      <c r="G5" s="29" t="n">
+      <c r="G5" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H5" s="24" t="inlineStr">
+      <c r="H5" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3757,19 +5009,19 @@
       <c r="C6" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D6" s="34" t="n">
+      <c r="D6" s="68" t="n">
         <v>0.7210530000000001</v>
       </c>
-      <c r="E6" s="34" t="n">
+      <c r="E6" s="68" t="n">
         <v>0.111579</v>
       </c>
-      <c r="F6" s="34" t="n">
+      <c r="F6" s="68" t="n">
         <v>0.167368</v>
       </c>
-      <c r="G6" s="29" t="n">
+      <c r="G6" s="63" t="n">
         <v>0.0006242415932771846</v>
       </c>
-      <c r="H6" s="24" t="inlineStr">
+      <c r="H6" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3789,19 +5041,19 @@
       <c r="C7" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D7" s="34" t="n">
+      <c r="D7" s="68" t="n">
         <v>0.676316</v>
       </c>
-      <c r="E7" s="34" t="n">
+      <c r="E7" s="68" t="n">
         <v>0.129474</v>
       </c>
-      <c r="F7" s="34" t="n">
+      <c r="F7" s="68" t="n">
         <v>0.194211</v>
       </c>
-      <c r="G7" s="29" t="n">
+      <c r="G7" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H7" s="24" t="inlineStr">
+      <c r="H7" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3821,19 +5073,19 @@
       <c r="C8" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D8" s="34" t="n">
+      <c r="D8" s="68" t="n">
         <v>0.631579</v>
       </c>
-      <c r="E8" s="34" t="n">
+      <c r="E8" s="68" t="n">
         <v>0.147368</v>
       </c>
-      <c r="F8" s="34" t="n">
+      <c r="F8" s="68" t="n">
         <v>0.221053</v>
       </c>
-      <c r="G8" s="29" t="n">
+      <c r="G8" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H8" s="24" t="inlineStr">
+      <c r="H8" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3853,19 +5105,19 @@
       <c r="C9" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D9" s="34" t="n">
+      <c r="D9" s="68" t="n">
         <v>0.586842</v>
       </c>
-      <c r="E9" s="34" t="n">
+      <c r="E9" s="68" t="n">
         <v>0.165263</v>
       </c>
-      <c r="F9" s="34" t="n">
+      <c r="F9" s="68" t="n">
         <v>0.247895</v>
       </c>
-      <c r="G9" s="29" t="n">
+      <c r="G9" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H9" s="24" t="inlineStr">
+      <c r="H9" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3885,19 +5137,19 @@
       <c r="C10" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D10" s="34" t="n">
+      <c r="D10" s="68" t="n">
         <v>0.5421049999999999</v>
       </c>
-      <c r="E10" s="34" t="n">
+      <c r="E10" s="68" t="n">
         <v>0.183158</v>
       </c>
-      <c r="F10" s="34" t="n">
+      <c r="F10" s="68" t="n">
         <v>0.274737</v>
       </c>
-      <c r="G10" s="29" t="n">
+      <c r="G10" s="63" t="n">
         <v>0.0006242415932771825</v>
       </c>
-      <c r="H10" s="24" t="inlineStr">
+      <c r="H10" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3917,19 +5169,19 @@
       <c r="C11" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D11" s="34" t="n">
+      <c r="D11" s="68" t="n">
         <v>0.497368</v>
       </c>
-      <c r="E11" s="34" t="n">
+      <c r="E11" s="68" t="n">
         <v>0.201053</v>
       </c>
-      <c r="F11" s="34" t="n">
+      <c r="F11" s="68" t="n">
         <v>0.301579</v>
       </c>
-      <c r="G11" s="29" t="n">
+      <c r="G11" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H11" s="24" t="inlineStr">
+      <c r="H11" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3949,19 +5201,19 @@
       <c r="C12" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D12" s="34" t="n">
+      <c r="D12" s="68" t="n">
         <v>0.452632</v>
       </c>
-      <c r="E12" s="34" t="n">
+      <c r="E12" s="68" t="n">
         <v>0.218947</v>
       </c>
-      <c r="F12" s="34" t="n">
+      <c r="F12" s="68" t="n">
         <v>0.328421</v>
       </c>
-      <c r="G12" s="29" t="n">
+      <c r="G12" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H12" s="24" t="inlineStr">
+      <c r="H12" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3981,19 +5233,19 @@
       <c r="C13" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D13" s="34" t="n">
+      <c r="D13" s="68" t="n">
         <v>0.407895</v>
       </c>
-      <c r="E13" s="34" t="n">
+      <c r="E13" s="68" t="n">
         <v>0.236842</v>
       </c>
-      <c r="F13" s="34" t="n">
+      <c r="F13" s="68" t="n">
         <v>0.355263</v>
       </c>
-      <c r="G13" s="29" t="n">
+      <c r="G13" s="63" t="n">
         <v>0.000624241593277183</v>
       </c>
-      <c r="H13" s="24" t="inlineStr">
+      <c r="H13" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4013,19 +5265,19 @@
       <c r="C14" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D14" s="34" t="n">
+      <c r="D14" s="68" t="n">
         <v>0.363158</v>
       </c>
-      <c r="E14" s="34" t="n">
+      <c r="E14" s="68" t="n">
         <v>0.254737</v>
       </c>
-      <c r="F14" s="34" t="n">
+      <c r="F14" s="68" t="n">
         <v>0.382105</v>
       </c>
-      <c r="G14" s="29" t="n">
+      <c r="G14" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H14" s="24" t="inlineStr">
+      <c r="H14" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4045,19 +5297,19 @@
       <c r="C15" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D15" s="34" t="n">
+      <c r="D15" s="68" t="n">
         <v>0.318421</v>
       </c>
-      <c r="E15" s="34" t="n">
+      <c r="E15" s="68" t="n">
         <v>0.272632</v>
       </c>
-      <c r="F15" s="34" t="n">
+      <c r="F15" s="68" t="n">
         <v>0.408947</v>
       </c>
-      <c r="G15" s="29" t="n">
+      <c r="G15" s="63" t="n">
         <v>0.0006242415932771846</v>
       </c>
-      <c r="H15" s="24" t="inlineStr">
+      <c r="H15" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4077,19 +5329,19 @@
       <c r="C16" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D16" s="34" t="n">
+      <c r="D16" s="68" t="n">
         <v>0.273684</v>
       </c>
-      <c r="E16" s="34" t="n">
+      <c r="E16" s="68" t="n">
         <v>0.290526</v>
       </c>
-      <c r="F16" s="34" t="n">
+      <c r="F16" s="68" t="n">
         <v>0.435789</v>
       </c>
-      <c r="G16" s="29" t="n">
+      <c r="G16" s="63" t="n">
         <v>0.000624241593277183</v>
       </c>
-      <c r="H16" s="24" t="inlineStr">
+      <c r="H16" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4109,19 +5361,19 @@
       <c r="C17" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D17" s="34" t="n">
+      <c r="D17" s="68" t="n">
         <v>0.228947</v>
       </c>
-      <c r="E17" s="34" t="n">
+      <c r="E17" s="68" t="n">
         <v>0.308421</v>
       </c>
-      <c r="F17" s="34" t="n">
+      <c r="F17" s="68" t="n">
         <v>0.462632</v>
       </c>
-      <c r="G17" s="29" t="n">
+      <c r="G17" s="63" t="n">
         <v>0.0006242415932771825</v>
       </c>
-      <c r="H17" s="24" t="inlineStr">
+      <c r="H17" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4141,19 +5393,19 @@
       <c r="C18" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D18" s="34" t="n">
+      <c r="D18" s="68" t="n">
         <v>0.184211</v>
       </c>
-      <c r="E18" s="34" t="n">
+      <c r="E18" s="68" t="n">
         <v>0.326316</v>
       </c>
-      <c r="F18" s="34" t="n">
+      <c r="F18" s="68" t="n">
         <v>0.489474</v>
       </c>
-      <c r="G18" s="29" t="n">
+      <c r="G18" s="63" t="n">
         <v>0.0006242415932771825</v>
       </c>
-      <c r="H18" s="24" t="inlineStr">
+      <c r="H18" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4173,19 +5425,19 @@
       <c r="C19" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D19" s="34" t="n">
+      <c r="D19" s="68" t="n">
         <v>0.139474</v>
       </c>
-      <c r="E19" s="34" t="n">
+      <c r="E19" s="68" t="n">
         <v>0.344211</v>
       </c>
-      <c r="F19" s="34" t="n">
+      <c r="F19" s="68" t="n">
         <v>0.516316</v>
       </c>
-      <c r="G19" s="29" t="n">
+      <c r="G19" s="63" t="n">
         <v>0.000624241593277183</v>
       </c>
-      <c r="H19" s="24" t="inlineStr">
+      <c r="H19" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4205,19 +5457,19 @@
       <c r="C20" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D20" s="34" t="n">
+      <c r="D20" s="68" t="n">
         <v>0.094737</v>
       </c>
-      <c r="E20" s="34" t="n">
+      <c r="E20" s="68" t="n">
         <v>0.362105</v>
       </c>
-      <c r="F20" s="34" t="n">
+      <c r="F20" s="68" t="n">
         <v>0.543158</v>
       </c>
-      <c r="G20" s="29" t="n">
+      <c r="G20" s="63" t="n">
         <v>0.0006242415932771825</v>
       </c>
-      <c r="H20" s="24" t="inlineStr">
+      <c r="H20" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4237,19 +5489,19 @@
       <c r="C21" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D21" s="34" t="n">
+      <c r="D21" s="68" t="n">
         <v>0.05</v>
       </c>
-      <c r="E21" s="34" t="n">
+      <c r="E21" s="68" t="n">
         <v>0.38</v>
       </c>
-      <c r="F21" s="34" t="n">
+      <c r="F21" s="68" t="n">
         <v>0.57</v>
       </c>
-      <c r="G21" s="29" t="n">
+      <c r="G21" s="63" t="n">
         <v>0.0006242415932771841</v>
       </c>
-      <c r="H21" s="24" t="inlineStr">
+      <c r="H21" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4269,19 +5521,19 @@
       <c r="C22" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D22" s="35" t="n">
+      <c r="D22" s="69" t="n">
         <v>0.9</v>
       </c>
-      <c r="E22" s="35" t="n">
+      <c r="E22" s="69" t="n">
         <v>0.05</v>
       </c>
-      <c r="F22" s="35" t="n">
+      <c r="F22" s="69" t="n">
         <v>0.05</v>
       </c>
-      <c r="G22" s="31" t="n">
+      <c r="G22" s="65" t="n">
         <v>0.0006234486982757811</v>
       </c>
-      <c r="H22" s="25" t="inlineStr">
+      <c r="H22" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4301,19 +5553,19 @@
       <c r="C23" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D23" s="35" t="n">
+      <c r="D23" s="69" t="n">
         <v>0.855263</v>
       </c>
-      <c r="E23" s="35" t="n">
+      <c r="E23" s="69" t="n">
         <v>0.072368</v>
       </c>
-      <c r="F23" s="35" t="n">
+      <c r="F23" s="69" t="n">
         <v>0.072368</v>
       </c>
-      <c r="G23" s="31" t="n">
+      <c r="G23" s="65" t="n">
         <v>0.0006234240698697985</v>
       </c>
-      <c r="H23" s="25" t="inlineStr">
+      <c r="H23" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4333,19 +5585,19 @@
       <c r="C24" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D24" s="35" t="n">
+      <c r="D24" s="69" t="n">
         <v>0.810526</v>
       </c>
-      <c r="E24" s="35" t="n">
+      <c r="E24" s="69" t="n">
         <v>0.094737</v>
       </c>
-      <c r="F24" s="35" t="n">
+      <c r="F24" s="69" t="n">
         <v>0.094737</v>
       </c>
-      <c r="G24" s="31" t="n">
+      <c r="G24" s="65" t="n">
         <v>0.000623390113702764</v>
       </c>
-      <c r="H24" s="25" t="inlineStr">
+      <c r="H24" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4365,19 +5617,19 @@
       <c r="C25" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D25" s="35" t="n">
+      <c r="D25" s="69" t="n">
         <v>0.7657890000000001</v>
       </c>
-      <c r="E25" s="35" t="n">
+      <c r="E25" s="69" t="n">
         <v>0.117105</v>
       </c>
-      <c r="F25" s="35" t="n">
+      <c r="F25" s="69" t="n">
         <v>0.117105</v>
       </c>
-      <c r="G25" s="31" t="n">
+      <c r="G25" s="65" t="n">
         <v>0.0006233465051459715</v>
       </c>
-      <c r="H25" s="25" t="inlineStr">
+      <c r="H25" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4397,19 +5649,19 @@
       <c r="C26" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D26" s="35" t="n">
+      <c r="D26" s="69" t="n">
         <v>0.7210530000000001</v>
       </c>
-      <c r="E26" s="35" t="n">
+      <c r="E26" s="69" t="n">
         <v>0.139474</v>
       </c>
-      <c r="F26" s="35" t="n">
+      <c r="F26" s="69" t="n">
         <v>0.139474</v>
       </c>
-      <c r="G26" s="31" t="n">
+      <c r="G26" s="65" t="n">
         <v>0.0006232927260585453</v>
       </c>
-      <c r="H26" s="25" t="inlineStr">
+      <c r="H26" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4429,19 +5681,19 @@
       <c r="C27" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D27" s="35" t="n">
+      <c r="D27" s="69" t="n">
         <v>0.676316</v>
       </c>
-      <c r="E27" s="35" t="n">
+      <c r="E27" s="69" t="n">
         <v>0.161842</v>
       </c>
-      <c r="F27" s="35" t="n">
+      <c r="F27" s="69" t="n">
         <v>0.161842</v>
       </c>
-      <c r="G27" s="31" t="n">
+      <c r="G27" s="65" t="n">
         <v>0.0006232279909242769</v>
       </c>
-      <c r="H27" s="25" t="inlineStr">
+      <c r="H27" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4461,19 +5713,19 @@
       <c r="C28" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D28" s="35" t="n">
+      <c r="D28" s="69" t="n">
         <v>0.631579</v>
       </c>
-      <c r="E28" s="35" t="n">
+      <c r="E28" s="69" t="n">
         <v>0.184211</v>
       </c>
-      <c r="F28" s="35" t="n">
+      <c r="F28" s="69" t="n">
         <v>0.184211</v>
       </c>
-      <c r="G28" s="31" t="n">
+      <c r="G28" s="65" t="n">
         <v>0.0006231511590811589</v>
       </c>
-      <c r="H28" s="25" t="inlineStr">
+      <c r="H28" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4493,19 +5745,19 @@
       <c r="C29" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D29" s="35" t="n">
+      <c r="D29" s="69" t="n">
         <v>0.586842</v>
       </c>
-      <c r="E29" s="35" t="n">
+      <c r="E29" s="69" t="n">
         <v>0.206579</v>
       </c>
-      <c r="F29" s="35" t="n">
+      <c r="F29" s="69" t="n">
         <v>0.206579</v>
       </c>
-      <c r="G29" s="31" t="n">
+      <c r="G29" s="65" t="n">
         <v>0.0006230606192890642</v>
       </c>
-      <c r="H29" s="25" t="inlineStr">
+      <c r="H29" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4525,19 +5777,19 @@
       <c r="C30" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D30" s="35" t="n">
+      <c r="D30" s="69" t="n">
         <v>0.5421049999999999</v>
       </c>
-      <c r="E30" s="35" t="n">
+      <c r="E30" s="69" t="n">
         <v>0.228947</v>
       </c>
-      <c r="F30" s="35" t="n">
+      <c r="F30" s="69" t="n">
         <v>0.228947</v>
       </c>
-      <c r="G30" s="31" t="n">
+      <c r="G30" s="65" t="n">
         <v>0.0006229541258469519</v>
       </c>
-      <c r="H30" s="25" t="inlineStr">
+      <c r="H30" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4557,19 +5809,19 @@
       <c r="C31" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D31" s="35" t="n">
+      <c r="D31" s="69" t="n">
         <v>0.497368</v>
       </c>
-      <c r="E31" s="35" t="n">
+      <c r="E31" s="69" t="n">
         <v>0.251316</v>
       </c>
-      <c r="F31" s="35" t="n">
+      <c r="F31" s="69" t="n">
         <v>0.251316</v>
       </c>
-      <c r="G31" s="31" t="n">
+      <c r="G31" s="65" t="n">
         <v>0.0006228285531386366</v>
       </c>
-      <c r="H31" s="25" t="inlineStr">
+      <c r="H31" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4589,19 +5841,19 @@
       <c r="C32" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D32" s="35" t="n">
+      <c r="D32" s="69" t="n">
         <v>0.452632</v>
       </c>
-      <c r="E32" s="35" t="n">
+      <c r="E32" s="69" t="n">
         <v>0.273684</v>
       </c>
-      <c r="F32" s="35" t="n">
+      <c r="F32" s="69" t="n">
         <v>0.273684</v>
       </c>
-      <c r="G32" s="31" t="n">
+      <c r="G32" s="65" t="n">
         <v>0.0006226795122556773</v>
       </c>
-      <c r="H32" s="25" t="inlineStr">
+      <c r="H32" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4621,19 +5873,19 @@
       <c r="C33" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D33" s="35" t="n">
+      <c r="D33" s="69" t="n">
         <v>0.407895</v>
       </c>
-      <c r="E33" s="35" t="n">
+      <c r="E33" s="69" t="n">
         <v>0.296053</v>
       </c>
-      <c r="F33" s="35" t="n">
+      <c r="F33" s="69" t="n">
         <v>0.296053</v>
       </c>
-      <c r="G33" s="31" t="n">
+      <c r="G33" s="65" t="n">
         <v>0.000622500727556083</v>
       </c>
-      <c r="H33" s="25" t="inlineStr">
+      <c r="H33" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4653,19 +5905,19 @@
       <c r="C34" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D34" s="35" t="n">
+      <c r="D34" s="69" t="n">
         <v>0.363158</v>
       </c>
-      <c r="E34" s="35" t="n">
+      <c r="E34" s="69" t="n">
         <v>0.318421</v>
       </c>
-      <c r="F34" s="35" t="n">
+      <c r="F34" s="69" t="n">
         <v>0.318421</v>
       </c>
-      <c r="G34" s="31" t="n">
+      <c r="G34" s="65" t="n">
         <v>0.0006222829760272391</v>
       </c>
-      <c r="H34" s="25" t="inlineStr">
+      <c r="H34" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4685,19 +5937,19 @@
       <c r="C35" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D35" s="35" t="n">
+      <c r="D35" s="69" t="n">
         <v>0.318421</v>
       </c>
-      <c r="E35" s="35" t="n">
+      <c r="E35" s="69" t="n">
         <v>0.340789</v>
       </c>
-      <c r="F35" s="35" t="n">
+      <c r="F35" s="69" t="n">
         <v>0.340789</v>
       </c>
-      <c r="G35" s="31" t="n">
+      <c r="G35" s="65" t="n">
         <v>0.0006220121819606671</v>
       </c>
-      <c r="H35" s="25" t="inlineStr">
+      <c r="H35" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4717,19 +5969,19 @@
       <c r="C36" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D36" s="35" t="n">
+      <c r="D36" s="69" t="n">
         <v>0.273684</v>
       </c>
-      <c r="E36" s="35" t="n">
+      <c r="E36" s="69" t="n">
         <v>0.363158</v>
       </c>
-      <c r="F36" s="35" t="n">
+      <c r="F36" s="69" t="n">
         <v>0.363158</v>
       </c>
-      <c r="G36" s="31" t="n">
+      <c r="G36" s="65" t="n">
         <v>0.0006216657532754782</v>
       </c>
-      <c r="H36" s="25" t="inlineStr">
+      <c r="H36" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4749,19 +6001,19 @@
       <c r="C37" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D37" s="35" t="n">
+      <c r="D37" s="69" t="n">
         <v>0.228947</v>
       </c>
-      <c r="E37" s="35" t="n">
+      <c r="E37" s="69" t="n">
         <v>0.385526</v>
       </c>
-      <c r="F37" s="35" t="n">
+      <c r="F37" s="69" t="n">
         <v>0.385526</v>
       </c>
-      <c r="G37" s="31" t="n">
+      <c r="G37" s="65" t="n">
         <v>0.0006212048918444731</v>
       </c>
-      <c r="H37" s="25" t="inlineStr">
+      <c r="H37" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4781,19 +6033,19 @@
       <c r="C38" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D38" s="35" t="n">
+      <c r="D38" s="69" t="n">
         <v>0.184211</v>
       </c>
-      <c r="E38" s="35" t="n">
+      <c r="E38" s="69" t="n">
         <v>0.407895</v>
       </c>
-      <c r="F38" s="35" t="n">
+      <c r="F38" s="69" t="n">
         <v>0.407895</v>
       </c>
-      <c r="G38" s="31" t="n">
+      <c r="G38" s="65" t="n">
         <v>0.0006205564490138872</v>
       </c>
-      <c r="H38" s="25" t="inlineStr">
+      <c r="H38" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4813,19 +6065,19 @@
       <c r="C39" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D39" s="35" t="n">
+      <c r="D39" s="69" t="n">
         <v>0.139474</v>
       </c>
-      <c r="E39" s="35" t="n">
+      <c r="E39" s="69" t="n">
         <v>0.430263</v>
       </c>
-      <c r="F39" s="35" t="n">
+      <c r="F39" s="69" t="n">
         <v>0.430263</v>
       </c>
-      <c r="G39" s="31" t="n">
+      <c r="G39" s="65" t="n">
         <v>0.0006195624103164132</v>
       </c>
-      <c r="H39" s="25" t="inlineStr">
+      <c r="H39" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4845,19 +6097,19 @@
       <c r="C40" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D40" s="35" t="n">
+      <c r="D40" s="69" t="n">
         <v>0.094737</v>
       </c>
-      <c r="E40" s="35" t="n">
+      <c r="E40" s="69" t="n">
         <v>0.452632</v>
       </c>
-      <c r="F40" s="35" t="n">
+      <c r="F40" s="69" t="n">
         <v>0.452632</v>
       </c>
-      <c r="G40" s="31" t="n">
+      <c r="G40" s="65" t="n">
         <v>0.0006177982099275926</v>
       </c>
-      <c r="H40" s="25" t="inlineStr">
+      <c r="H40" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4877,19 +6129,19 @@
       <c r="C41" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D41" s="35" t="n">
+      <c r="D41" s="69" t="n">
         <v>0.05</v>
       </c>
-      <c r="E41" s="35" t="n">
+      <c r="E41" s="69" t="n">
         <v>0.475</v>
       </c>
-      <c r="F41" s="35" t="n">
+      <c r="F41" s="69" t="n">
         <v>0.475</v>
       </c>
-      <c r="G41" s="31" t="n">
+      <c r="G41" s="65" t="n">
         <v>0.0006135214100988033</v>
       </c>
-      <c r="H41" s="25" t="inlineStr">
+      <c r="H41" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4909,19 +6161,19 @@
       <c r="C42" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D42" s="34" t="n">
+      <c r="D42" s="68" t="n">
         <v>0.9</v>
       </c>
-      <c r="E42" s="34" t="n">
+      <c r="E42" s="68" t="n">
         <v>0.05</v>
       </c>
-      <c r="F42" s="34" t="n">
+      <c r="F42" s="68" t="n">
         <v>0.05</v>
       </c>
-      <c r="G42" s="29" t="n">
+      <c r="G42" s="63" t="n">
         <v>0.0006192201975493238</v>
       </c>
-      <c r="H42" s="24" t="inlineStr">
+      <c r="H42" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -4941,19 +6193,19 @@
       <c r="C43" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D43" s="34" t="n">
+      <c r="D43" s="68" t="n">
         <v>0.855263</v>
       </c>
-      <c r="E43" s="34" t="n">
+      <c r="E43" s="68" t="n">
         <v>0.072368</v>
       </c>
-      <c r="F43" s="34" t="n">
+      <c r="F43" s="68" t="n">
         <v>0.072368</v>
       </c>
-      <c r="G43" s="29" t="n">
+      <c r="G43" s="63" t="n">
         <v>0.0006178389962257873</v>
       </c>
-      <c r="H43" s="24" t="inlineStr">
+      <c r="H43" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -4973,19 +6225,19 @@
       <c r="C44" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D44" s="34" t="n">
+      <c r="D44" s="68" t="n">
         <v>0.810526</v>
       </c>
-      <c r="E44" s="34" t="n">
+      <c r="E44" s="68" t="n">
         <v>0.094737</v>
       </c>
-      <c r="F44" s="34" t="n">
+      <c r="F44" s="68" t="n">
         <v>0.094737</v>
       </c>
-      <c r="G44" s="29" t="n">
+      <c r="G44" s="63" t="n">
         <v>0.0006164156519341792</v>
       </c>
-      <c r="H44" s="24" t="inlineStr">
+      <c r="H44" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5005,19 +6257,19 @@
       <c r="C45" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D45" s="34" t="n">
+      <c r="D45" s="68" t="n">
         <v>0.7657890000000001</v>
       </c>
-      <c r="E45" s="34" t="n">
+      <c r="E45" s="68" t="n">
         <v>0.117105</v>
       </c>
-      <c r="F45" s="34" t="n">
+      <c r="F45" s="68" t="n">
         <v>0.117105</v>
       </c>
-      <c r="G45" s="29" t="n">
+      <c r="G45" s="63" t="n">
         <v>0.0006149434371808388</v>
       </c>
-      <c r="H45" s="24" t="inlineStr">
+      <c r="H45" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5037,19 +6289,19 @@
       <c r="C46" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D46" s="34" t="n">
+      <c r="D46" s="68" t="n">
         <v>0.7210530000000001</v>
       </c>
-      <c r="E46" s="34" t="n">
+      <c r="E46" s="68" t="n">
         <v>0.139474</v>
       </c>
-      <c r="F46" s="34" t="n">
+      <c r="F46" s="68" t="n">
         <v>0.139474</v>
       </c>
-      <c r="G46" s="29" t="n">
+      <c r="G46" s="63" t="n">
         <v>0.0006134086362605692</v>
       </c>
-      <c r="H46" s="24" t="inlineStr">
+      <c r="H46" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5069,19 +6321,19 @@
       <c r="C47" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D47" s="34" t="n">
+      <c r="D47" s="68" t="n">
         <v>0.676316</v>
       </c>
-      <c r="E47" s="34" t="n">
+      <c r="E47" s="68" t="n">
         <v>0.161842</v>
       </c>
-      <c r="F47" s="34" t="n">
+      <c r="F47" s="68" t="n">
         <v>0.161842</v>
       </c>
-      <c r="G47" s="29" t="n">
+      <c r="G47" s="63" t="n">
         <v>0.000611794507683605</v>
       </c>
-      <c r="H47" s="24" t="inlineStr">
+      <c r="H47" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5101,19 +6353,19 @@
       <c r="C48" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D48" s="34" t="n">
+      <c r="D48" s="68" t="n">
         <v>0.631579</v>
       </c>
-      <c r="E48" s="34" t="n">
+      <c r="E48" s="68" t="n">
         <v>0.184211</v>
       </c>
-      <c r="F48" s="34" t="n">
+      <c r="F48" s="68" t="n">
         <v>0.184211</v>
       </c>
-      <c r="G48" s="29" t="n">
+      <c r="G48" s="63" t="n">
         <v>0.0006100815926117644</v>
       </c>
-      <c r="H48" s="24" t="inlineStr">
+      <c r="H48" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5133,19 +6385,19 @@
       <c r="C49" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D49" s="34" t="n">
+      <c r="D49" s="68" t="n">
         <v>0.586842</v>
       </c>
-      <c r="E49" s="34" t="n">
+      <c r="E49" s="68" t="n">
         <v>0.206579</v>
       </c>
-      <c r="F49" s="34" t="n">
+      <c r="F49" s="68" t="n">
         <v>0.206579</v>
       </c>
-      <c r="G49" s="29" t="n">
+      <c r="G49" s="63" t="n">
         <v>0.0006082469669095847</v>
       </c>
-      <c r="H49" s="24" t="inlineStr">
+      <c r="H49" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5165,19 +6417,19 @@
       <c r="C50" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D50" s="34" t="n">
+      <c r="D50" s="68" t="n">
         <v>0.5421049999999999</v>
       </c>
-      <c r="E50" s="34" t="n">
+      <c r="E50" s="68" t="n">
         <v>0.228947</v>
       </c>
-      <c r="F50" s="34" t="n">
+      <c r="F50" s="68" t="n">
         <v>0.228947</v>
       </c>
-      <c r="G50" s="29" t="n">
+      <c r="G50" s="63" t="n">
         <v>0.0006062629201632612</v>
       </c>
-      <c r="H50" s="24" t="inlineStr">
+      <c r="H50" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5197,19 +6449,19 @@
       <c r="C51" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D51" s="34" t="n">
+      <c r="D51" s="68" t="n">
         <v>0.497368</v>
       </c>
-      <c r="E51" s="34" t="n">
+      <c r="E51" s="68" t="n">
         <v>0.251316</v>
       </c>
-      <c r="F51" s="34" t="n">
+      <c r="F51" s="68" t="n">
         <v>0.251316</v>
       </c>
-      <c r="G51" s="29" t="n">
+      <c r="G51" s="63" t="n">
         <v>0.0006040950268609877</v>
       </c>
-      <c r="H51" s="24" t="inlineStr">
+      <c r="H51" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5229,19 +6481,19 @@
       <c r="C52" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D52" s="34" t="n">
+      <c r="D52" s="68" t="n">
         <v>0.452632</v>
       </c>
-      <c r="E52" s="34" t="n">
+      <c r="E52" s="68" t="n">
         <v>0.273684</v>
       </c>
-      <c r="F52" s="34" t="n">
+      <c r="F52" s="68" t="n">
         <v>0.273684</v>
       </c>
-      <c r="G52" s="29" t="n">
+      <c r="G52" s="63" t="n">
         <v>0.00060169933822934</v>
       </c>
-      <c r="H52" s="24" t="inlineStr">
+      <c r="H52" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5261,19 +6513,19 @@
       <c r="C53" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D53" s="34" t="n">
+      <c r="D53" s="68" t="n">
         <v>0.407895</v>
       </c>
-      <c r="E53" s="34" t="n">
+      <c r="E53" s="68" t="n">
         <v>0.296053</v>
       </c>
-      <c r="F53" s="34" t="n">
+      <c r="F53" s="68" t="n">
         <v>0.296053</v>
       </c>
-      <c r="G53" s="29" t="n">
+      <c r="G53" s="63" t="n">
         <v>0.0005990181736125742</v>
       </c>
-      <c r="H53" s="24" t="inlineStr">
+      <c r="H53" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5293,19 +6545,19 @@
       <c r="C54" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D54" s="34" t="n">
+      <c r="D54" s="68" t="n">
         <v>0.363158</v>
       </c>
-      <c r="E54" s="34" t="n">
+      <c r="E54" s="68" t="n">
         <v>0.318421</v>
       </c>
-      <c r="F54" s="34" t="n">
+      <c r="F54" s="68" t="n">
         <v>0.318421</v>
       </c>
-      <c r="G54" s="29" t="n">
+      <c r="G54" s="63" t="n">
         <v>0.0005959735807338218</v>
       </c>
-      <c r="H54" s="24" t="inlineStr">
+      <c r="H54" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5325,19 +6577,19 @@
       <c r="C55" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D55" s="34" t="n">
+      <c r="D55" s="68" t="n">
         <v>0.318421</v>
       </c>
-      <c r="E55" s="34" t="n">
+      <c r="E55" s="68" t="n">
         <v>0.340789</v>
       </c>
-      <c r="F55" s="34" t="n">
+      <c r="F55" s="68" t="n">
         <v>0.340789</v>
       </c>
-      <c r="G55" s="29" t="n">
+      <c r="G55" s="63" t="n">
         <v>0.0005924567681126914</v>
       </c>
-      <c r="H55" s="24" t="inlineStr">
+      <c r="H55" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5357,19 +6609,19 @@
       <c r="C56" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D56" s="34" t="n">
+      <c r="D56" s="68" t="n">
         <v>0.273684</v>
       </c>
-      <c r="E56" s="34" t="n">
+      <c r="E56" s="68" t="n">
         <v>0.363158</v>
       </c>
-      <c r="F56" s="34" t="n">
+      <c r="F56" s="68" t="n">
         <v>0.363158</v>
       </c>
-      <c r="G56" s="29" t="n">
+      <c r="G56" s="63" t="n">
         <v>0.0005883103133506319</v>
       </c>
-      <c r="H56" s="24" t="inlineStr">
+      <c r="H56" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5389,19 +6641,19 @@
       <c r="C57" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D57" s="34" t="n">
+      <c r="D57" s="68" t="n">
         <v>0.228947</v>
       </c>
-      <c r="E57" s="34" t="n">
+      <c r="E57" s="68" t="n">
         <v>0.385526</v>
       </c>
-      <c r="F57" s="34" t="n">
+      <c r="F57" s="68" t="n">
         <v>0.385526</v>
       </c>
-      <c r="G57" s="29" t="n">
+      <c r="G57" s="63" t="n">
         <v>0.0005832970131890047</v>
       </c>
-      <c r="H57" s="24" t="inlineStr">
+      <c r="H57" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5421,19 +6673,19 @@
       <c r="C58" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D58" s="34" t="n">
+      <c r="D58" s="68" t="n">
         <v>0.184211</v>
       </c>
-      <c r="E58" s="34" t="n">
+      <c r="E58" s="68" t="n">
         <v>0.407895</v>
       </c>
-      <c r="F58" s="34" t="n">
+      <c r="F58" s="68" t="n">
         <v>0.407895</v>
       </c>
-      <c r="G58" s="29" t="n">
+      <c r="G58" s="63" t="n">
         <v>0.0005770442311225281</v>
       </c>
-      <c r="H58" s="24" t="inlineStr">
+      <c r="H58" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5453,19 +6705,19 @@
       <c r="C59" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D59" s="34" t="n">
+      <c r="D59" s="68" t="n">
         <v>0.139474</v>
       </c>
-      <c r="E59" s="34" t="n">
+      <c r="E59" s="68" t="n">
         <v>0.430263</v>
       </c>
-      <c r="F59" s="34" t="n">
+      <c r="F59" s="68" t="n">
         <v>0.430263</v>
       </c>
-      <c r="G59" s="29" t="n">
+      <c r="G59" s="63" t="n">
         <v>0.0005689524243180519</v>
       </c>
-      <c r="H59" s="24" t="inlineStr">
+      <c r="H59" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5485,19 +6737,19 @@
       <c r="C60" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D60" s="34" t="n">
+      <c r="D60" s="68" t="n">
         <v>0.094737</v>
       </c>
-      <c r="E60" s="34" t="n">
+      <c r="E60" s="68" t="n">
         <v>0.452632</v>
       </c>
-      <c r="F60" s="34" t="n">
+      <c r="F60" s="68" t="n">
         <v>0.452632</v>
       </c>
-      <c r="G60" s="29" t="n">
+      <c r="G60" s="63" t="n">
         <v>0.0005581573496582796</v>
       </c>
-      <c r="H60" s="24" t="inlineStr">
+      <c r="H60" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5517,19 +6769,19 @@
       <c r="C61" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D61" s="34" t="n">
+      <c r="D61" s="68" t="n">
         <v>0.05</v>
       </c>
-      <c r="E61" s="34" t="n">
+      <c r="E61" s="68" t="n">
         <v>0.475</v>
       </c>
-      <c r="F61" s="34" t="n">
+      <c r="F61" s="68" t="n">
         <v>0.475</v>
       </c>
-      <c r="G61" s="29" t="n">
+      <c r="G61" s="63" t="n">
         <v>0.0005441813023263959</v>
       </c>
-      <c r="H61" s="24" t="inlineStr">
+      <c r="H61" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5549,19 +6801,19 @@
       <c r="C62" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D62" s="35" t="n">
+      <c r="D62" s="69" t="n">
         <v>0.9</v>
       </c>
-      <c r="E62" s="35" t="n">
+      <c r="E62" s="69" t="n">
         <v>0.028571</v>
       </c>
-      <c r="F62" s="35" t="n">
+      <c r="F62" s="69" t="n">
         <v>0.07142900000000001</v>
       </c>
-      <c r="G62" s="31" t="n">
+      <c r="G62" s="65" t="n">
         <v>0.0006089752639324707</v>
       </c>
-      <c r="H62" s="25" t="inlineStr">
+      <c r="H62" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2; V3O5_HT#1</t>
         </is>
@@ -5581,19 +6833,19 @@
       <c r="C63" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D63" s="35" t="n">
+      <c r="D63" s="69" t="n">
         <v>0.855263</v>
       </c>
-      <c r="E63" s="35" t="n">
+      <c r="E63" s="69" t="n">
         <v>0.041353</v>
       </c>
-      <c r="F63" s="35" t="n">
+      <c r="F63" s="69" t="n">
         <v>0.103383</v>
       </c>
-      <c r="G63" s="31" t="n">
+      <c r="G63" s="65" t="n">
         <v>0.0006089752639324707</v>
       </c>
-      <c r="H63" s="25" t="inlineStr">
+      <c r="H63" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2; V3O5_HT#1</t>
         </is>
@@ -5613,19 +6865,19 @@
       <c r="C64" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D64" s="35" t="n">
+      <c r="D64" s="69" t="n">
         <v>0.810526</v>
       </c>
-      <c r="E64" s="35" t="n">
+      <c r="E64" s="69" t="n">
         <v>0.054135</v>
       </c>
-      <c r="F64" s="35" t="n">
+      <c r="F64" s="69" t="n">
         <v>0.135338</v>
       </c>
-      <c r="G64" s="31" t="n">
+      <c r="G64" s="65" t="n">
         <v>0.000608975263932468</v>
       </c>
-      <c r="H64" s="25" t="inlineStr">
+      <c r="H64" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2; V3O5_HT#1</t>
         </is>
@@ -5645,19 +6897,19 @@
       <c r="C65" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D65" s="35" t="n">
+      <c r="D65" s="69" t="n">
         <v>0.7657890000000001</v>
       </c>
-      <c r="E65" s="35" t="n">
+      <c r="E65" s="69" t="n">
         <v>0.066917</v>
       </c>
-      <c r="F65" s="35" t="n">
+      <c r="F65" s="69" t="n">
         <v>0.167293</v>
       </c>
-      <c r="G65" s="31" t="n">
+      <c r="G65" s="65" t="n">
         <v>0.0006089752639324696</v>
       </c>
-      <c r="H65" s="25" t="inlineStr">
+      <c r="H65" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2; V3O5_HT#1</t>
         </is>
@@ -5677,19 +6929,19 @@
       <c r="C66" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D66" s="35" t="n">
+      <c r="D66" s="69" t="n">
         <v>0.7210530000000001</v>
       </c>
-      <c r="E66" s="35" t="n">
+      <c r="E66" s="69" t="n">
         <v>0.07969900000000001</v>
       </c>
-      <c r="F66" s="35" t="n">
+      <c r="F66" s="69" t="n">
         <v>0.199248</v>
       </c>
-      <c r="G66" s="31" t="n">
+      <c r="G66" s="65" t="n">
         <v>0.0006086989931423054</v>
       </c>
-      <c r="H66" s="25" t="inlineStr">
+      <c r="H66" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5709,19 +6961,19 @@
       <c r="C67" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D67" s="35" t="n">
+      <c r="D67" s="69" t="n">
         <v>0.676316</v>
       </c>
-      <c r="E67" s="35" t="n">
+      <c r="E67" s="69" t="n">
         <v>0.09248099999999999</v>
       </c>
-      <c r="F67" s="35" t="n">
+      <c r="F67" s="69" t="n">
         <v>0.231203</v>
       </c>
-      <c r="G67" s="31" t="n">
+      <c r="G67" s="65" t="n">
         <v>0.0006075806595837329</v>
       </c>
-      <c r="H67" s="25" t="inlineStr">
+      <c r="H67" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5741,19 +6993,19 @@
       <c r="C68" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D68" s="35" t="n">
+      <c r="D68" s="69" t="n">
         <v>0.631579</v>
       </c>
-      <c r="E68" s="35" t="n">
+      <c r="E68" s="69" t="n">
         <v>0.105263</v>
       </c>
-      <c r="F68" s="35" t="n">
+      <c r="F68" s="69" t="n">
         <v>0.263158</v>
       </c>
-      <c r="G68" s="31" t="n">
+      <c r="G68" s="65" t="n">
         <v>0.0006066170076563114</v>
       </c>
-      <c r="H68" s="25" t="inlineStr">
+      <c r="H68" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5773,19 +7025,19 @@
       <c r="C69" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D69" s="35" t="n">
+      <c r="D69" s="69" t="n">
         <v>0.586842</v>
       </c>
-      <c r="E69" s="35" t="n">
+      <c r="E69" s="69" t="n">
         <v>0.118045</v>
       </c>
-      <c r="F69" s="35" t="n">
+      <c r="F69" s="69" t="n">
         <v>0.295113</v>
       </c>
-      <c r="G69" s="31" t="n">
+      <c r="G69" s="65" t="n">
         <v>0.0006057789423692359</v>
       </c>
-      <c r="H69" s="25" t="inlineStr">
+      <c r="H69" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5805,19 +7057,19 @@
       <c r="C70" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D70" s="35" t="n">
+      <c r="D70" s="69" t="n">
         <v>0.5421049999999999</v>
       </c>
-      <c r="E70" s="35" t="n">
+      <c r="E70" s="69" t="n">
         <v>0.130827</v>
       </c>
-      <c r="F70" s="35" t="n">
+      <c r="F70" s="69" t="n">
         <v>0.327068</v>
       </c>
-      <c r="G70" s="31" t="n">
+      <c r="G70" s="65" t="n">
         <v>0.0006050440821113034</v>
       </c>
-      <c r="H70" s="25" t="inlineStr">
+      <c r="H70" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5837,19 +7089,19 @@
       <c r="C71" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D71" s="35" t="n">
+      <c r="D71" s="69" t="n">
         <v>0.497368</v>
       </c>
-      <c r="E71" s="35" t="n">
+      <c r="E71" s="69" t="n">
         <v>0.143609</v>
       </c>
-      <c r="F71" s="35" t="n">
+      <c r="F71" s="69" t="n">
         <v>0.359023</v>
       </c>
-      <c r="G71" s="31" t="n">
+      <c r="G71" s="65" t="n">
         <v>0.0006043949529175177</v>
       </c>
-      <c r="H71" s="25" t="inlineStr">
+      <c r="H71" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5869,19 +7121,19 @@
       <c r="C72" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D72" s="35" t="n">
+      <c r="D72" s="69" t="n">
         <v>0.452632</v>
       </c>
-      <c r="E72" s="35" t="n">
+      <c r="E72" s="69" t="n">
         <v>0.156391</v>
       </c>
-      <c r="F72" s="35" t="n">
+      <c r="F72" s="69" t="n">
         <v>0.390977</v>
       </c>
-      <c r="G72" s="31" t="n">
+      <c r="G72" s="65" t="n">
         <v>0.0006038177336590362</v>
       </c>
-      <c r="H72" s="25" t="inlineStr">
+      <c r="H72" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5901,19 +7153,19 @@
       <c r="C73" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D73" s="35" t="n">
+      <c r="D73" s="69" t="n">
         <v>0.407895</v>
       </c>
-      <c r="E73" s="35" t="n">
+      <c r="E73" s="69" t="n">
         <v>0.169173</v>
       </c>
-      <c r="F73" s="35" t="n">
+      <c r="F73" s="69" t="n">
         <v>0.422932</v>
       </c>
-      <c r="G73" s="31" t="n">
+      <c r="G73" s="65" t="n">
         <v>0.0006033013642003349</v>
       </c>
-      <c r="H73" s="25" t="inlineStr">
+      <c r="H73" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5933,19 +7185,19 @@
       <c r="C74" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D74" s="35" t="n">
+      <c r="D74" s="69" t="n">
         <v>0.363158</v>
       </c>
-      <c r="E74" s="35" t="n">
+      <c r="E74" s="69" t="n">
         <v>0.181955</v>
       </c>
-      <c r="F74" s="35" t="n">
+      <c r="F74" s="69" t="n">
         <v>0.454887</v>
       </c>
-      <c r="G74" s="31" t="n">
+      <c r="G74" s="65" t="n">
         <v>0.0006028368997837505</v>
       </c>
-      <c r="H74" s="25" t="inlineStr">
+      <c r="H74" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5965,19 +7217,19 @@
       <c r="C75" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D75" s="35" t="n">
+      <c r="D75" s="69" t="n">
         <v>0.318421</v>
       </c>
-      <c r="E75" s="35" t="n">
+      <c r="E75" s="69" t="n">
         <v>0.194737</v>
       </c>
-      <c r="F75" s="35" t="n">
+      <c r="F75" s="69" t="n">
         <v>0.486842</v>
       </c>
-      <c r="G75" s="31" t="n">
+      <c r="G75" s="65" t="n">
         <v>0.0006024170362593856</v>
       </c>
-      <c r="H75" s="25" t="inlineStr">
+      <c r="H75" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5997,19 +7249,19 @@
       <c r="C76" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D76" s="35" t="n">
+      <c r="D76" s="69" t="n">
         <v>0.273684</v>
       </c>
-      <c r="E76" s="35" t="n">
+      <c r="E76" s="69" t="n">
         <v>0.207519</v>
       </c>
-      <c r="F76" s="35" t="n">
+      <c r="F76" s="69" t="n">
         <v>0.518797</v>
       </c>
-      <c r="G76" s="31" t="n">
+      <c r="G76" s="65" t="n">
         <v>0.0006020357560719341</v>
       </c>
-      <c r="H76" s="25" t="inlineStr">
+      <c r="H76" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6029,19 +7281,19 @@
       <c r="C77" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D77" s="35" t="n">
+      <c r="D77" s="69" t="n">
         <v>0.228947</v>
       </c>
-      <c r="E77" s="35" t="n">
+      <c r="E77" s="69" t="n">
         <v>0.220301</v>
       </c>
-      <c r="F77" s="35" t="n">
+      <c r="F77" s="69" t="n">
         <v>0.550752</v>
       </c>
-      <c r="G77" s="31" t="n">
+      <c r="G77" s="65" t="n">
         <v>0.0006016880609681081</v>
       </c>
-      <c r="H77" s="25" t="inlineStr">
+      <c r="H77" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6061,19 +7313,19 @@
       <c r="C78" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D78" s="35" t="n">
+      <c r="D78" s="69" t="n">
         <v>0.184211</v>
       </c>
-      <c r="E78" s="35" t="n">
+      <c r="E78" s="69" t="n">
         <v>0.233083</v>
       </c>
-      <c r="F78" s="35" t="n">
+      <c r="F78" s="69" t="n">
         <v>0.582707</v>
       </c>
-      <c r="G78" s="31" t="n">
+      <c r="G78" s="65" t="n">
         <v>0.0003420427646720472</v>
       </c>
-      <c r="H78" s="25" t="inlineStr">
+      <c r="H78" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#2</t>
         </is>
@@ -6093,19 +7345,19 @@
       <c r="C79" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D79" s="35" t="n">
+      <c r="D79" s="69" t="n">
         <v>0.139474</v>
       </c>
-      <c r="E79" s="35" t="n">
+      <c r="E79" s="69" t="n">
         <v>0.245865</v>
       </c>
-      <c r="F79" s="35" t="n">
+      <c r="F79" s="69" t="n">
         <v>0.614662</v>
       </c>
-      <c r="G79" s="31" t="n">
+      <c r="G79" s="65" t="n">
         <v>0.0001478601310591977</v>
       </c>
-      <c r="H79" s="25" t="inlineStr">
+      <c r="H79" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#2</t>
         </is>
@@ -6125,26 +7377,26 @@
       <c r="C80" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D80" s="35" t="n">
+      <c r="D80" s="69" t="n">
         <v>0.094737</v>
       </c>
-      <c r="E80" s="35" t="n">
+      <c r="E80" s="69" t="n">
         <v>0.258647</v>
       </c>
-      <c r="F80" s="35" t="n">
+      <c r="F80" s="69" t="n">
         <v>0.646617</v>
       </c>
-      <c r="G80" s="31" t="n">
+      <c r="G80" s="65" t="n">
         <v>6.016951044280985e-05</v>
       </c>
-      <c r="H80" s="25" t="inlineStr">
+      <c r="H80" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#2</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="26" t="inlineStr">
+      <c r="A81" s="60" t="inlineStr">
         <is>
           <t>Cu-V-O</t>
         </is>
@@ -6157,19 +7409,19 @@
       <c r="C81" s="15" t="n">
         <v>1800</v>
       </c>
-      <c r="D81" s="36" t="n">
+      <c r="D81" s="70" t="n">
         <v>0.05</v>
       </c>
-      <c r="E81" s="36" t="n">
+      <c r="E81" s="70" t="n">
         <v>0.271429</v>
       </c>
-      <c r="F81" s="36" t="n">
+      <c r="F81" s="70" t="n">
         <v>0.678571</v>
       </c>
-      <c r="G81" s="33" t="n">
+      <c r="G81" s="67" t="n">
         <v>3.304376173394248e-05</v>
       </c>
-      <c r="H81" s="27" t="inlineStr">
+      <c r="H81" s="61" t="inlineStr">
         <is>
           <t>GAS#1; IONIC_LIQ#2</t>
         </is>
@@ -6180,7 +7432,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6244,7 +7496,7 @@
           <t>Fine-resolution dG vs T for top 6 ternary candidates (25 K steps, 800-1900 K)</t>
         </is>
       </c>
-      <c r="E2" s="24" t="inlineStr">
+      <c r="E2" s="58" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
@@ -6271,7 +7523,7 @@
           <t>CuFe2O4 formation decomposed into Cu-capture vs Fe-oxidation components (50 K steps, 800-1900 K)</t>
         </is>
       </c>
-      <c r="E3" s="25" t="inlineStr">
+      <c r="E3" s="59" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
@@ -6298,7 +7550,7 @@
           <t>Pre-computed Fe-oxidation and Cu-capture percentages</t>
         </is>
       </c>
-      <c r="E4" s="24" t="inlineStr">
+      <c r="E4" s="58" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
@@ -6325,7 +7577,7 @@
           <t>Cu activity in quaternary slag systems (Cu-Mn-Si-O, Cu-Al-Si-O) vs basicity ratio at 1800 K</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="59" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
@@ -6337,22 +7589,22 @@
           <t>cu_activity_vs_oxide.csv</t>
         </is>
       </c>
-      <c r="B6" s="37" t="inlineStr">
+      <c r="B6" s="45" t="inlineStr">
         <is>
           <t>simulations/tcpython/cu_activity_vs_oxide.py</t>
         </is>
       </c>
-      <c r="C6" s="37" t="inlineStr">
+      <c r="C6" s="45" t="inlineStr">
         <is>
           <t>TCOX14</t>
         </is>
       </c>
-      <c r="D6" s="37" t="inlineStr">
+      <c r="D6" s="45" t="inlineStr">
         <is>
           <t>Cu activity sweep at 1800 K across 4 ternary systems (Cu-Al-O, Cu-Mn-O, Cu-Fe-O, Cu-V-O), 20 compositions each</t>
         </is>
       </c>
-      <c r="E6" s="38" t="inlineStr">
+      <c r="E6" s="71" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>

</xml_diff>

<commit_message>
Revert xlsx files opened for reading (Excel bloat, no actual edits)
Oxide_Screening_Complete.xlsx ballooned from 24KB to 600KB just from
being opened in Excel. All three xlsx files reverted to previous state.
</commit_message>
<xml_diff>
--- a/screening/Validation_Results.xlsx
+++ b/screening/Validation_Results.xlsx
@@ -9,11 +9,10 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dG_vs_T" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CuFe2O4_Decomposition" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity_Correction" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Ranking" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slag_Effects" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cu_Activity" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Sources" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Ranking" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slag_Effects" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cu_Activity" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Sources" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,17 +21,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="+0.00;-0.00;0.00"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="+0.0;-0.0"/>
-    <numFmt numFmtId="169" formatCode="+0.0;-0.0;0.0"/>
-    <numFmt numFmtId="170" formatCode="0.0000E+00"/>
-    <numFmt numFmtId="171" formatCode="0.000000"/>
+    <numFmt numFmtId="166" formatCode="0.0000E+00"/>
+    <numFmt numFmtId="167" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,15 +43,6 @@
     <font>
       <b val="1"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00666666"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="5">
@@ -151,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -222,78 +208,6 @@
     <xf numFmtId="165" fontId="0" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="3" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -309,28 +223,31 @@
     <xf numFmtId="165" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -340,24 +257,6 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00C6EFCE"/>
-          <bgColor rgb="00C6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFC7CE"/>
-          <bgColor rgb="00FFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -2603,1157 +2502,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="24" t="inlineStr">
-        <is>
-          <t>ACTIVITY CORRECTION PARAMETERS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="25" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="B2" s="26" t="inlineStr">
-        <is>
-          <t>Symbol</t>
-        </is>
-      </c>
-      <c r="C2" s="26" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D2" s="27" t="inlineStr">
-        <is>
-          <t>Unit / Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="28" t="inlineStr">
-        <is>
-          <t>Cu mole fraction in steel</t>
-        </is>
-      </c>
-      <c r="B3" s="29" t="inlineStr">
-        <is>
-          <t>X_Cu</t>
-        </is>
-      </c>
-      <c r="C3" s="30" t="n">
-        <v>0.003</v>
-      </c>
-      <c r="D3" s="31" t="inlineStr">
-        <is>
-          <t>~0.3 wt% Cu</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="32" t="inlineStr">
-        <is>
-          <t>Raoultian activity coefficient</t>
-        </is>
-      </c>
-      <c r="B4" s="33" t="inlineStr">
-        <is>
-          <t>γ_Cu</t>
-        </is>
-      </c>
-      <c r="C4" s="34" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="D4" s="35" t="inlineStr">
-        <is>
-          <t>Literature range: 5-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="28" t="inlineStr">
-        <is>
-          <t>Cu activity in liquid Fe</t>
-        </is>
-      </c>
-      <c r="B5" s="29" t="inlineStr">
-        <is>
-          <t>a_Cu</t>
-        </is>
-      </c>
-      <c r="C5" s="30">
-        <f>C3*C4</f>
-        <v/>
-      </c>
-      <c r="D5" s="31" t="inlineStr">
-        <is>
-          <t>X_Cu × γ_Cu</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="32" t="inlineStr">
-        <is>
-          <t>Temperature</t>
-        </is>
-      </c>
-      <c r="B6" s="33" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="C6" s="33" t="n">
-        <v>1800</v>
-      </c>
-      <c r="D6" s="35" t="inlineStr">
-        <is>
-          <t>K (steelmaking)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="28" t="inlineStr">
-        <is>
-          <t>Gas constant</t>
-        </is>
-      </c>
-      <c r="B7" s="29" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="C7" s="36" t="n">
-        <v>8.314</v>
-      </c>
-      <c r="D7" s="31" t="inlineStr">
-        <is>
-          <t>J/(mol·K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="37" t="inlineStr">
-        <is>
-          <t>Penalty per Cu atom consumed</t>
-        </is>
-      </c>
-      <c r="B8" s="38" t="inlineStr">
-        <is>
-          <t>-RT·ln(a_Cu)</t>
-        </is>
-      </c>
-      <c r="C8" s="39">
-        <f>-C7*C6*LN(C5)/1000</f>
-        <v/>
-      </c>
-      <c r="D8" s="40" t="inlineStr">
-        <is>
-          <t>kJ/mol (positive = less favorable)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="24" t="inlineStr">
-        <is>
-          <t>ACTIVITY-CORRECTED ΔG AT 1800 K</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Parent Oxide</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>n_Cu</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>ΔG° (kJ)</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Cu Penalty (kJ)</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>ΔG_eff (kJ)</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Verdict</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>ΔG per Cu (kJ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>CuFe2O4</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>FeO</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="41" t="n">
-        <v>-111.88</v>
-      </c>
-      <c r="E12" s="41">
-        <f>C12*$C$8</f>
-        <v/>
-      </c>
-      <c r="F12" s="41">
-        <f>D12+E12</f>
-        <v/>
-      </c>
-      <c r="G12" s="12">
-        <f>IF(F12&lt;-10,"ROBUST",IF(F12&lt;0,"MARGINAL",IF(F12&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
-        <v/>
-      </c>
-      <c r="H12" s="42">
-        <f>D12/C12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>CuMn2O4</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>MnO</t>
-        </is>
-      </c>
-      <c r="C13" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="43" t="n">
-        <v>-64.44</v>
-      </c>
-      <c r="E13" s="43">
-        <f>C13*$C$8</f>
-        <v/>
-      </c>
-      <c r="F13" s="43">
-        <f>D13+E13</f>
-        <v/>
-      </c>
-      <c r="G13" s="13">
-        <f>IF(F13&lt;-10,"ROBUST",IF(F13&lt;0,"MARGINAL",IF(F13&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
-        <v/>
-      </c>
-      <c r="H13" s="44">
-        <f>D13/C13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>CuB2O4</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>B2O3</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="41" t="n">
-        <v>-47.71</v>
-      </c>
-      <c r="E14" s="41">
-        <f>C14*$C$8</f>
-        <v/>
-      </c>
-      <c r="F14" s="41">
-        <f>D14+E14</f>
-        <v/>
-      </c>
-      <c r="G14" s="12">
-        <f>IF(F14&lt;-10,"ROBUST",IF(F14&lt;0,"MARGINAL",IF(F14&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
-        <v/>
-      </c>
-      <c r="H14" s="42">
-        <f>D14/C14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>CuV2O6</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="inlineStr">
-        <is>
-          <t>V2O5</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="43" t="n">
-        <v>-44.98</v>
-      </c>
-      <c r="E15" s="43">
-        <f>C15*$C$8</f>
-        <v/>
-      </c>
-      <c r="F15" s="43">
-        <f>D15+E15</f>
-        <v/>
-      </c>
-      <c r="G15" s="13">
-        <f>IF(F15&lt;-10,"ROBUST",IF(F15&lt;0,"MARGINAL",IF(F15&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
-        <v/>
-      </c>
-      <c r="H15" s="44">
-        <f>D15/C15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>CuAl2O4</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>Al2O3</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="41" t="n">
-        <v>-32.31</v>
-      </c>
-      <c r="E16" s="41">
-        <f>C16*$C$8</f>
-        <v/>
-      </c>
-      <c r="F16" s="41">
-        <f>D16+E16</f>
-        <v/>
-      </c>
-      <c r="G16" s="12">
-        <f>IF(F16&lt;-10,"ROBUST",IF(F16&lt;0,"MARGINAL",IF(F16&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
-        <v/>
-      </c>
-      <c r="H16" s="42">
-        <f>D16/C16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Cu3V2O8</t>
-        </is>
-      </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>V2O5</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D17" s="43" t="n">
-        <v>-109.15</v>
-      </c>
-      <c r="E17" s="43">
-        <f>C17*$C$8</f>
-        <v/>
-      </c>
-      <c r="F17" s="43">
-        <f>D17+E17</f>
-        <v/>
-      </c>
-      <c r="G17" s="13">
-        <f>IF(F17&lt;-10,"ROBUST",IF(F17&lt;0,"MARGINAL",IF(F17&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
-        <v/>
-      </c>
-      <c r="H17" s="44">
-        <f>D17/C17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="20" t="inlineStr">
-        <is>
-          <t>Cu2SiO4</t>
-        </is>
-      </c>
-      <c r="B18" s="45" t="inlineStr">
-        <is>
-          <t>SiO2</t>
-        </is>
-      </c>
-      <c r="C18" s="45" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="46" t="n">
-        <v>-52.21</v>
-      </c>
-      <c r="E18" s="46">
-        <f>C18*$C$8</f>
-        <v/>
-      </c>
-      <c r="F18" s="46">
-        <f>D18+E18</f>
-        <v/>
-      </c>
-      <c r="G18" s="45">
-        <f>IF(F18&lt;-10,"ROBUST",IF(F18&lt;0,"MARGINAL",IF(F18&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
-        <v/>
-      </c>
-      <c r="H18" s="47">
-        <f>D18/C18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="24" t="inlineStr">
-        <is>
-          <t>γ_Cu SENSITIVITY ANALYSIS</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="48" t="inlineStr">
-        <is>
-          <t>Change γ_Cu in cell C4 above to see all corrections update automatically.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>γ_Cu</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>a_Cu</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Penalty/Cu (kJ)</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>ΔG_eff CuFe2O4</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>ΔG_eff CuMn2O4</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>ΔG_eff CuB2O4</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>ΔG_eff CuV2O6</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>ΔG_eff CuAl2O4</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>ΔG_eff Cu3V2O8</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>ΔG_eff Cu2SiO4</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="49" t="n">
-        <v>3</v>
-      </c>
-      <c r="B23" s="50">
-        <f>A23*$C$3</f>
-        <v/>
-      </c>
-      <c r="C23" s="51">
-        <f>-$C$7*$C$6*LN(B23)/1000</f>
-        <v/>
-      </c>
-      <c r="D23" s="41">
-        <f>-111.88+1*C23</f>
-        <v/>
-      </c>
-      <c r="E23" s="41">
-        <f>-64.44+1*C23</f>
-        <v/>
-      </c>
-      <c r="F23" s="41">
-        <f>-47.71+1*C23</f>
-        <v/>
-      </c>
-      <c r="G23" s="41">
-        <f>-44.98+1*C23</f>
-        <v/>
-      </c>
-      <c r="H23" s="41">
-        <f>-32.31+1*C23</f>
-        <v/>
-      </c>
-      <c r="I23" s="41">
-        <f>-109.15+3*C23</f>
-        <v/>
-      </c>
-      <c r="J23" s="42">
-        <f>-52.21+2*C23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="52" t="n">
-        <v>4</v>
-      </c>
-      <c r="B24" s="53">
-        <f>A24*$C$3</f>
-        <v/>
-      </c>
-      <c r="C24" s="54">
-        <f>-$C$7*$C$6*LN(B24)/1000</f>
-        <v/>
-      </c>
-      <c r="D24" s="43">
-        <f>-111.88+1*C24</f>
-        <v/>
-      </c>
-      <c r="E24" s="43">
-        <f>-64.44+1*C24</f>
-        <v/>
-      </c>
-      <c r="F24" s="43">
-        <f>-47.71+1*C24</f>
-        <v/>
-      </c>
-      <c r="G24" s="43">
-        <f>-44.98+1*C24</f>
-        <v/>
-      </c>
-      <c r="H24" s="43">
-        <f>-32.31+1*C24</f>
-        <v/>
-      </c>
-      <c r="I24" s="43">
-        <f>-109.15+3*C24</f>
-        <v/>
-      </c>
-      <c r="J24" s="44">
-        <f>-52.21+2*C24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="49" t="n">
-        <v>5</v>
-      </c>
-      <c r="B25" s="50">
-        <f>A25*$C$3</f>
-        <v/>
-      </c>
-      <c r="C25" s="51">
-        <f>-$C$7*$C$6*LN(B25)/1000</f>
-        <v/>
-      </c>
-      <c r="D25" s="41">
-        <f>-111.88+1*C25</f>
-        <v/>
-      </c>
-      <c r="E25" s="41">
-        <f>-64.44+1*C25</f>
-        <v/>
-      </c>
-      <c r="F25" s="41">
-        <f>-47.71+1*C25</f>
-        <v/>
-      </c>
-      <c r="G25" s="41">
-        <f>-44.98+1*C25</f>
-        <v/>
-      </c>
-      <c r="H25" s="41">
-        <f>-32.31+1*C25</f>
-        <v/>
-      </c>
-      <c r="I25" s="41">
-        <f>-109.15+3*C25</f>
-        <v/>
-      </c>
-      <c r="J25" s="42">
-        <f>-52.21+2*C25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="52" t="n">
-        <v>6</v>
-      </c>
-      <c r="B26" s="53">
-        <f>A26*$C$3</f>
-        <v/>
-      </c>
-      <c r="C26" s="54">
-        <f>-$C$7*$C$6*LN(B26)/1000</f>
-        <v/>
-      </c>
-      <c r="D26" s="43">
-        <f>-111.88+1*C26</f>
-        <v/>
-      </c>
-      <c r="E26" s="43">
-        <f>-64.44+1*C26</f>
-        <v/>
-      </c>
-      <c r="F26" s="43">
-        <f>-47.71+1*C26</f>
-        <v/>
-      </c>
-      <c r="G26" s="43">
-        <f>-44.98+1*C26</f>
-        <v/>
-      </c>
-      <c r="H26" s="43">
-        <f>-32.31+1*C26</f>
-        <v/>
-      </c>
-      <c r="I26" s="43">
-        <f>-109.15+3*C26</f>
-        <v/>
-      </c>
-      <c r="J26" s="44">
-        <f>-52.21+2*C26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="49" t="n">
-        <v>7</v>
-      </c>
-      <c r="B27" s="50">
-        <f>A27*$C$3</f>
-        <v/>
-      </c>
-      <c r="C27" s="51">
-        <f>-$C$7*$C$6*LN(B27)/1000</f>
-        <v/>
-      </c>
-      <c r="D27" s="41">
-        <f>-111.88+1*C27</f>
-        <v/>
-      </c>
-      <c r="E27" s="41">
-        <f>-64.44+1*C27</f>
-        <v/>
-      </c>
-      <c r="F27" s="41">
-        <f>-47.71+1*C27</f>
-        <v/>
-      </c>
-      <c r="G27" s="41">
-        <f>-44.98+1*C27</f>
-        <v/>
-      </c>
-      <c r="H27" s="41">
-        <f>-32.31+1*C27</f>
-        <v/>
-      </c>
-      <c r="I27" s="41">
-        <f>-109.15+3*C27</f>
-        <v/>
-      </c>
-      <c r="J27" s="42">
-        <f>-52.21+2*C27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="52" t="n">
-        <v>8</v>
-      </c>
-      <c r="B28" s="53">
-        <f>A28*$C$3</f>
-        <v/>
-      </c>
-      <c r="C28" s="54">
-        <f>-$C$7*$C$6*LN(B28)/1000</f>
-        <v/>
-      </c>
-      <c r="D28" s="43">
-        <f>-111.88+1*C28</f>
-        <v/>
-      </c>
-      <c r="E28" s="43">
-        <f>-64.44+1*C28</f>
-        <v/>
-      </c>
-      <c r="F28" s="43">
-        <f>-47.71+1*C28</f>
-        <v/>
-      </c>
-      <c r="G28" s="43">
-        <f>-44.98+1*C28</f>
-        <v/>
-      </c>
-      <c r="H28" s="43">
-        <f>-32.31+1*C28</f>
-        <v/>
-      </c>
-      <c r="I28" s="43">
-        <f>-109.15+3*C28</f>
-        <v/>
-      </c>
-      <c r="J28" s="44">
-        <f>-52.21+2*C28</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="49" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="B29" s="50">
-        <f>A29*$C$3</f>
-        <v/>
-      </c>
-      <c r="C29" s="51">
-        <f>-$C$7*$C$6*LN(B29)/1000</f>
-        <v/>
-      </c>
-      <c r="D29" s="41">
-        <f>-111.88+1*C29</f>
-        <v/>
-      </c>
-      <c r="E29" s="41">
-        <f>-64.44+1*C29</f>
-        <v/>
-      </c>
-      <c r="F29" s="41">
-        <f>-47.71+1*C29</f>
-        <v/>
-      </c>
-      <c r="G29" s="41">
-        <f>-44.98+1*C29</f>
-        <v/>
-      </c>
-      <c r="H29" s="41">
-        <f>-32.31+1*C29</f>
-        <v/>
-      </c>
-      <c r="I29" s="41">
-        <f>-109.15+3*C29</f>
-        <v/>
-      </c>
-      <c r="J29" s="42">
-        <f>-52.21+2*C29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="52" t="n">
-        <v>9</v>
-      </c>
-      <c r="B30" s="53">
-        <f>A30*$C$3</f>
-        <v/>
-      </c>
-      <c r="C30" s="54">
-        <f>-$C$7*$C$6*LN(B30)/1000</f>
-        <v/>
-      </c>
-      <c r="D30" s="43">
-        <f>-111.88+1*C30</f>
-        <v/>
-      </c>
-      <c r="E30" s="43">
-        <f>-64.44+1*C30</f>
-        <v/>
-      </c>
-      <c r="F30" s="43">
-        <f>-47.71+1*C30</f>
-        <v/>
-      </c>
-      <c r="G30" s="43">
-        <f>-44.98+1*C30</f>
-        <v/>
-      </c>
-      <c r="H30" s="43">
-        <f>-32.31+1*C30</f>
-        <v/>
-      </c>
-      <c r="I30" s="43">
-        <f>-109.15+3*C30</f>
-        <v/>
-      </c>
-      <c r="J30" s="44">
-        <f>-52.21+2*C30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="49" t="n">
-        <v>10</v>
-      </c>
-      <c r="B31" s="50">
-        <f>A31*$C$3</f>
-        <v/>
-      </c>
-      <c r="C31" s="51">
-        <f>-$C$7*$C$6*LN(B31)/1000</f>
-        <v/>
-      </c>
-      <c r="D31" s="41">
-        <f>-111.88+1*C31</f>
-        <v/>
-      </c>
-      <c r="E31" s="41">
-        <f>-64.44+1*C31</f>
-        <v/>
-      </c>
-      <c r="F31" s="41">
-        <f>-47.71+1*C31</f>
-        <v/>
-      </c>
-      <c r="G31" s="41">
-        <f>-44.98+1*C31</f>
-        <v/>
-      </c>
-      <c r="H31" s="41">
-        <f>-32.31+1*C31</f>
-        <v/>
-      </c>
-      <c r="I31" s="41">
-        <f>-109.15+3*C31</f>
-        <v/>
-      </c>
-      <c r="J31" s="42">
-        <f>-52.21+2*C31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="52" t="n">
-        <v>11</v>
-      </c>
-      <c r="B32" s="53">
-        <f>A32*$C$3</f>
-        <v/>
-      </c>
-      <c r="C32" s="54">
-        <f>-$C$7*$C$6*LN(B32)/1000</f>
-        <v/>
-      </c>
-      <c r="D32" s="43">
-        <f>-111.88+1*C32</f>
-        <v/>
-      </c>
-      <c r="E32" s="43">
-        <f>-64.44+1*C32</f>
-        <v/>
-      </c>
-      <c r="F32" s="43">
-        <f>-47.71+1*C32</f>
-        <v/>
-      </c>
-      <c r="G32" s="43">
-        <f>-44.98+1*C32</f>
-        <v/>
-      </c>
-      <c r="H32" s="43">
-        <f>-32.31+1*C32</f>
-        <v/>
-      </c>
-      <c r="I32" s="43">
-        <f>-109.15+3*C32</f>
-        <v/>
-      </c>
-      <c r="J32" s="44">
-        <f>-52.21+2*C32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="49" t="n">
-        <v>12</v>
-      </c>
-      <c r="B33" s="50">
-        <f>A33*$C$3</f>
-        <v/>
-      </c>
-      <c r="C33" s="51">
-        <f>-$C$7*$C$6*LN(B33)/1000</f>
-        <v/>
-      </c>
-      <c r="D33" s="41">
-        <f>-111.88+1*C33</f>
-        <v/>
-      </c>
-      <c r="E33" s="41">
-        <f>-64.44+1*C33</f>
-        <v/>
-      </c>
-      <c r="F33" s="41">
-        <f>-47.71+1*C33</f>
-        <v/>
-      </c>
-      <c r="G33" s="41">
-        <f>-44.98+1*C33</f>
-        <v/>
-      </c>
-      <c r="H33" s="41">
-        <f>-32.31+1*C33</f>
-        <v/>
-      </c>
-      <c r="I33" s="41">
-        <f>-109.15+3*C33</f>
-        <v/>
-      </c>
-      <c r="J33" s="42">
-        <f>-52.21+2*C33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="52" t="n">
-        <v>13</v>
-      </c>
-      <c r="B34" s="53">
-        <f>A34*$C$3</f>
-        <v/>
-      </c>
-      <c r="C34" s="54">
-        <f>-$C$7*$C$6*LN(B34)/1000</f>
-        <v/>
-      </c>
-      <c r="D34" s="43">
-        <f>-111.88+1*C34</f>
-        <v/>
-      </c>
-      <c r="E34" s="43">
-        <f>-64.44+1*C34</f>
-        <v/>
-      </c>
-      <c r="F34" s="43">
-        <f>-47.71+1*C34</f>
-        <v/>
-      </c>
-      <c r="G34" s="43">
-        <f>-44.98+1*C34</f>
-        <v/>
-      </c>
-      <c r="H34" s="43">
-        <f>-32.31+1*C34</f>
-        <v/>
-      </c>
-      <c r="I34" s="43">
-        <f>-109.15+3*C34</f>
-        <v/>
-      </c>
-      <c r="J34" s="44">
-        <f>-52.21+2*C34</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="55" t="n">
-        <v>15</v>
-      </c>
-      <c r="B35" s="56">
-        <f>A35*$C$3</f>
-        <v/>
-      </c>
-      <c r="C35" s="57">
-        <f>-$C$7*$C$6*LN(B35)/1000</f>
-        <v/>
-      </c>
-      <c r="D35" s="46">
-        <f>-111.88+1*C35</f>
-        <v/>
-      </c>
-      <c r="E35" s="46">
-        <f>-64.44+1*C35</f>
-        <v/>
-      </c>
-      <c r="F35" s="46">
-        <f>-47.71+1*C35</f>
-        <v/>
-      </c>
-      <c r="G35" s="46">
-        <f>-44.98+1*C35</f>
-        <v/>
-      </c>
-      <c r="H35" s="46">
-        <f>-32.31+1*C35</f>
-        <v/>
-      </c>
-      <c r="I35" s="46">
-        <f>-109.15+3*C35</f>
-        <v/>
-      </c>
-      <c r="J35" s="47">
-        <f>-52.21+2*C35</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="48" t="inlineStr">
-        <is>
-          <t>NOTE: V₂O₅ can form either Cu₃V₂O₈ (3 Cu, ΔG° = -109.2 kJ) or CuV₂O₆ (1 Cu, ΔG° = -45.0 kJ). Under dilute Cu conditions, CuV₂O₆ is preferred because the 3× penalty makes Cu₃V₂O₈ unfavorable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="48" t="inlineStr">
-        <is>
-          <t>Bureau of Mines (1960s) used ~1 wt% Cu (a_Cu ≈ 0.13), where both V₂O₅ products are favorable. Their 40-60% removal is consistent with our model.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A37:H37"/>
-  </mergeCells>
-  <conditionalFormatting sqref="D23:D35">
-    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E23:E35">
-    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="greaterThanOrEqual" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F23:F35">
-    <cfRule type="cellIs" priority="5" operator="lessThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="6" operator="greaterThanOrEqual" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G23:G35">
-    <cfRule type="cellIs" priority="7" operator="lessThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H23:H35">
-    <cfRule type="cellIs" priority="9" operator="lessThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="10" operator="greaterThanOrEqual" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I23:I35">
-    <cfRule type="cellIs" priority="11" operator="lessThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="12" operator="greaterThanOrEqual" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J23:J35">
-    <cfRule type="cellIs" priority="13" operator="lessThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="14" operator="greaterThanOrEqual" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F12:F18">
-    <cfRule type="cellIs" priority="15" operator="lessThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="16" operator="greaterThanOrEqual" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3809,7 +2557,7 @@
       <c r="D2" s="12" t="n">
         <v>1700</v>
       </c>
-      <c r="E2" s="58" t="inlineStr">
+      <c r="E2" s="24" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
@@ -3835,7 +2583,7 @@
           <t>N/A (liquid)</t>
         </is>
       </c>
-      <c r="E3" s="59" t="inlineStr">
+      <c r="E3" s="25" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
@@ -3859,7 +2607,7 @@
       <c r="D4" s="12" t="n">
         <v>1700</v>
       </c>
-      <c r="E4" s="58" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
@@ -3885,7 +2633,7 @@
           <t>N/A (liquid)</t>
         </is>
       </c>
-      <c r="E5" s="59" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
@@ -3909,14 +2657,14 @@
       <c r="D6" s="12" t="n">
         <v>1300</v>
       </c>
-      <c r="E6" s="58" t="inlineStr">
+      <c r="E6" s="24" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="60" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>CuAl2O4</t>
         </is>
@@ -3933,7 +2681,7 @@
       <c r="D7" s="15" t="n">
         <v>1550</v>
       </c>
-      <c r="E7" s="61" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
@@ -3944,7 +2692,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4004,10 +2752,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C2" s="62" t="n">
+      <c r="C2" s="28" t="n">
         <v>0.2</v>
       </c>
-      <c r="D2" s="63" t="n">
+      <c r="D2" s="29" t="n">
         <v>0.0006024287195135149</v>
       </c>
       <c r="E2" s="12" t="inlineStr">
@@ -4030,10 +2778,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C3" s="62" t="n">
+      <c r="C3" s="28" t="n">
         <v>0.4</v>
       </c>
-      <c r="D3" s="63" t="n">
+      <c r="D3" s="29" t="n">
         <v>0.0005921646682545373</v>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -4057,10 +2805,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C4" s="62" t="n">
+      <c r="C4" s="28" t="n">
         <v>0.6</v>
       </c>
-      <c r="D4" s="63" t="n">
+      <c r="D4" s="29" t="n">
         <v>0.0005849859614188124</v>
       </c>
       <c r="E4" s="12" t="inlineStr">
@@ -4084,10 +2832,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C5" s="62" t="n">
+      <c r="C5" s="28" t="n">
         <v>0.8</v>
       </c>
-      <c r="D5" s="63" t="n">
+      <c r="D5" s="29" t="n">
         <v>0.0005795578709134352</v>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -4111,10 +2859,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C6" s="62" t="n">
+      <c r="C6" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="63" t="n">
+      <c r="D6" s="29" t="n">
         <v>0.0005747540319710688</v>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -4138,10 +2886,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C7" s="62" t="n">
+      <c r="C7" s="28" t="n">
         <v>1.2</v>
       </c>
-      <c r="D7" s="63" t="n">
+      <c r="D7" s="29" t="n">
         <v>0.0005690086100650586</v>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -4165,10 +2913,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C8" s="62" t="n">
+      <c r="C8" s="28" t="n">
         <v>1.4</v>
       </c>
-      <c r="D8" s="63" t="n">
+      <c r="D8" s="29" t="n">
         <v>0.0005623991726393003</v>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -4192,10 +2940,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C9" s="62" t="n">
+      <c r="C9" s="28" t="n">
         <v>1.6</v>
       </c>
-      <c r="D9" s="63" t="n">
+      <c r="D9" s="29" t="n">
         <v>0.0005549646048769486</v>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -4219,10 +2967,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C10" s="62" t="n">
+      <c r="C10" s="28" t="n">
         <v>1.8</v>
       </c>
-      <c r="D10" s="63" t="n">
+      <c r="D10" s="29" t="n">
         <v>0.0005469620453455369</v>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -4246,10 +2994,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C11" s="62" t="n">
+      <c r="C11" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="63" t="n">
+      <c r="D11" s="29" t="n">
         <v>0.0005386374910615401</v>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -4273,10 +3021,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C12" s="62" t="n">
+      <c r="C12" s="28" t="n">
         <v>2.2</v>
       </c>
-      <c r="D12" s="63" t="n">
+      <c r="D12" s="29" t="n">
         <v>0.0005302395956835024</v>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -4300,10 +3048,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C13" s="62" t="n">
+      <c r="C13" s="28" t="n">
         <v>2.4</v>
       </c>
-      <c r="D13" s="63" t="n">
+      <c r="D13" s="29" t="n">
         <v>0.0005220166239764437</v>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -4327,10 +3075,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C14" s="62" t="n">
+      <c r="C14" s="28" t="n">
         <v>2.6</v>
       </c>
-      <c r="D14" s="63" t="n">
+      <c r="D14" s="29" t="n">
         <v>0.0005141731215264483</v>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -4354,10 +3102,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C15" s="62" t="n">
+      <c r="C15" s="28" t="n">
         <v>2.8</v>
       </c>
-      <c r="D15" s="63" t="n">
+      <c r="D15" s="29" t="n">
         <v>0.000506844968432079</v>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -4381,10 +3129,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C16" s="62" t="n">
+      <c r="C16" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="D16" s="63" t="n">
+      <c r="D16" s="29" t="n">
         <v>0.0005001045724686611</v>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -4408,10 +3156,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C17" s="64" t="n">
+      <c r="C17" s="30" t="n">
         <v>0.2</v>
       </c>
-      <c r="D17" s="65" t="n">
+      <c r="D17" s="31" t="n">
         <v>0.0006238595135610499</v>
       </c>
       <c r="E17" s="13" t="inlineStr">
@@ -4434,10 +3182,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C18" s="64" t="n">
+      <c r="C18" s="30" t="n">
         <v>0.4</v>
       </c>
-      <c r="D18" s="65" t="n">
+      <c r="D18" s="31" t="n">
         <v>0.0006238595135610499</v>
       </c>
       <c r="E18" s="13" t="inlineStr">
@@ -4461,10 +3209,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C19" s="64" t="n">
+      <c r="C19" s="30" t="n">
         <v>0.6</v>
       </c>
-      <c r="D19" s="65" t="n">
+      <c r="D19" s="31" t="n">
         <v>0.0006238595135610521</v>
       </c>
       <c r="E19" s="13" t="inlineStr">
@@ -4488,10 +3236,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C20" s="64" t="n">
+      <c r="C20" s="30" t="n">
         <v>0.8</v>
       </c>
-      <c r="D20" s="65" t="n">
+      <c r="D20" s="31" t="n">
         <v>0.0006238595135610521</v>
       </c>
       <c r="E20" s="13" t="inlineStr">
@@ -4515,10 +3263,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C21" s="64" t="n">
+      <c r="C21" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="65" t="n">
+      <c r="D21" s="31" t="n">
         <v>0.0006238595135610521</v>
       </c>
       <c r="E21" s="13" t="inlineStr">
@@ -4542,10 +3290,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C22" s="64" t="n">
+      <c r="C22" s="30" t="n">
         <v>1.2</v>
       </c>
-      <c r="D22" s="65" t="n">
+      <c r="D22" s="31" t="n">
         <v>0.0006238595135610504</v>
       </c>
       <c r="E22" s="13" t="inlineStr">
@@ -4569,10 +3317,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C23" s="64" t="n">
+      <c r="C23" s="30" t="n">
         <v>1.4</v>
       </c>
-      <c r="D23" s="65" t="n">
+      <c r="D23" s="31" t="n">
         <v>0.0006238595135610504</v>
       </c>
       <c r="E23" s="13" t="inlineStr">
@@ -4596,10 +3344,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C24" s="64" t="n">
+      <c r="C24" s="30" t="n">
         <v>1.6</v>
       </c>
-      <c r="D24" s="65" t="n">
+      <c r="D24" s="31" t="n">
         <v>0.0006240110028708597</v>
       </c>
       <c r="E24" s="13" t="inlineStr">
@@ -4623,10 +3371,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C25" s="64" t="n">
+      <c r="C25" s="30" t="n">
         <v>1.8</v>
       </c>
-      <c r="D25" s="65" t="n">
+      <c r="D25" s="31" t="n">
         <v>0.0006240764395684967</v>
       </c>
       <c r="E25" s="13" t="inlineStr">
@@ -4650,10 +3398,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C26" s="64" t="n">
+      <c r="C26" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="D26" s="65" t="n">
+      <c r="D26" s="31" t="n">
         <v>0.0006240764395684967</v>
       </c>
       <c r="E26" s="13" t="inlineStr">
@@ -4677,10 +3425,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C27" s="64" t="n">
+      <c r="C27" s="30" t="n">
         <v>2.2</v>
       </c>
-      <c r="D27" s="65" t="n">
+      <c r="D27" s="31" t="n">
         <v>0.0006240764395684956</v>
       </c>
       <c r="E27" s="13" t="inlineStr">
@@ -4704,10 +3452,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C28" s="64" t="n">
+      <c r="C28" s="30" t="n">
         <v>2.4</v>
       </c>
-      <c r="D28" s="65" t="n">
+      <c r="D28" s="31" t="n">
         <v>0.0006240764395684967</v>
       </c>
       <c r="E28" s="13" t="inlineStr">
@@ -4731,10 +3479,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C29" s="64" t="n">
+      <c r="C29" s="30" t="n">
         <v>2.6</v>
       </c>
-      <c r="D29" s="65" t="n">
+      <c r="D29" s="31" t="n">
         <v>0.0006240764395684967</v>
       </c>
       <c r="E29" s="13" t="inlineStr">
@@ -4758,10 +3506,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C30" s="64" t="n">
+      <c r="C30" s="30" t="n">
         <v>2.8</v>
       </c>
-      <c r="D30" s="65" t="n">
+      <c r="D30" s="31" t="n">
         <v>0.0006240764395684973</v>
       </c>
       <c r="E30" s="13" t="inlineStr">
@@ -4775,7 +3523,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="60" t="inlineStr">
+      <c r="A31" s="26" t="inlineStr">
         <is>
           <t>Cu-Al-Si-O</t>
         </is>
@@ -4785,10 +3533,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C31" s="66" t="n">
+      <c r="C31" s="32" t="n">
         <v>3</v>
       </c>
-      <c r="D31" s="67" t="n">
+      <c r="D31" s="33" t="n">
         <v>0.0006240764395684973</v>
       </c>
       <c r="E31" s="15" t="inlineStr">
@@ -4806,7 +3554,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4881,19 +3629,19 @@
       <c r="C2" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D2" s="68" t="n">
+      <c r="D2" s="34" t="n">
         <v>0.9</v>
       </c>
-      <c r="E2" s="68" t="n">
+      <c r="E2" s="34" t="n">
         <v>0.04</v>
       </c>
-      <c r="F2" s="68" t="n">
+      <c r="F2" s="34" t="n">
         <v>0.06</v>
       </c>
-      <c r="G2" s="63" t="n">
+      <c r="G2" s="29" t="n">
         <v>0.0006242415932771841</v>
       </c>
-      <c r="H2" s="58" t="inlineStr">
+      <c r="H2" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4913,19 +3661,19 @@
       <c r="C3" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D3" s="68" t="n">
+      <c r="D3" s="34" t="n">
         <v>0.855263</v>
       </c>
-      <c r="E3" s="68" t="n">
+      <c r="E3" s="34" t="n">
         <v>0.057895</v>
       </c>
-      <c r="F3" s="68" t="n">
+      <c r="F3" s="34" t="n">
         <v>0.086842</v>
       </c>
-      <c r="G3" s="63" t="n">
+      <c r="G3" s="29" t="n">
         <v>0.000624241593277183</v>
       </c>
-      <c r="H3" s="58" t="inlineStr">
+      <c r="H3" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4945,19 +3693,19 @@
       <c r="C4" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D4" s="68" t="n">
+      <c r="D4" s="34" t="n">
         <v>0.810526</v>
       </c>
-      <c r="E4" s="68" t="n">
+      <c r="E4" s="34" t="n">
         <v>0.075789</v>
       </c>
-      <c r="F4" s="68" t="n">
+      <c r="F4" s="34" t="n">
         <v>0.113684</v>
       </c>
-      <c r="G4" s="63" t="n">
+      <c r="G4" s="29" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H4" s="58" t="inlineStr">
+      <c r="H4" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4977,19 +3725,19 @@
       <c r="C5" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D5" s="68" t="n">
+      <c r="D5" s="34" t="n">
         <v>0.7657890000000001</v>
       </c>
-      <c r="E5" s="68" t="n">
+      <c r="E5" s="34" t="n">
         <v>0.093684</v>
       </c>
-      <c r="F5" s="68" t="n">
+      <c r="F5" s="34" t="n">
         <v>0.140526</v>
       </c>
-      <c r="G5" s="63" t="n">
+      <c r="G5" s="29" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H5" s="58" t="inlineStr">
+      <c r="H5" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5009,19 +3757,19 @@
       <c r="C6" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D6" s="68" t="n">
+      <c r="D6" s="34" t="n">
         <v>0.7210530000000001</v>
       </c>
-      <c r="E6" s="68" t="n">
+      <c r="E6" s="34" t="n">
         <v>0.111579</v>
       </c>
-      <c r="F6" s="68" t="n">
+      <c r="F6" s="34" t="n">
         <v>0.167368</v>
       </c>
-      <c r="G6" s="63" t="n">
+      <c r="G6" s="29" t="n">
         <v>0.0006242415932771846</v>
       </c>
-      <c r="H6" s="58" t="inlineStr">
+      <c r="H6" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5041,19 +3789,19 @@
       <c r="C7" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D7" s="68" t="n">
+      <c r="D7" s="34" t="n">
         <v>0.676316</v>
       </c>
-      <c r="E7" s="68" t="n">
+      <c r="E7" s="34" t="n">
         <v>0.129474</v>
       </c>
-      <c r="F7" s="68" t="n">
+      <c r="F7" s="34" t="n">
         <v>0.194211</v>
       </c>
-      <c r="G7" s="63" t="n">
+      <c r="G7" s="29" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H7" s="58" t="inlineStr">
+      <c r="H7" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5073,19 +3821,19 @@
       <c r="C8" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D8" s="68" t="n">
+      <c r="D8" s="34" t="n">
         <v>0.631579</v>
       </c>
-      <c r="E8" s="68" t="n">
+      <c r="E8" s="34" t="n">
         <v>0.147368</v>
       </c>
-      <c r="F8" s="68" t="n">
+      <c r="F8" s="34" t="n">
         <v>0.221053</v>
       </c>
-      <c r="G8" s="63" t="n">
+      <c r="G8" s="29" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H8" s="58" t="inlineStr">
+      <c r="H8" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5105,19 +3853,19 @@
       <c r="C9" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D9" s="68" t="n">
+      <c r="D9" s="34" t="n">
         <v>0.586842</v>
       </c>
-      <c r="E9" s="68" t="n">
+      <c r="E9" s="34" t="n">
         <v>0.165263</v>
       </c>
-      <c r="F9" s="68" t="n">
+      <c r="F9" s="34" t="n">
         <v>0.247895</v>
       </c>
-      <c r="G9" s="63" t="n">
+      <c r="G9" s="29" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H9" s="58" t="inlineStr">
+      <c r="H9" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5137,19 +3885,19 @@
       <c r="C10" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D10" s="68" t="n">
+      <c r="D10" s="34" t="n">
         <v>0.5421049999999999</v>
       </c>
-      <c r="E10" s="68" t="n">
+      <c r="E10" s="34" t="n">
         <v>0.183158</v>
       </c>
-      <c r="F10" s="68" t="n">
+      <c r="F10" s="34" t="n">
         <v>0.274737</v>
       </c>
-      <c r="G10" s="63" t="n">
+      <c r="G10" s="29" t="n">
         <v>0.0006242415932771825</v>
       </c>
-      <c r="H10" s="58" t="inlineStr">
+      <c r="H10" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5169,19 +3917,19 @@
       <c r="C11" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D11" s="68" t="n">
+      <c r="D11" s="34" t="n">
         <v>0.497368</v>
       </c>
-      <c r="E11" s="68" t="n">
+      <c r="E11" s="34" t="n">
         <v>0.201053</v>
       </c>
-      <c r="F11" s="68" t="n">
+      <c r="F11" s="34" t="n">
         <v>0.301579</v>
       </c>
-      <c r="G11" s="63" t="n">
+      <c r="G11" s="29" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H11" s="58" t="inlineStr">
+      <c r="H11" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5201,19 +3949,19 @@
       <c r="C12" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D12" s="68" t="n">
+      <c r="D12" s="34" t="n">
         <v>0.452632</v>
       </c>
-      <c r="E12" s="68" t="n">
+      <c r="E12" s="34" t="n">
         <v>0.218947</v>
       </c>
-      <c r="F12" s="68" t="n">
+      <c r="F12" s="34" t="n">
         <v>0.328421</v>
       </c>
-      <c r="G12" s="63" t="n">
+      <c r="G12" s="29" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H12" s="58" t="inlineStr">
+      <c r="H12" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5233,19 +3981,19 @@
       <c r="C13" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D13" s="68" t="n">
+      <c r="D13" s="34" t="n">
         <v>0.407895</v>
       </c>
-      <c r="E13" s="68" t="n">
+      <c r="E13" s="34" t="n">
         <v>0.236842</v>
       </c>
-      <c r="F13" s="68" t="n">
+      <c r="F13" s="34" t="n">
         <v>0.355263</v>
       </c>
-      <c r="G13" s="63" t="n">
+      <c r="G13" s="29" t="n">
         <v>0.000624241593277183</v>
       </c>
-      <c r="H13" s="58" t="inlineStr">
+      <c r="H13" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5265,19 +4013,19 @@
       <c r="C14" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D14" s="68" t="n">
+      <c r="D14" s="34" t="n">
         <v>0.363158</v>
       </c>
-      <c r="E14" s="68" t="n">
+      <c r="E14" s="34" t="n">
         <v>0.254737</v>
       </c>
-      <c r="F14" s="68" t="n">
+      <c r="F14" s="34" t="n">
         <v>0.382105</v>
       </c>
-      <c r="G14" s="63" t="n">
+      <c r="G14" s="29" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H14" s="58" t="inlineStr">
+      <c r="H14" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5297,19 +4045,19 @@
       <c r="C15" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D15" s="68" t="n">
+      <c r="D15" s="34" t="n">
         <v>0.318421</v>
       </c>
-      <c r="E15" s="68" t="n">
+      <c r="E15" s="34" t="n">
         <v>0.272632</v>
       </c>
-      <c r="F15" s="68" t="n">
+      <c r="F15" s="34" t="n">
         <v>0.408947</v>
       </c>
-      <c r="G15" s="63" t="n">
+      <c r="G15" s="29" t="n">
         <v>0.0006242415932771846</v>
       </c>
-      <c r="H15" s="58" t="inlineStr">
+      <c r="H15" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5329,19 +4077,19 @@
       <c r="C16" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D16" s="68" t="n">
+      <c r="D16" s="34" t="n">
         <v>0.273684</v>
       </c>
-      <c r="E16" s="68" t="n">
+      <c r="E16" s="34" t="n">
         <v>0.290526</v>
       </c>
-      <c r="F16" s="68" t="n">
+      <c r="F16" s="34" t="n">
         <v>0.435789</v>
       </c>
-      <c r="G16" s="63" t="n">
+      <c r="G16" s="29" t="n">
         <v>0.000624241593277183</v>
       </c>
-      <c r="H16" s="58" t="inlineStr">
+      <c r="H16" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5361,19 +4109,19 @@
       <c r="C17" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D17" s="68" t="n">
+      <c r="D17" s="34" t="n">
         <v>0.228947</v>
       </c>
-      <c r="E17" s="68" t="n">
+      <c r="E17" s="34" t="n">
         <v>0.308421</v>
       </c>
-      <c r="F17" s="68" t="n">
+      <c r="F17" s="34" t="n">
         <v>0.462632</v>
       </c>
-      <c r="G17" s="63" t="n">
+      <c r="G17" s="29" t="n">
         <v>0.0006242415932771825</v>
       </c>
-      <c r="H17" s="58" t="inlineStr">
+      <c r="H17" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5393,19 +4141,19 @@
       <c r="C18" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D18" s="68" t="n">
+      <c r="D18" s="34" t="n">
         <v>0.184211</v>
       </c>
-      <c r="E18" s="68" t="n">
+      <c r="E18" s="34" t="n">
         <v>0.326316</v>
       </c>
-      <c r="F18" s="68" t="n">
+      <c r="F18" s="34" t="n">
         <v>0.489474</v>
       </c>
-      <c r="G18" s="63" t="n">
+      <c r="G18" s="29" t="n">
         <v>0.0006242415932771825</v>
       </c>
-      <c r="H18" s="58" t="inlineStr">
+      <c r="H18" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5425,19 +4173,19 @@
       <c r="C19" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D19" s="68" t="n">
+      <c r="D19" s="34" t="n">
         <v>0.139474</v>
       </c>
-      <c r="E19" s="68" t="n">
+      <c r="E19" s="34" t="n">
         <v>0.344211</v>
       </c>
-      <c r="F19" s="68" t="n">
+      <c r="F19" s="34" t="n">
         <v>0.516316</v>
       </c>
-      <c r="G19" s="63" t="n">
+      <c r="G19" s="29" t="n">
         <v>0.000624241593277183</v>
       </c>
-      <c r="H19" s="58" t="inlineStr">
+      <c r="H19" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5457,19 +4205,19 @@
       <c r="C20" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D20" s="68" t="n">
+      <c r="D20" s="34" t="n">
         <v>0.094737</v>
       </c>
-      <c r="E20" s="68" t="n">
+      <c r="E20" s="34" t="n">
         <v>0.362105</v>
       </c>
-      <c r="F20" s="68" t="n">
+      <c r="F20" s="34" t="n">
         <v>0.543158</v>
       </c>
-      <c r="G20" s="63" t="n">
+      <c r="G20" s="29" t="n">
         <v>0.0006242415932771825</v>
       </c>
-      <c r="H20" s="58" t="inlineStr">
+      <c r="H20" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5489,19 +4237,19 @@
       <c r="C21" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D21" s="68" t="n">
+      <c r="D21" s="34" t="n">
         <v>0.05</v>
       </c>
-      <c r="E21" s="68" t="n">
+      <c r="E21" s="34" t="n">
         <v>0.38</v>
       </c>
-      <c r="F21" s="68" t="n">
+      <c r="F21" s="34" t="n">
         <v>0.57</v>
       </c>
-      <c r="G21" s="63" t="n">
+      <c r="G21" s="29" t="n">
         <v>0.0006242415932771841</v>
       </c>
-      <c r="H21" s="58" t="inlineStr">
+      <c r="H21" s="24" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -5521,19 +4269,19 @@
       <c r="C22" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D22" s="69" t="n">
+      <c r="D22" s="35" t="n">
         <v>0.9</v>
       </c>
-      <c r="E22" s="69" t="n">
+      <c r="E22" s="35" t="n">
         <v>0.05</v>
       </c>
-      <c r="F22" s="69" t="n">
+      <c r="F22" s="35" t="n">
         <v>0.05</v>
       </c>
-      <c r="G22" s="65" t="n">
+      <c r="G22" s="31" t="n">
         <v>0.0006234486982757811</v>
       </c>
-      <c r="H22" s="59" t="inlineStr">
+      <c r="H22" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -5553,19 +4301,19 @@
       <c r="C23" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D23" s="69" t="n">
+      <c r="D23" s="35" t="n">
         <v>0.855263</v>
       </c>
-      <c r="E23" s="69" t="n">
+      <c r="E23" s="35" t="n">
         <v>0.072368</v>
       </c>
-      <c r="F23" s="69" t="n">
+      <c r="F23" s="35" t="n">
         <v>0.072368</v>
       </c>
-      <c r="G23" s="65" t="n">
+      <c r="G23" s="31" t="n">
         <v>0.0006234240698697985</v>
       </c>
-      <c r="H23" s="59" t="inlineStr">
+      <c r="H23" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -5585,19 +4333,19 @@
       <c r="C24" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D24" s="69" t="n">
+      <c r="D24" s="35" t="n">
         <v>0.810526</v>
       </c>
-      <c r="E24" s="69" t="n">
+      <c r="E24" s="35" t="n">
         <v>0.094737</v>
       </c>
-      <c r="F24" s="69" t="n">
+      <c r="F24" s="35" t="n">
         <v>0.094737</v>
       </c>
-      <c r="G24" s="65" t="n">
+      <c r="G24" s="31" t="n">
         <v>0.000623390113702764</v>
       </c>
-      <c r="H24" s="59" t="inlineStr">
+      <c r="H24" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -5617,19 +4365,19 @@
       <c r="C25" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D25" s="69" t="n">
+      <c r="D25" s="35" t="n">
         <v>0.7657890000000001</v>
       </c>
-      <c r="E25" s="69" t="n">
+      <c r="E25" s="35" t="n">
         <v>0.117105</v>
       </c>
-      <c r="F25" s="69" t="n">
+      <c r="F25" s="35" t="n">
         <v>0.117105</v>
       </c>
-      <c r="G25" s="65" t="n">
+      <c r="G25" s="31" t="n">
         <v>0.0006233465051459715</v>
       </c>
-      <c r="H25" s="59" t="inlineStr">
+      <c r="H25" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -5649,19 +4397,19 @@
       <c r="C26" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D26" s="69" t="n">
+      <c r="D26" s="35" t="n">
         <v>0.7210530000000001</v>
       </c>
-      <c r="E26" s="69" t="n">
+      <c r="E26" s="35" t="n">
         <v>0.139474</v>
       </c>
-      <c r="F26" s="69" t="n">
+      <c r="F26" s="35" t="n">
         <v>0.139474</v>
       </c>
-      <c r="G26" s="65" t="n">
+      <c r="G26" s="31" t="n">
         <v>0.0006232927260585453</v>
       </c>
-      <c r="H26" s="59" t="inlineStr">
+      <c r="H26" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -5681,19 +4429,19 @@
       <c r="C27" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D27" s="69" t="n">
+      <c r="D27" s="35" t="n">
         <v>0.676316</v>
       </c>
-      <c r="E27" s="69" t="n">
+      <c r="E27" s="35" t="n">
         <v>0.161842</v>
       </c>
-      <c r="F27" s="69" t="n">
+      <c r="F27" s="35" t="n">
         <v>0.161842</v>
       </c>
-      <c r="G27" s="65" t="n">
+      <c r="G27" s="31" t="n">
         <v>0.0006232279909242769</v>
       </c>
-      <c r="H27" s="59" t="inlineStr">
+      <c r="H27" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -5713,19 +4461,19 @@
       <c r="C28" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D28" s="69" t="n">
+      <c r="D28" s="35" t="n">
         <v>0.631579</v>
       </c>
-      <c r="E28" s="69" t="n">
+      <c r="E28" s="35" t="n">
         <v>0.184211</v>
       </c>
-      <c r="F28" s="69" t="n">
+      <c r="F28" s="35" t="n">
         <v>0.184211</v>
       </c>
-      <c r="G28" s="65" t="n">
+      <c r="G28" s="31" t="n">
         <v>0.0006231511590811589</v>
       </c>
-      <c r="H28" s="59" t="inlineStr">
+      <c r="H28" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -5745,19 +4493,19 @@
       <c r="C29" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D29" s="69" t="n">
+      <c r="D29" s="35" t="n">
         <v>0.586842</v>
       </c>
-      <c r="E29" s="69" t="n">
+      <c r="E29" s="35" t="n">
         <v>0.206579</v>
       </c>
-      <c r="F29" s="69" t="n">
+      <c r="F29" s="35" t="n">
         <v>0.206579</v>
       </c>
-      <c r="G29" s="65" t="n">
+      <c r="G29" s="31" t="n">
         <v>0.0006230606192890642</v>
       </c>
-      <c r="H29" s="59" t="inlineStr">
+      <c r="H29" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -5777,19 +4525,19 @@
       <c r="C30" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D30" s="69" t="n">
+      <c r="D30" s="35" t="n">
         <v>0.5421049999999999</v>
       </c>
-      <c r="E30" s="69" t="n">
+      <c r="E30" s="35" t="n">
         <v>0.228947</v>
       </c>
-      <c r="F30" s="69" t="n">
+      <c r="F30" s="35" t="n">
         <v>0.228947</v>
       </c>
-      <c r="G30" s="65" t="n">
+      <c r="G30" s="31" t="n">
         <v>0.0006229541258469519</v>
       </c>
-      <c r="H30" s="59" t="inlineStr">
+      <c r="H30" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -5809,19 +4557,19 @@
       <c r="C31" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D31" s="69" t="n">
+      <c r="D31" s="35" t="n">
         <v>0.497368</v>
       </c>
-      <c r="E31" s="69" t="n">
+      <c r="E31" s="35" t="n">
         <v>0.251316</v>
       </c>
-      <c r="F31" s="69" t="n">
+      <c r="F31" s="35" t="n">
         <v>0.251316</v>
       </c>
-      <c r="G31" s="65" t="n">
+      <c r="G31" s="31" t="n">
         <v>0.0006228285531386366</v>
       </c>
-      <c r="H31" s="59" t="inlineStr">
+      <c r="H31" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -5841,19 +4589,19 @@
       <c r="C32" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D32" s="69" t="n">
+      <c r="D32" s="35" t="n">
         <v>0.452632</v>
       </c>
-      <c r="E32" s="69" t="n">
+      <c r="E32" s="35" t="n">
         <v>0.273684</v>
       </c>
-      <c r="F32" s="69" t="n">
+      <c r="F32" s="35" t="n">
         <v>0.273684</v>
       </c>
-      <c r="G32" s="65" t="n">
+      <c r="G32" s="31" t="n">
         <v>0.0006226795122556773</v>
       </c>
-      <c r="H32" s="59" t="inlineStr">
+      <c r="H32" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -5873,19 +4621,19 @@
       <c r="C33" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D33" s="69" t="n">
+      <c r="D33" s="35" t="n">
         <v>0.407895</v>
       </c>
-      <c r="E33" s="69" t="n">
+      <c r="E33" s="35" t="n">
         <v>0.296053</v>
       </c>
-      <c r="F33" s="69" t="n">
+      <c r="F33" s="35" t="n">
         <v>0.296053</v>
       </c>
-      <c r="G33" s="65" t="n">
+      <c r="G33" s="31" t="n">
         <v>0.000622500727556083</v>
       </c>
-      <c r="H33" s="59" t="inlineStr">
+      <c r="H33" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -5905,19 +4653,19 @@
       <c r="C34" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D34" s="69" t="n">
+      <c r="D34" s="35" t="n">
         <v>0.363158</v>
       </c>
-      <c r="E34" s="69" t="n">
+      <c r="E34" s="35" t="n">
         <v>0.318421</v>
       </c>
-      <c r="F34" s="69" t="n">
+      <c r="F34" s="35" t="n">
         <v>0.318421</v>
       </c>
-      <c r="G34" s="65" t="n">
+      <c r="G34" s="31" t="n">
         <v>0.0006222829760272391</v>
       </c>
-      <c r="H34" s="59" t="inlineStr">
+      <c r="H34" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -5937,19 +4685,19 @@
       <c r="C35" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D35" s="69" t="n">
+      <c r="D35" s="35" t="n">
         <v>0.318421</v>
       </c>
-      <c r="E35" s="69" t="n">
+      <c r="E35" s="35" t="n">
         <v>0.340789</v>
       </c>
-      <c r="F35" s="69" t="n">
+      <c r="F35" s="35" t="n">
         <v>0.340789</v>
       </c>
-      <c r="G35" s="65" t="n">
+      <c r="G35" s="31" t="n">
         <v>0.0006220121819606671</v>
       </c>
-      <c r="H35" s="59" t="inlineStr">
+      <c r="H35" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -5969,19 +4717,19 @@
       <c r="C36" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D36" s="69" t="n">
+      <c r="D36" s="35" t="n">
         <v>0.273684</v>
       </c>
-      <c r="E36" s="69" t="n">
+      <c r="E36" s="35" t="n">
         <v>0.363158</v>
       </c>
-      <c r="F36" s="69" t="n">
+      <c r="F36" s="35" t="n">
         <v>0.363158</v>
       </c>
-      <c r="G36" s="65" t="n">
+      <c r="G36" s="31" t="n">
         <v>0.0006216657532754782</v>
       </c>
-      <c r="H36" s="59" t="inlineStr">
+      <c r="H36" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -6001,19 +4749,19 @@
       <c r="C37" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D37" s="69" t="n">
+      <c r="D37" s="35" t="n">
         <v>0.228947</v>
       </c>
-      <c r="E37" s="69" t="n">
+      <c r="E37" s="35" t="n">
         <v>0.385526</v>
       </c>
-      <c r="F37" s="69" t="n">
+      <c r="F37" s="35" t="n">
         <v>0.385526</v>
       </c>
-      <c r="G37" s="65" t="n">
+      <c r="G37" s="31" t="n">
         <v>0.0006212048918444731</v>
       </c>
-      <c r="H37" s="59" t="inlineStr">
+      <c r="H37" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -6033,19 +4781,19 @@
       <c r="C38" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D38" s="69" t="n">
+      <c r="D38" s="35" t="n">
         <v>0.184211</v>
       </c>
-      <c r="E38" s="69" t="n">
+      <c r="E38" s="35" t="n">
         <v>0.407895</v>
       </c>
-      <c r="F38" s="69" t="n">
+      <c r="F38" s="35" t="n">
         <v>0.407895</v>
       </c>
-      <c r="G38" s="65" t="n">
+      <c r="G38" s="31" t="n">
         <v>0.0006205564490138872</v>
       </c>
-      <c r="H38" s="59" t="inlineStr">
+      <c r="H38" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -6065,19 +4813,19 @@
       <c r="C39" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D39" s="69" t="n">
+      <c r="D39" s="35" t="n">
         <v>0.139474</v>
       </c>
-      <c r="E39" s="69" t="n">
+      <c r="E39" s="35" t="n">
         <v>0.430263</v>
       </c>
-      <c r="F39" s="69" t="n">
+      <c r="F39" s="35" t="n">
         <v>0.430263</v>
       </c>
-      <c r="G39" s="65" t="n">
+      <c r="G39" s="31" t="n">
         <v>0.0006195624103164132</v>
       </c>
-      <c r="H39" s="59" t="inlineStr">
+      <c r="H39" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -6097,19 +4845,19 @@
       <c r="C40" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D40" s="69" t="n">
+      <c r="D40" s="35" t="n">
         <v>0.094737</v>
       </c>
-      <c r="E40" s="69" t="n">
+      <c r="E40" s="35" t="n">
         <v>0.452632</v>
       </c>
-      <c r="F40" s="69" t="n">
+      <c r="F40" s="35" t="n">
         <v>0.452632</v>
       </c>
-      <c r="G40" s="65" t="n">
+      <c r="G40" s="31" t="n">
         <v>0.0006177982099275926</v>
       </c>
-      <c r="H40" s="59" t="inlineStr">
+      <c r="H40" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -6129,19 +4877,19 @@
       <c r="C41" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D41" s="69" t="n">
+      <c r="D41" s="35" t="n">
         <v>0.05</v>
       </c>
-      <c r="E41" s="69" t="n">
+      <c r="E41" s="35" t="n">
         <v>0.475</v>
       </c>
-      <c r="F41" s="69" t="n">
+      <c r="F41" s="35" t="n">
         <v>0.475</v>
       </c>
-      <c r="G41" s="65" t="n">
+      <c r="G41" s="31" t="n">
         <v>0.0006135214100988033</v>
       </c>
-      <c r="H41" s="59" t="inlineStr">
+      <c r="H41" s="25" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -6161,19 +4909,19 @@
       <c r="C42" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D42" s="68" t="n">
+      <c r="D42" s="34" t="n">
         <v>0.9</v>
       </c>
-      <c r="E42" s="68" t="n">
+      <c r="E42" s="34" t="n">
         <v>0.05</v>
       </c>
-      <c r="F42" s="68" t="n">
+      <c r="F42" s="34" t="n">
         <v>0.05</v>
       </c>
-      <c r="G42" s="63" t="n">
+      <c r="G42" s="29" t="n">
         <v>0.0006192201975493238</v>
       </c>
-      <c r="H42" s="58" t="inlineStr">
+      <c r="H42" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6193,19 +4941,19 @@
       <c r="C43" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D43" s="68" t="n">
+      <c r="D43" s="34" t="n">
         <v>0.855263</v>
       </c>
-      <c r="E43" s="68" t="n">
+      <c r="E43" s="34" t="n">
         <v>0.072368</v>
       </c>
-      <c r="F43" s="68" t="n">
+      <c r="F43" s="34" t="n">
         <v>0.072368</v>
       </c>
-      <c r="G43" s="63" t="n">
+      <c r="G43" s="29" t="n">
         <v>0.0006178389962257873</v>
       </c>
-      <c r="H43" s="58" t="inlineStr">
+      <c r="H43" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6225,19 +4973,19 @@
       <c r="C44" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D44" s="68" t="n">
+      <c r="D44" s="34" t="n">
         <v>0.810526</v>
       </c>
-      <c r="E44" s="68" t="n">
+      <c r="E44" s="34" t="n">
         <v>0.094737</v>
       </c>
-      <c r="F44" s="68" t="n">
+      <c r="F44" s="34" t="n">
         <v>0.094737</v>
       </c>
-      <c r="G44" s="63" t="n">
+      <c r="G44" s="29" t="n">
         <v>0.0006164156519341792</v>
       </c>
-      <c r="H44" s="58" t="inlineStr">
+      <c r="H44" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6257,19 +5005,19 @@
       <c r="C45" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D45" s="68" t="n">
+      <c r="D45" s="34" t="n">
         <v>0.7657890000000001</v>
       </c>
-      <c r="E45" s="68" t="n">
+      <c r="E45" s="34" t="n">
         <v>0.117105</v>
       </c>
-      <c r="F45" s="68" t="n">
+      <c r="F45" s="34" t="n">
         <v>0.117105</v>
       </c>
-      <c r="G45" s="63" t="n">
+      <c r="G45" s="29" t="n">
         <v>0.0006149434371808388</v>
       </c>
-      <c r="H45" s="58" t="inlineStr">
+      <c r="H45" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6289,19 +5037,19 @@
       <c r="C46" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D46" s="68" t="n">
+      <c r="D46" s="34" t="n">
         <v>0.7210530000000001</v>
       </c>
-      <c r="E46" s="68" t="n">
+      <c r="E46" s="34" t="n">
         <v>0.139474</v>
       </c>
-      <c r="F46" s="68" t="n">
+      <c r="F46" s="34" t="n">
         <v>0.139474</v>
       </c>
-      <c r="G46" s="63" t="n">
+      <c r="G46" s="29" t="n">
         <v>0.0006134086362605692</v>
       </c>
-      <c r="H46" s="58" t="inlineStr">
+      <c r="H46" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6321,19 +5069,19 @@
       <c r="C47" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D47" s="68" t="n">
+      <c r="D47" s="34" t="n">
         <v>0.676316</v>
       </c>
-      <c r="E47" s="68" t="n">
+      <c r="E47" s="34" t="n">
         <v>0.161842</v>
       </c>
-      <c r="F47" s="68" t="n">
+      <c r="F47" s="34" t="n">
         <v>0.161842</v>
       </c>
-      <c r="G47" s="63" t="n">
+      <c r="G47" s="29" t="n">
         <v>0.000611794507683605</v>
       </c>
-      <c r="H47" s="58" t="inlineStr">
+      <c r="H47" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6353,19 +5101,19 @@
       <c r="C48" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D48" s="68" t="n">
+      <c r="D48" s="34" t="n">
         <v>0.631579</v>
       </c>
-      <c r="E48" s="68" t="n">
+      <c r="E48" s="34" t="n">
         <v>0.184211</v>
       </c>
-      <c r="F48" s="68" t="n">
+      <c r="F48" s="34" t="n">
         <v>0.184211</v>
       </c>
-      <c r="G48" s="63" t="n">
+      <c r="G48" s="29" t="n">
         <v>0.0006100815926117644</v>
       </c>
-      <c r="H48" s="58" t="inlineStr">
+      <c r="H48" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6385,19 +5133,19 @@
       <c r="C49" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D49" s="68" t="n">
+      <c r="D49" s="34" t="n">
         <v>0.586842</v>
       </c>
-      <c r="E49" s="68" t="n">
+      <c r="E49" s="34" t="n">
         <v>0.206579</v>
       </c>
-      <c r="F49" s="68" t="n">
+      <c r="F49" s="34" t="n">
         <v>0.206579</v>
       </c>
-      <c r="G49" s="63" t="n">
+      <c r="G49" s="29" t="n">
         <v>0.0006082469669095847</v>
       </c>
-      <c r="H49" s="58" t="inlineStr">
+      <c r="H49" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -6417,19 +5165,19 @@
       <c r="C50" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D50" s="68" t="n">
+      <c r="D50" s="34" t="n">
         <v>0.5421049999999999</v>
       </c>
-      <c r="E50" s="68" t="n">
+      <c r="E50" s="34" t="n">
         <v>0.228947</v>
       </c>
-      <c r="F50" s="68" t="n">
+      <c r="F50" s="34" t="n">
         <v>0.228947</v>
       </c>
-      <c r="G50" s="63" t="n">
+      <c r="G50" s="29" t="n">
         <v>0.0006062629201632612</v>
       </c>
-      <c r="H50" s="58" t="inlineStr">
+      <c r="H50" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -6449,19 +5197,19 @@
       <c r="C51" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D51" s="68" t="n">
+      <c r="D51" s="34" t="n">
         <v>0.497368</v>
       </c>
-      <c r="E51" s="68" t="n">
+      <c r="E51" s="34" t="n">
         <v>0.251316</v>
       </c>
-      <c r="F51" s="68" t="n">
+      <c r="F51" s="34" t="n">
         <v>0.251316</v>
       </c>
-      <c r="G51" s="63" t="n">
+      <c r="G51" s="29" t="n">
         <v>0.0006040950268609877</v>
       </c>
-      <c r="H51" s="58" t="inlineStr">
+      <c r="H51" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -6481,19 +5229,19 @@
       <c r="C52" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D52" s="68" t="n">
+      <c r="D52" s="34" t="n">
         <v>0.452632</v>
       </c>
-      <c r="E52" s="68" t="n">
+      <c r="E52" s="34" t="n">
         <v>0.273684</v>
       </c>
-      <c r="F52" s="68" t="n">
+      <c r="F52" s="34" t="n">
         <v>0.273684</v>
       </c>
-      <c r="G52" s="63" t="n">
+      <c r="G52" s="29" t="n">
         <v>0.00060169933822934</v>
       </c>
-      <c r="H52" s="58" t="inlineStr">
+      <c r="H52" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -6513,19 +5261,19 @@
       <c r="C53" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D53" s="68" t="n">
+      <c r="D53" s="34" t="n">
         <v>0.407895</v>
       </c>
-      <c r="E53" s="68" t="n">
+      <c r="E53" s="34" t="n">
         <v>0.296053</v>
       </c>
-      <c r="F53" s="68" t="n">
+      <c r="F53" s="34" t="n">
         <v>0.296053</v>
       </c>
-      <c r="G53" s="63" t="n">
+      <c r="G53" s="29" t="n">
         <v>0.0005990181736125742</v>
       </c>
-      <c r="H53" s="58" t="inlineStr">
+      <c r="H53" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -6545,19 +5293,19 @@
       <c r="C54" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D54" s="68" t="n">
+      <c r="D54" s="34" t="n">
         <v>0.363158</v>
       </c>
-      <c r="E54" s="68" t="n">
+      <c r="E54" s="34" t="n">
         <v>0.318421</v>
       </c>
-      <c r="F54" s="68" t="n">
+      <c r="F54" s="34" t="n">
         <v>0.318421</v>
       </c>
-      <c r="G54" s="63" t="n">
+      <c r="G54" s="29" t="n">
         <v>0.0005959735807338218</v>
       </c>
-      <c r="H54" s="58" t="inlineStr">
+      <c r="H54" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -6577,19 +5325,19 @@
       <c r="C55" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D55" s="68" t="n">
+      <c r="D55" s="34" t="n">
         <v>0.318421</v>
       </c>
-      <c r="E55" s="68" t="n">
+      <c r="E55" s="34" t="n">
         <v>0.340789</v>
       </c>
-      <c r="F55" s="68" t="n">
+      <c r="F55" s="34" t="n">
         <v>0.340789</v>
       </c>
-      <c r="G55" s="63" t="n">
+      <c r="G55" s="29" t="n">
         <v>0.0005924567681126914</v>
       </c>
-      <c r="H55" s="58" t="inlineStr">
+      <c r="H55" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -6609,19 +5357,19 @@
       <c r="C56" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D56" s="68" t="n">
+      <c r="D56" s="34" t="n">
         <v>0.273684</v>
       </c>
-      <c r="E56" s="68" t="n">
+      <c r="E56" s="34" t="n">
         <v>0.363158</v>
       </c>
-      <c r="F56" s="68" t="n">
+      <c r="F56" s="34" t="n">
         <v>0.363158</v>
       </c>
-      <c r="G56" s="63" t="n">
+      <c r="G56" s="29" t="n">
         <v>0.0005883103133506319</v>
       </c>
-      <c r="H56" s="58" t="inlineStr">
+      <c r="H56" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6641,19 +5389,19 @@
       <c r="C57" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D57" s="68" t="n">
+      <c r="D57" s="34" t="n">
         <v>0.228947</v>
       </c>
-      <c r="E57" s="68" t="n">
+      <c r="E57" s="34" t="n">
         <v>0.385526</v>
       </c>
-      <c r="F57" s="68" t="n">
+      <c r="F57" s="34" t="n">
         <v>0.385526</v>
       </c>
-      <c r="G57" s="63" t="n">
+      <c r="G57" s="29" t="n">
         <v>0.0005832970131890047</v>
       </c>
-      <c r="H57" s="58" t="inlineStr">
+      <c r="H57" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6673,19 +5421,19 @@
       <c r="C58" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D58" s="68" t="n">
+      <c r="D58" s="34" t="n">
         <v>0.184211</v>
       </c>
-      <c r="E58" s="68" t="n">
+      <c r="E58" s="34" t="n">
         <v>0.407895</v>
       </c>
-      <c r="F58" s="68" t="n">
+      <c r="F58" s="34" t="n">
         <v>0.407895</v>
       </c>
-      <c r="G58" s="63" t="n">
+      <c r="G58" s="29" t="n">
         <v>0.0005770442311225281</v>
       </c>
-      <c r="H58" s="58" t="inlineStr">
+      <c r="H58" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6705,19 +5453,19 @@
       <c r="C59" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D59" s="68" t="n">
+      <c r="D59" s="34" t="n">
         <v>0.139474</v>
       </c>
-      <c r="E59" s="68" t="n">
+      <c r="E59" s="34" t="n">
         <v>0.430263</v>
       </c>
-      <c r="F59" s="68" t="n">
+      <c r="F59" s="34" t="n">
         <v>0.430263</v>
       </c>
-      <c r="G59" s="63" t="n">
+      <c r="G59" s="29" t="n">
         <v>0.0005689524243180519</v>
       </c>
-      <c r="H59" s="58" t="inlineStr">
+      <c r="H59" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6737,19 +5485,19 @@
       <c r="C60" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D60" s="68" t="n">
+      <c r="D60" s="34" t="n">
         <v>0.094737</v>
       </c>
-      <c r="E60" s="68" t="n">
+      <c r="E60" s="34" t="n">
         <v>0.452632</v>
       </c>
-      <c r="F60" s="68" t="n">
+      <c r="F60" s="34" t="n">
         <v>0.452632</v>
       </c>
-      <c r="G60" s="63" t="n">
+      <c r="G60" s="29" t="n">
         <v>0.0005581573496582796</v>
       </c>
-      <c r="H60" s="58" t="inlineStr">
+      <c r="H60" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -6769,19 +5517,19 @@
       <c r="C61" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D61" s="68" t="n">
+      <c r="D61" s="34" t="n">
         <v>0.05</v>
       </c>
-      <c r="E61" s="68" t="n">
+      <c r="E61" s="34" t="n">
         <v>0.475</v>
       </c>
-      <c r="F61" s="68" t="n">
+      <c r="F61" s="34" t="n">
         <v>0.475</v>
       </c>
-      <c r="G61" s="63" t="n">
+      <c r="G61" s="29" t="n">
         <v>0.0005441813023263959</v>
       </c>
-      <c r="H61" s="58" t="inlineStr">
+      <c r="H61" s="24" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -6801,19 +5549,19 @@
       <c r="C62" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D62" s="69" t="n">
+      <c r="D62" s="35" t="n">
         <v>0.9</v>
       </c>
-      <c r="E62" s="69" t="n">
+      <c r="E62" s="35" t="n">
         <v>0.028571</v>
       </c>
-      <c r="F62" s="69" t="n">
+      <c r="F62" s="35" t="n">
         <v>0.07142900000000001</v>
       </c>
-      <c r="G62" s="65" t="n">
+      <c r="G62" s="31" t="n">
         <v>0.0006089752639324707</v>
       </c>
-      <c r="H62" s="59" t="inlineStr">
+      <c r="H62" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2; V3O5_HT#1</t>
         </is>
@@ -6833,19 +5581,19 @@
       <c r="C63" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D63" s="69" t="n">
+      <c r="D63" s="35" t="n">
         <v>0.855263</v>
       </c>
-      <c r="E63" s="69" t="n">
+      <c r="E63" s="35" t="n">
         <v>0.041353</v>
       </c>
-      <c r="F63" s="69" t="n">
+      <c r="F63" s="35" t="n">
         <v>0.103383</v>
       </c>
-      <c r="G63" s="65" t="n">
+      <c r="G63" s="31" t="n">
         <v>0.0006089752639324707</v>
       </c>
-      <c r="H63" s="59" t="inlineStr">
+      <c r="H63" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2; V3O5_HT#1</t>
         </is>
@@ -6865,19 +5613,19 @@
       <c r="C64" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D64" s="69" t="n">
+      <c r="D64" s="35" t="n">
         <v>0.810526</v>
       </c>
-      <c r="E64" s="69" t="n">
+      <c r="E64" s="35" t="n">
         <v>0.054135</v>
       </c>
-      <c r="F64" s="69" t="n">
+      <c r="F64" s="35" t="n">
         <v>0.135338</v>
       </c>
-      <c r="G64" s="65" t="n">
+      <c r="G64" s="31" t="n">
         <v>0.000608975263932468</v>
       </c>
-      <c r="H64" s="59" t="inlineStr">
+      <c r="H64" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2; V3O5_HT#1</t>
         </is>
@@ -6897,19 +5645,19 @@
       <c r="C65" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D65" s="69" t="n">
+      <c r="D65" s="35" t="n">
         <v>0.7657890000000001</v>
       </c>
-      <c r="E65" s="69" t="n">
+      <c r="E65" s="35" t="n">
         <v>0.066917</v>
       </c>
-      <c r="F65" s="69" t="n">
+      <c r="F65" s="35" t="n">
         <v>0.167293</v>
       </c>
-      <c r="G65" s="65" t="n">
+      <c r="G65" s="31" t="n">
         <v>0.0006089752639324696</v>
       </c>
-      <c r="H65" s="59" t="inlineStr">
+      <c r="H65" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2; V3O5_HT#1</t>
         </is>
@@ -6929,19 +5677,19 @@
       <c r="C66" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D66" s="69" t="n">
+      <c r="D66" s="35" t="n">
         <v>0.7210530000000001</v>
       </c>
-      <c r="E66" s="69" t="n">
+      <c r="E66" s="35" t="n">
         <v>0.07969900000000001</v>
       </c>
-      <c r="F66" s="69" t="n">
+      <c r="F66" s="35" t="n">
         <v>0.199248</v>
       </c>
-      <c r="G66" s="65" t="n">
+      <c r="G66" s="31" t="n">
         <v>0.0006086989931423054</v>
       </c>
-      <c r="H66" s="59" t="inlineStr">
+      <c r="H66" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6961,19 +5709,19 @@
       <c r="C67" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D67" s="69" t="n">
+      <c r="D67" s="35" t="n">
         <v>0.676316</v>
       </c>
-      <c r="E67" s="69" t="n">
+      <c r="E67" s="35" t="n">
         <v>0.09248099999999999</v>
       </c>
-      <c r="F67" s="69" t="n">
+      <c r="F67" s="35" t="n">
         <v>0.231203</v>
       </c>
-      <c r="G67" s="65" t="n">
+      <c r="G67" s="31" t="n">
         <v>0.0006075806595837329</v>
       </c>
-      <c r="H67" s="59" t="inlineStr">
+      <c r="H67" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6993,19 +5741,19 @@
       <c r="C68" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D68" s="69" t="n">
+      <c r="D68" s="35" t="n">
         <v>0.631579</v>
       </c>
-      <c r="E68" s="69" t="n">
+      <c r="E68" s="35" t="n">
         <v>0.105263</v>
       </c>
-      <c r="F68" s="69" t="n">
+      <c r="F68" s="35" t="n">
         <v>0.263158</v>
       </c>
-      <c r="G68" s="65" t="n">
+      <c r="G68" s="31" t="n">
         <v>0.0006066170076563114</v>
       </c>
-      <c r="H68" s="59" t="inlineStr">
+      <c r="H68" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -7025,19 +5773,19 @@
       <c r="C69" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D69" s="69" t="n">
+      <c r="D69" s="35" t="n">
         <v>0.586842</v>
       </c>
-      <c r="E69" s="69" t="n">
+      <c r="E69" s="35" t="n">
         <v>0.118045</v>
       </c>
-      <c r="F69" s="69" t="n">
+      <c r="F69" s="35" t="n">
         <v>0.295113</v>
       </c>
-      <c r="G69" s="65" t="n">
+      <c r="G69" s="31" t="n">
         <v>0.0006057789423692359</v>
       </c>
-      <c r="H69" s="59" t="inlineStr">
+      <c r="H69" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -7057,19 +5805,19 @@
       <c r="C70" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D70" s="69" t="n">
+      <c r="D70" s="35" t="n">
         <v>0.5421049999999999</v>
       </c>
-      <c r="E70" s="69" t="n">
+      <c r="E70" s="35" t="n">
         <v>0.130827</v>
       </c>
-      <c r="F70" s="69" t="n">
+      <c r="F70" s="35" t="n">
         <v>0.327068</v>
       </c>
-      <c r="G70" s="65" t="n">
+      <c r="G70" s="31" t="n">
         <v>0.0006050440821113034</v>
       </c>
-      <c r="H70" s="59" t="inlineStr">
+      <c r="H70" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -7089,19 +5837,19 @@
       <c r="C71" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D71" s="69" t="n">
+      <c r="D71" s="35" t="n">
         <v>0.497368</v>
       </c>
-      <c r="E71" s="69" t="n">
+      <c r="E71" s="35" t="n">
         <v>0.143609</v>
       </c>
-      <c r="F71" s="69" t="n">
+      <c r="F71" s="35" t="n">
         <v>0.359023</v>
       </c>
-      <c r="G71" s="65" t="n">
+      <c r="G71" s="31" t="n">
         <v>0.0006043949529175177</v>
       </c>
-      <c r="H71" s="59" t="inlineStr">
+      <c r="H71" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -7121,19 +5869,19 @@
       <c r="C72" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D72" s="69" t="n">
+      <c r="D72" s="35" t="n">
         <v>0.452632</v>
       </c>
-      <c r="E72" s="69" t="n">
+      <c r="E72" s="35" t="n">
         <v>0.156391</v>
       </c>
-      <c r="F72" s="69" t="n">
+      <c r="F72" s="35" t="n">
         <v>0.390977</v>
       </c>
-      <c r="G72" s="65" t="n">
+      <c r="G72" s="31" t="n">
         <v>0.0006038177336590362</v>
       </c>
-      <c r="H72" s="59" t="inlineStr">
+      <c r="H72" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -7153,19 +5901,19 @@
       <c r="C73" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D73" s="69" t="n">
+      <c r="D73" s="35" t="n">
         <v>0.407895</v>
       </c>
-      <c r="E73" s="69" t="n">
+      <c r="E73" s="35" t="n">
         <v>0.169173</v>
       </c>
-      <c r="F73" s="69" t="n">
+      <c r="F73" s="35" t="n">
         <v>0.422932</v>
       </c>
-      <c r="G73" s="65" t="n">
+      <c r="G73" s="31" t="n">
         <v>0.0006033013642003349</v>
       </c>
-      <c r="H73" s="59" t="inlineStr">
+      <c r="H73" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -7185,19 +5933,19 @@
       <c r="C74" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D74" s="69" t="n">
+      <c r="D74" s="35" t="n">
         <v>0.363158</v>
       </c>
-      <c r="E74" s="69" t="n">
+      <c r="E74" s="35" t="n">
         <v>0.181955</v>
       </c>
-      <c r="F74" s="69" t="n">
+      <c r="F74" s="35" t="n">
         <v>0.454887</v>
       </c>
-      <c r="G74" s="65" t="n">
+      <c r="G74" s="31" t="n">
         <v>0.0006028368997837505</v>
       </c>
-      <c r="H74" s="59" t="inlineStr">
+      <c r="H74" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -7217,19 +5965,19 @@
       <c r="C75" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D75" s="69" t="n">
+      <c r="D75" s="35" t="n">
         <v>0.318421</v>
       </c>
-      <c r="E75" s="69" t="n">
+      <c r="E75" s="35" t="n">
         <v>0.194737</v>
       </c>
-      <c r="F75" s="69" t="n">
+      <c r="F75" s="35" t="n">
         <v>0.486842</v>
       </c>
-      <c r="G75" s="65" t="n">
+      <c r="G75" s="31" t="n">
         <v>0.0006024170362593856</v>
       </c>
-      <c r="H75" s="59" t="inlineStr">
+      <c r="H75" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -7249,19 +5997,19 @@
       <c r="C76" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D76" s="69" t="n">
+      <c r="D76" s="35" t="n">
         <v>0.273684</v>
       </c>
-      <c r="E76" s="69" t="n">
+      <c r="E76" s="35" t="n">
         <v>0.207519</v>
       </c>
-      <c r="F76" s="69" t="n">
+      <c r="F76" s="35" t="n">
         <v>0.518797</v>
       </c>
-      <c r="G76" s="65" t="n">
+      <c r="G76" s="31" t="n">
         <v>0.0006020357560719341</v>
       </c>
-      <c r="H76" s="59" t="inlineStr">
+      <c r="H76" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -7281,19 +6029,19 @@
       <c r="C77" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D77" s="69" t="n">
+      <c r="D77" s="35" t="n">
         <v>0.228947</v>
       </c>
-      <c r="E77" s="69" t="n">
+      <c r="E77" s="35" t="n">
         <v>0.220301</v>
       </c>
-      <c r="F77" s="69" t="n">
+      <c r="F77" s="35" t="n">
         <v>0.550752</v>
       </c>
-      <c r="G77" s="65" t="n">
+      <c r="G77" s="31" t="n">
         <v>0.0006016880609681081</v>
       </c>
-      <c r="H77" s="59" t="inlineStr">
+      <c r="H77" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -7313,19 +6061,19 @@
       <c r="C78" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D78" s="69" t="n">
+      <c r="D78" s="35" t="n">
         <v>0.184211</v>
       </c>
-      <c r="E78" s="69" t="n">
+      <c r="E78" s="35" t="n">
         <v>0.233083</v>
       </c>
-      <c r="F78" s="69" t="n">
+      <c r="F78" s="35" t="n">
         <v>0.582707</v>
       </c>
-      <c r="G78" s="65" t="n">
+      <c r="G78" s="31" t="n">
         <v>0.0003420427646720472</v>
       </c>
-      <c r="H78" s="59" t="inlineStr">
+      <c r="H78" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#2</t>
         </is>
@@ -7345,19 +6093,19 @@
       <c r="C79" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D79" s="69" t="n">
+      <c r="D79" s="35" t="n">
         <v>0.139474</v>
       </c>
-      <c r="E79" s="69" t="n">
+      <c r="E79" s="35" t="n">
         <v>0.245865</v>
       </c>
-      <c r="F79" s="69" t="n">
+      <c r="F79" s="35" t="n">
         <v>0.614662</v>
       </c>
-      <c r="G79" s="65" t="n">
+      <c r="G79" s="31" t="n">
         <v>0.0001478601310591977</v>
       </c>
-      <c r="H79" s="59" t="inlineStr">
+      <c r="H79" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#2</t>
         </is>
@@ -7377,26 +6125,26 @@
       <c r="C80" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D80" s="69" t="n">
+      <c r="D80" s="35" t="n">
         <v>0.094737</v>
       </c>
-      <c r="E80" s="69" t="n">
+      <c r="E80" s="35" t="n">
         <v>0.258647</v>
       </c>
-      <c r="F80" s="69" t="n">
+      <c r="F80" s="35" t="n">
         <v>0.646617</v>
       </c>
-      <c r="G80" s="65" t="n">
+      <c r="G80" s="31" t="n">
         <v>6.016951044280985e-05</v>
       </c>
-      <c r="H80" s="59" t="inlineStr">
+      <c r="H80" s="25" t="inlineStr">
         <is>
           <t>IONIC_LIQ#2</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="60" t="inlineStr">
+      <c r="A81" s="26" t="inlineStr">
         <is>
           <t>Cu-V-O</t>
         </is>
@@ -7409,19 +6157,19 @@
       <c r="C81" s="15" t="n">
         <v>1800</v>
       </c>
-      <c r="D81" s="70" t="n">
+      <c r="D81" s="36" t="n">
         <v>0.05</v>
       </c>
-      <c r="E81" s="70" t="n">
+      <c r="E81" s="36" t="n">
         <v>0.271429</v>
       </c>
-      <c r="F81" s="70" t="n">
+      <c r="F81" s="36" t="n">
         <v>0.678571</v>
       </c>
-      <c r="G81" s="67" t="n">
+      <c r="G81" s="33" t="n">
         <v>3.304376173394248e-05</v>
       </c>
-      <c r="H81" s="61" t="inlineStr">
+      <c r="H81" s="27" t="inlineStr">
         <is>
           <t>GAS#1; IONIC_LIQ#2</t>
         </is>
@@ -7432,7 +6180,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7496,7 +6244,7 @@
           <t>Fine-resolution dG vs T for top 6 ternary candidates (25 K steps, 800-1900 K)</t>
         </is>
       </c>
-      <c r="E2" s="58" t="inlineStr">
+      <c r="E2" s="24" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
@@ -7523,7 +6271,7 @@
           <t>CuFe2O4 formation decomposed into Cu-capture vs Fe-oxidation components (50 K steps, 800-1900 K)</t>
         </is>
       </c>
-      <c r="E3" s="59" t="inlineStr">
+      <c r="E3" s="25" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
@@ -7550,7 +6298,7 @@
           <t>Pre-computed Fe-oxidation and Cu-capture percentages</t>
         </is>
       </c>
-      <c r="E4" s="58" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
@@ -7577,7 +6325,7 @@
           <t>Cu activity in quaternary slag systems (Cu-Mn-Si-O, Cu-Al-Si-O) vs basicity ratio at 1800 K</t>
         </is>
       </c>
-      <c r="E5" s="59" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
@@ -7589,22 +6337,22 @@
           <t>cu_activity_vs_oxide.csv</t>
         </is>
       </c>
-      <c r="B6" s="45" t="inlineStr">
+      <c r="B6" s="37" t="inlineStr">
         <is>
           <t>simulations/tcpython/cu_activity_vs_oxide.py</t>
         </is>
       </c>
-      <c r="C6" s="45" t="inlineStr">
+      <c r="C6" s="37" t="inlineStr">
         <is>
           <t>TCOX14</t>
         </is>
       </c>
-      <c r="D6" s="45" t="inlineStr">
+      <c r="D6" s="37" t="inlineStr">
         <is>
           <t>Cu activity sweep at 1800 K across 4 ternary systems (Cu-Al-O, Cu-Mn-O, Cu-Fe-O, Cu-V-O), 20 compositions each</t>
         </is>
       </c>
-      <c r="E6" s="71" t="inlineStr">
+      <c r="E6" s="38" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>

</xml_diff>

<commit_message>
Restore Ternary and Validation xlsx to disk versions
Previous revert was incorrect - should not revert binary files
without inspecting contents or asking user first.
</commit_message>
<xml_diff>
--- a/screening/Validation_Results.xlsx
+++ b/screening/Validation_Results.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dG_vs_T" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CuFe2O4_Decomposition" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Ranking" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slag_Effects" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cu_Activity" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Sources" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity_Correction" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Ranking" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slag_Effects" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cu_Activity" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Sources" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,13 +22,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="+0.00;-0.00;0.00"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0.0000E+00"/>
-    <numFmt numFmtId="167" formatCode="0.000000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
+    <numFmt numFmtId="168" formatCode="+0.0;-0.0"/>
+    <numFmt numFmtId="169" formatCode="+0.0;-0.0;0.0"/>
+    <numFmt numFmtId="170" formatCode="0.0000E+00"/>
+    <numFmt numFmtId="171" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +48,15 @@
     <font>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="5">
@@ -137,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -208,6 +222,78 @@
     <xf numFmtId="165" fontId="0" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -223,31 +309,28 @@
     <xf numFmtId="165" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="0" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -257,6 +340,24 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+          <bgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -2502,6 +2603,1157 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>ACTIVITY CORRECTION PARAMETERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D2" s="27" t="inlineStr">
+        <is>
+          <t>Unit / Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>Cu mole fraction in steel</t>
+        </is>
+      </c>
+      <c r="B3" s="29" t="inlineStr">
+        <is>
+          <t>X_Cu</t>
+        </is>
+      </c>
+      <c r="C3" s="30" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D3" s="31" t="inlineStr">
+        <is>
+          <t>~0.3 wt% Cu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>Raoultian activity coefficient</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>γ_Cu</t>
+        </is>
+      </c>
+      <c r="C4" s="34" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>Literature range: 5-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>Cu activity in liquid Fe</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>a_Cu</t>
+        </is>
+      </c>
+      <c r="C5" s="30">
+        <f>C3*C4</f>
+        <v/>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
+          <t>X_Cu × γ_Cu</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>Temperature</t>
+        </is>
+      </c>
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D6" s="35" t="inlineStr">
+        <is>
+          <t>K (steelmaking)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Gas constant</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C7" s="36" t="n">
+        <v>8.314</v>
+      </c>
+      <c r="D7" s="31" t="inlineStr">
+        <is>
+          <t>J/(mol·K)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="37" t="inlineStr">
+        <is>
+          <t>Penalty per Cu atom consumed</t>
+        </is>
+      </c>
+      <c r="B8" s="38" t="inlineStr">
+        <is>
+          <t>-RT·ln(a_Cu)</t>
+        </is>
+      </c>
+      <c r="C8" s="39">
+        <f>-C7*C6*LN(C5)/1000</f>
+        <v/>
+      </c>
+      <c r="D8" s="40" t="inlineStr">
+        <is>
+          <t>kJ/mol (positive = less favorable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>ACTIVITY-CORRECTED ΔG AT 1800 K</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Parent Oxide</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>n_Cu</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>ΔG° (kJ)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Cu Penalty (kJ)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>ΔG_eff (kJ)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>ΔG per Cu (kJ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>CuFe2O4</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>FeO</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="41" t="n">
+        <v>-111.88</v>
+      </c>
+      <c r="E12" s="41">
+        <f>C12*$C$8</f>
+        <v/>
+      </c>
+      <c r="F12" s="41">
+        <f>D12+E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="12">
+        <f>IF(F12&lt;-10,"ROBUST",IF(F12&lt;0,"MARGINAL",IF(F12&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
+        <v/>
+      </c>
+      <c r="H12" s="42">
+        <f>D12/C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>CuMn2O4</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>MnO</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="43" t="n">
+        <v>-64.44</v>
+      </c>
+      <c r="E13" s="43">
+        <f>C13*$C$8</f>
+        <v/>
+      </c>
+      <c r="F13" s="43">
+        <f>D13+E13</f>
+        <v/>
+      </c>
+      <c r="G13" s="13">
+        <f>IF(F13&lt;-10,"ROBUST",IF(F13&lt;0,"MARGINAL",IF(F13&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
+        <v/>
+      </c>
+      <c r="H13" s="44">
+        <f>D13/C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>CuB2O4</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>B2O3</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="41" t="n">
+        <v>-47.71</v>
+      </c>
+      <c r="E14" s="41">
+        <f>C14*$C$8</f>
+        <v/>
+      </c>
+      <c r="F14" s="41">
+        <f>D14+E14</f>
+        <v/>
+      </c>
+      <c r="G14" s="12">
+        <f>IF(F14&lt;-10,"ROBUST",IF(F14&lt;0,"MARGINAL",IF(F14&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
+        <v/>
+      </c>
+      <c r="H14" s="42">
+        <f>D14/C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>CuV2O6</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>V2O5</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="43" t="n">
+        <v>-44.98</v>
+      </c>
+      <c r="E15" s="43">
+        <f>C15*$C$8</f>
+        <v/>
+      </c>
+      <c r="F15" s="43">
+        <f>D15+E15</f>
+        <v/>
+      </c>
+      <c r="G15" s="13">
+        <f>IF(F15&lt;-10,"ROBUST",IF(F15&lt;0,"MARGINAL",IF(F15&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
+        <v/>
+      </c>
+      <c r="H15" s="44">
+        <f>D15/C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>CuAl2O4</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Al2O3</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="41" t="n">
+        <v>-32.31</v>
+      </c>
+      <c r="E16" s="41">
+        <f>C16*$C$8</f>
+        <v/>
+      </c>
+      <c r="F16" s="41">
+        <f>D16+E16</f>
+        <v/>
+      </c>
+      <c r="G16" s="12">
+        <f>IF(F16&lt;-10,"ROBUST",IF(F16&lt;0,"MARGINAL",IF(F16&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
+        <v/>
+      </c>
+      <c r="H16" s="42">
+        <f>D16/C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Cu3V2O8</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>V2O5</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="43" t="n">
+        <v>-109.15</v>
+      </c>
+      <c r="E17" s="43">
+        <f>C17*$C$8</f>
+        <v/>
+      </c>
+      <c r="F17" s="43">
+        <f>D17+E17</f>
+        <v/>
+      </c>
+      <c r="G17" s="13">
+        <f>IF(F17&lt;-10,"ROBUST",IF(F17&lt;0,"MARGINAL",IF(F17&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
+        <v/>
+      </c>
+      <c r="H17" s="44">
+        <f>D17/C17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>Cu2SiO4</t>
+        </is>
+      </c>
+      <c r="B18" s="45" t="inlineStr">
+        <is>
+          <t>SiO2</t>
+        </is>
+      </c>
+      <c r="C18" s="45" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="46" t="n">
+        <v>-52.21</v>
+      </c>
+      <c r="E18" s="46">
+        <f>C18*$C$8</f>
+        <v/>
+      </c>
+      <c r="F18" s="46">
+        <f>D18+E18</f>
+        <v/>
+      </c>
+      <c r="G18" s="45">
+        <f>IF(F18&lt;-10,"ROBUST",IF(F18&lt;0,"MARGINAL",IF(F18&lt;15,"UNCERTAIN","UNFAVORABLE")))</f>
+        <v/>
+      </c>
+      <c r="H18" s="47">
+        <f>D18/C18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>γ_Cu SENSITIVITY ANALYSIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="48" t="inlineStr">
+        <is>
+          <t>Change γ_Cu in cell C4 above to see all corrections update automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>γ_Cu</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>a_Cu</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Penalty/Cu (kJ)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>ΔG_eff CuFe2O4</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>ΔG_eff CuMn2O4</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>ΔG_eff CuB2O4</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>ΔG_eff CuV2O6</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>ΔG_eff CuAl2O4</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>ΔG_eff Cu3V2O8</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>ΔG_eff Cu2SiO4</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="49" t="n">
+        <v>3</v>
+      </c>
+      <c r="B23" s="50">
+        <f>A23*$C$3</f>
+        <v/>
+      </c>
+      <c r="C23" s="51">
+        <f>-$C$7*$C$6*LN(B23)/1000</f>
+        <v/>
+      </c>
+      <c r="D23" s="41">
+        <f>-111.88+1*C23</f>
+        <v/>
+      </c>
+      <c r="E23" s="41">
+        <f>-64.44+1*C23</f>
+        <v/>
+      </c>
+      <c r="F23" s="41">
+        <f>-47.71+1*C23</f>
+        <v/>
+      </c>
+      <c r="G23" s="41">
+        <f>-44.98+1*C23</f>
+        <v/>
+      </c>
+      <c r="H23" s="41">
+        <f>-32.31+1*C23</f>
+        <v/>
+      </c>
+      <c r="I23" s="41">
+        <f>-109.15+3*C23</f>
+        <v/>
+      </c>
+      <c r="J23" s="42">
+        <f>-52.21+2*C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="B24" s="53">
+        <f>A24*$C$3</f>
+        <v/>
+      </c>
+      <c r="C24" s="54">
+        <f>-$C$7*$C$6*LN(B24)/1000</f>
+        <v/>
+      </c>
+      <c r="D24" s="43">
+        <f>-111.88+1*C24</f>
+        <v/>
+      </c>
+      <c r="E24" s="43">
+        <f>-64.44+1*C24</f>
+        <v/>
+      </c>
+      <c r="F24" s="43">
+        <f>-47.71+1*C24</f>
+        <v/>
+      </c>
+      <c r="G24" s="43">
+        <f>-44.98+1*C24</f>
+        <v/>
+      </c>
+      <c r="H24" s="43">
+        <f>-32.31+1*C24</f>
+        <v/>
+      </c>
+      <c r="I24" s="43">
+        <f>-109.15+3*C24</f>
+        <v/>
+      </c>
+      <c r="J24" s="44">
+        <f>-52.21+2*C24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="49" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" s="50">
+        <f>A25*$C$3</f>
+        <v/>
+      </c>
+      <c r="C25" s="51">
+        <f>-$C$7*$C$6*LN(B25)/1000</f>
+        <v/>
+      </c>
+      <c r="D25" s="41">
+        <f>-111.88+1*C25</f>
+        <v/>
+      </c>
+      <c r="E25" s="41">
+        <f>-64.44+1*C25</f>
+        <v/>
+      </c>
+      <c r="F25" s="41">
+        <f>-47.71+1*C25</f>
+        <v/>
+      </c>
+      <c r="G25" s="41">
+        <f>-44.98+1*C25</f>
+        <v/>
+      </c>
+      <c r="H25" s="41">
+        <f>-32.31+1*C25</f>
+        <v/>
+      </c>
+      <c r="I25" s="41">
+        <f>-109.15+3*C25</f>
+        <v/>
+      </c>
+      <c r="J25" s="42">
+        <f>-52.21+2*C25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="52" t="n">
+        <v>6</v>
+      </c>
+      <c r="B26" s="53">
+        <f>A26*$C$3</f>
+        <v/>
+      </c>
+      <c r="C26" s="54">
+        <f>-$C$7*$C$6*LN(B26)/1000</f>
+        <v/>
+      </c>
+      <c r="D26" s="43">
+        <f>-111.88+1*C26</f>
+        <v/>
+      </c>
+      <c r="E26" s="43">
+        <f>-64.44+1*C26</f>
+        <v/>
+      </c>
+      <c r="F26" s="43">
+        <f>-47.71+1*C26</f>
+        <v/>
+      </c>
+      <c r="G26" s="43">
+        <f>-44.98+1*C26</f>
+        <v/>
+      </c>
+      <c r="H26" s="43">
+        <f>-32.31+1*C26</f>
+        <v/>
+      </c>
+      <c r="I26" s="43">
+        <f>-109.15+3*C26</f>
+        <v/>
+      </c>
+      <c r="J26" s="44">
+        <f>-52.21+2*C26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="49" t="n">
+        <v>7</v>
+      </c>
+      <c r="B27" s="50">
+        <f>A27*$C$3</f>
+        <v/>
+      </c>
+      <c r="C27" s="51">
+        <f>-$C$7*$C$6*LN(B27)/1000</f>
+        <v/>
+      </c>
+      <c r="D27" s="41">
+        <f>-111.88+1*C27</f>
+        <v/>
+      </c>
+      <c r="E27" s="41">
+        <f>-64.44+1*C27</f>
+        <v/>
+      </c>
+      <c r="F27" s="41">
+        <f>-47.71+1*C27</f>
+        <v/>
+      </c>
+      <c r="G27" s="41">
+        <f>-44.98+1*C27</f>
+        <v/>
+      </c>
+      <c r="H27" s="41">
+        <f>-32.31+1*C27</f>
+        <v/>
+      </c>
+      <c r="I27" s="41">
+        <f>-109.15+3*C27</f>
+        <v/>
+      </c>
+      <c r="J27" s="42">
+        <f>-52.21+2*C27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="52" t="n">
+        <v>8</v>
+      </c>
+      <c r="B28" s="53">
+        <f>A28*$C$3</f>
+        <v/>
+      </c>
+      <c r="C28" s="54">
+        <f>-$C$7*$C$6*LN(B28)/1000</f>
+        <v/>
+      </c>
+      <c r="D28" s="43">
+        <f>-111.88+1*C28</f>
+        <v/>
+      </c>
+      <c r="E28" s="43">
+        <f>-64.44+1*C28</f>
+        <v/>
+      </c>
+      <c r="F28" s="43">
+        <f>-47.71+1*C28</f>
+        <v/>
+      </c>
+      <c r="G28" s="43">
+        <f>-44.98+1*C28</f>
+        <v/>
+      </c>
+      <c r="H28" s="43">
+        <f>-32.31+1*C28</f>
+        <v/>
+      </c>
+      <c r="I28" s="43">
+        <f>-109.15+3*C28</f>
+        <v/>
+      </c>
+      <c r="J28" s="44">
+        <f>-52.21+2*C28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="49" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="B29" s="50">
+        <f>A29*$C$3</f>
+        <v/>
+      </c>
+      <c r="C29" s="51">
+        <f>-$C$7*$C$6*LN(B29)/1000</f>
+        <v/>
+      </c>
+      <c r="D29" s="41">
+        <f>-111.88+1*C29</f>
+        <v/>
+      </c>
+      <c r="E29" s="41">
+        <f>-64.44+1*C29</f>
+        <v/>
+      </c>
+      <c r="F29" s="41">
+        <f>-47.71+1*C29</f>
+        <v/>
+      </c>
+      <c r="G29" s="41">
+        <f>-44.98+1*C29</f>
+        <v/>
+      </c>
+      <c r="H29" s="41">
+        <f>-32.31+1*C29</f>
+        <v/>
+      </c>
+      <c r="I29" s="41">
+        <f>-109.15+3*C29</f>
+        <v/>
+      </c>
+      <c r="J29" s="42">
+        <f>-52.21+2*C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="52" t="n">
+        <v>9</v>
+      </c>
+      <c r="B30" s="53">
+        <f>A30*$C$3</f>
+        <v/>
+      </c>
+      <c r="C30" s="54">
+        <f>-$C$7*$C$6*LN(B30)/1000</f>
+        <v/>
+      </c>
+      <c r="D30" s="43">
+        <f>-111.88+1*C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="43">
+        <f>-64.44+1*C30</f>
+        <v/>
+      </c>
+      <c r="F30" s="43">
+        <f>-47.71+1*C30</f>
+        <v/>
+      </c>
+      <c r="G30" s="43">
+        <f>-44.98+1*C30</f>
+        <v/>
+      </c>
+      <c r="H30" s="43">
+        <f>-32.31+1*C30</f>
+        <v/>
+      </c>
+      <c r="I30" s="43">
+        <f>-109.15+3*C30</f>
+        <v/>
+      </c>
+      <c r="J30" s="44">
+        <f>-52.21+2*C30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="49" t="n">
+        <v>10</v>
+      </c>
+      <c r="B31" s="50">
+        <f>A31*$C$3</f>
+        <v/>
+      </c>
+      <c r="C31" s="51">
+        <f>-$C$7*$C$6*LN(B31)/1000</f>
+        <v/>
+      </c>
+      <c r="D31" s="41">
+        <f>-111.88+1*C31</f>
+        <v/>
+      </c>
+      <c r="E31" s="41">
+        <f>-64.44+1*C31</f>
+        <v/>
+      </c>
+      <c r="F31" s="41">
+        <f>-47.71+1*C31</f>
+        <v/>
+      </c>
+      <c r="G31" s="41">
+        <f>-44.98+1*C31</f>
+        <v/>
+      </c>
+      <c r="H31" s="41">
+        <f>-32.31+1*C31</f>
+        <v/>
+      </c>
+      <c r="I31" s="41">
+        <f>-109.15+3*C31</f>
+        <v/>
+      </c>
+      <c r="J31" s="42">
+        <f>-52.21+2*C31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="52" t="n">
+        <v>11</v>
+      </c>
+      <c r="B32" s="53">
+        <f>A32*$C$3</f>
+        <v/>
+      </c>
+      <c r="C32" s="54">
+        <f>-$C$7*$C$6*LN(B32)/1000</f>
+        <v/>
+      </c>
+      <c r="D32" s="43">
+        <f>-111.88+1*C32</f>
+        <v/>
+      </c>
+      <c r="E32" s="43">
+        <f>-64.44+1*C32</f>
+        <v/>
+      </c>
+      <c r="F32" s="43">
+        <f>-47.71+1*C32</f>
+        <v/>
+      </c>
+      <c r="G32" s="43">
+        <f>-44.98+1*C32</f>
+        <v/>
+      </c>
+      <c r="H32" s="43">
+        <f>-32.31+1*C32</f>
+        <v/>
+      </c>
+      <c r="I32" s="43">
+        <f>-109.15+3*C32</f>
+        <v/>
+      </c>
+      <c r="J32" s="44">
+        <f>-52.21+2*C32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="49" t="n">
+        <v>12</v>
+      </c>
+      <c r="B33" s="50">
+        <f>A33*$C$3</f>
+        <v/>
+      </c>
+      <c r="C33" s="51">
+        <f>-$C$7*$C$6*LN(B33)/1000</f>
+        <v/>
+      </c>
+      <c r="D33" s="41">
+        <f>-111.88+1*C33</f>
+        <v/>
+      </c>
+      <c r="E33" s="41">
+        <f>-64.44+1*C33</f>
+        <v/>
+      </c>
+      <c r="F33" s="41">
+        <f>-47.71+1*C33</f>
+        <v/>
+      </c>
+      <c r="G33" s="41">
+        <f>-44.98+1*C33</f>
+        <v/>
+      </c>
+      <c r="H33" s="41">
+        <f>-32.31+1*C33</f>
+        <v/>
+      </c>
+      <c r="I33" s="41">
+        <f>-109.15+3*C33</f>
+        <v/>
+      </c>
+      <c r="J33" s="42">
+        <f>-52.21+2*C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="52" t="n">
+        <v>13</v>
+      </c>
+      <c r="B34" s="53">
+        <f>A34*$C$3</f>
+        <v/>
+      </c>
+      <c r="C34" s="54">
+        <f>-$C$7*$C$6*LN(B34)/1000</f>
+        <v/>
+      </c>
+      <c r="D34" s="43">
+        <f>-111.88+1*C34</f>
+        <v/>
+      </c>
+      <c r="E34" s="43">
+        <f>-64.44+1*C34</f>
+        <v/>
+      </c>
+      <c r="F34" s="43">
+        <f>-47.71+1*C34</f>
+        <v/>
+      </c>
+      <c r="G34" s="43">
+        <f>-44.98+1*C34</f>
+        <v/>
+      </c>
+      <c r="H34" s="43">
+        <f>-32.31+1*C34</f>
+        <v/>
+      </c>
+      <c r="I34" s="43">
+        <f>-109.15+3*C34</f>
+        <v/>
+      </c>
+      <c r="J34" s="44">
+        <f>-52.21+2*C34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="55" t="n">
+        <v>15</v>
+      </c>
+      <c r="B35" s="56">
+        <f>A35*$C$3</f>
+        <v/>
+      </c>
+      <c r="C35" s="57">
+        <f>-$C$7*$C$6*LN(B35)/1000</f>
+        <v/>
+      </c>
+      <c r="D35" s="46">
+        <f>-111.88+1*C35</f>
+        <v/>
+      </c>
+      <c r="E35" s="46">
+        <f>-64.44+1*C35</f>
+        <v/>
+      </c>
+      <c r="F35" s="46">
+        <f>-47.71+1*C35</f>
+        <v/>
+      </c>
+      <c r="G35" s="46">
+        <f>-44.98+1*C35</f>
+        <v/>
+      </c>
+      <c r="H35" s="46">
+        <f>-32.31+1*C35</f>
+        <v/>
+      </c>
+      <c r="I35" s="46">
+        <f>-109.15+3*C35</f>
+        <v/>
+      </c>
+      <c r="J35" s="47">
+        <f>-52.21+2*C35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="48" t="inlineStr">
+        <is>
+          <t>NOTE: V₂O₅ can form either Cu₃V₂O₈ (3 Cu, ΔG° = -109.2 kJ) or CuV₂O₆ (1 Cu, ΔG° = -45.0 kJ). Under dilute Cu conditions, CuV₂O₆ is preferred because the 3× penalty makes Cu₃V₂O₈ unfavorable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="48" t="inlineStr">
+        <is>
+          <t>Bureau of Mines (1960s) used ~1 wt% Cu (a_Cu ≈ 0.13), where both V₂O₅ products are favorable. Their 40-60% removal is consistent with our model.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A37:H37"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D23:D35">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E23:E35">
+    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F23:F35">
+    <cfRule type="cellIs" priority="5" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G23:G35">
+    <cfRule type="cellIs" priority="7" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H23:H35">
+    <cfRule type="cellIs" priority="9" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I23:I35">
+    <cfRule type="cellIs" priority="11" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="12" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J23:J35">
+    <cfRule type="cellIs" priority="13" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="14" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F12:F18">
+    <cfRule type="cellIs" priority="15" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="16" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2557,7 +3809,7 @@
       <c r="D2" s="12" t="n">
         <v>1700</v>
       </c>
-      <c r="E2" s="24" t="inlineStr">
+      <c r="E2" s="58" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
@@ -2583,7 +3835,7 @@
           <t>N/A (liquid)</t>
         </is>
       </c>
-      <c r="E3" s="25" t="inlineStr">
+      <c r="E3" s="59" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
@@ -2607,7 +3859,7 @@
       <c r="D4" s="12" t="n">
         <v>1700</v>
       </c>
-      <c r="E4" s="24" t="inlineStr">
+      <c r="E4" s="58" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
@@ -2633,7 +3885,7 @@
           <t>N/A (liquid)</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="59" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
@@ -2657,14 +3909,14 @@
       <c r="D6" s="12" t="n">
         <v>1300</v>
       </c>
-      <c r="E6" s="24" t="inlineStr">
+      <c r="E6" s="58" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>CuAl2O4</t>
         </is>
@@ -2681,7 +3933,7 @@
       <c r="D7" s="15" t="n">
         <v>1550</v>
       </c>
-      <c r="E7" s="27" t="inlineStr">
+      <c r="E7" s="61" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
@@ -2692,7 +3944,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2752,10 +4004,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C2" s="28" t="n">
+      <c r="C2" s="62" t="n">
         <v>0.2</v>
       </c>
-      <c r="D2" s="29" t="n">
+      <c r="D2" s="63" t="n">
         <v>0.0006024287195135149</v>
       </c>
       <c r="E2" s="12" t="inlineStr">
@@ -2778,10 +4030,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C3" s="28" t="n">
+      <c r="C3" s="62" t="n">
         <v>0.4</v>
       </c>
-      <c r="D3" s="29" t="n">
+      <c r="D3" s="63" t="n">
         <v>0.0005921646682545373</v>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -2805,10 +4057,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C4" s="28" t="n">
+      <c r="C4" s="62" t="n">
         <v>0.6</v>
       </c>
-      <c r="D4" s="29" t="n">
+      <c r="D4" s="63" t="n">
         <v>0.0005849859614188124</v>
       </c>
       <c r="E4" s="12" t="inlineStr">
@@ -2832,10 +4084,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C5" s="28" t="n">
+      <c r="C5" s="62" t="n">
         <v>0.8</v>
       </c>
-      <c r="D5" s="29" t="n">
+      <c r="D5" s="63" t="n">
         <v>0.0005795578709134352</v>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -2859,10 +4111,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C6" s="28" t="n">
+      <c r="C6" s="62" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="29" t="n">
+      <c r="D6" s="63" t="n">
         <v>0.0005747540319710688</v>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -2886,10 +4138,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C7" s="28" t="n">
+      <c r="C7" s="62" t="n">
         <v>1.2</v>
       </c>
-      <c r="D7" s="29" t="n">
+      <c r="D7" s="63" t="n">
         <v>0.0005690086100650586</v>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -2913,10 +4165,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C8" s="28" t="n">
+      <c r="C8" s="62" t="n">
         <v>1.4</v>
       </c>
-      <c r="D8" s="29" t="n">
+      <c r="D8" s="63" t="n">
         <v>0.0005623991726393003</v>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -2940,10 +4192,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="62" t="n">
         <v>1.6</v>
       </c>
-      <c r="D9" s="29" t="n">
+      <c r="D9" s="63" t="n">
         <v>0.0005549646048769486</v>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -2967,10 +4219,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="62" t="n">
         <v>1.8</v>
       </c>
-      <c r="D10" s="29" t="n">
+      <c r="D10" s="63" t="n">
         <v>0.0005469620453455369</v>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -2994,10 +4246,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C11" s="28" t="n">
+      <c r="C11" s="62" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="29" t="n">
+      <c r="D11" s="63" t="n">
         <v>0.0005386374910615401</v>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -3021,10 +4273,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C12" s="28" t="n">
+      <c r="C12" s="62" t="n">
         <v>2.2</v>
       </c>
-      <c r="D12" s="29" t="n">
+      <c r="D12" s="63" t="n">
         <v>0.0005302395956835024</v>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -3048,10 +4300,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C13" s="28" t="n">
+      <c r="C13" s="62" t="n">
         <v>2.4</v>
       </c>
-      <c r="D13" s="29" t="n">
+      <c r="D13" s="63" t="n">
         <v>0.0005220166239764437</v>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -3075,10 +4327,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C14" s="28" t="n">
+      <c r="C14" s="62" t="n">
         <v>2.6</v>
       </c>
-      <c r="D14" s="29" t="n">
+      <c r="D14" s="63" t="n">
         <v>0.0005141731215264483</v>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -3102,10 +4354,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C15" s="28" t="n">
+      <c r="C15" s="62" t="n">
         <v>2.8</v>
       </c>
-      <c r="D15" s="29" t="n">
+      <c r="D15" s="63" t="n">
         <v>0.000506844968432079</v>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -3129,10 +4381,10 @@
           <t>MnO:SiO2</t>
         </is>
       </c>
-      <c r="C16" s="28" t="n">
+      <c r="C16" s="62" t="n">
         <v>3</v>
       </c>
-      <c r="D16" s="29" t="n">
+      <c r="D16" s="63" t="n">
         <v>0.0005001045724686611</v>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -3156,10 +4408,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C17" s="30" t="n">
+      <c r="C17" s="64" t="n">
         <v>0.2</v>
       </c>
-      <c r="D17" s="31" t="n">
+      <c r="D17" s="65" t="n">
         <v>0.0006238595135610499</v>
       </c>
       <c r="E17" s="13" t="inlineStr">
@@ -3182,10 +4434,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C18" s="30" t="n">
+      <c r="C18" s="64" t="n">
         <v>0.4</v>
       </c>
-      <c r="D18" s="31" t="n">
+      <c r="D18" s="65" t="n">
         <v>0.0006238595135610499</v>
       </c>
       <c r="E18" s="13" t="inlineStr">
@@ -3209,10 +4461,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C19" s="30" t="n">
+      <c r="C19" s="64" t="n">
         <v>0.6</v>
       </c>
-      <c r="D19" s="31" t="n">
+      <c r="D19" s="65" t="n">
         <v>0.0006238595135610521</v>
       </c>
       <c r="E19" s="13" t="inlineStr">
@@ -3236,10 +4488,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C20" s="30" t="n">
+      <c r="C20" s="64" t="n">
         <v>0.8</v>
       </c>
-      <c r="D20" s="31" t="n">
+      <c r="D20" s="65" t="n">
         <v>0.0006238595135610521</v>
       </c>
       <c r="E20" s="13" t="inlineStr">
@@ -3263,10 +4515,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C21" s="30" t="n">
+      <c r="C21" s="64" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="31" t="n">
+      <c r="D21" s="65" t="n">
         <v>0.0006238595135610521</v>
       </c>
       <c r="E21" s="13" t="inlineStr">
@@ -3290,10 +4542,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C22" s="30" t="n">
+      <c r="C22" s="64" t="n">
         <v>1.2</v>
       </c>
-      <c r="D22" s="31" t="n">
+      <c r="D22" s="65" t="n">
         <v>0.0006238595135610504</v>
       </c>
       <c r="E22" s="13" t="inlineStr">
@@ -3317,10 +4569,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C23" s="30" t="n">
+      <c r="C23" s="64" t="n">
         <v>1.4</v>
       </c>
-      <c r="D23" s="31" t="n">
+      <c r="D23" s="65" t="n">
         <v>0.0006238595135610504</v>
       </c>
       <c r="E23" s="13" t="inlineStr">
@@ -3344,10 +4596,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C24" s="30" t="n">
+      <c r="C24" s="64" t="n">
         <v>1.6</v>
       </c>
-      <c r="D24" s="31" t="n">
+      <c r="D24" s="65" t="n">
         <v>0.0006240110028708597</v>
       </c>
       <c r="E24" s="13" t="inlineStr">
@@ -3371,10 +4623,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C25" s="30" t="n">
+      <c r="C25" s="64" t="n">
         <v>1.8</v>
       </c>
-      <c r="D25" s="31" t="n">
+      <c r="D25" s="65" t="n">
         <v>0.0006240764395684967</v>
       </c>
       <c r="E25" s="13" t="inlineStr">
@@ -3398,10 +4650,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C26" s="30" t="n">
+      <c r="C26" s="64" t="n">
         <v>2</v>
       </c>
-      <c r="D26" s="31" t="n">
+      <c r="D26" s="65" t="n">
         <v>0.0006240764395684967</v>
       </c>
       <c r="E26" s="13" t="inlineStr">
@@ -3425,10 +4677,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C27" s="30" t="n">
+      <c r="C27" s="64" t="n">
         <v>2.2</v>
       </c>
-      <c r="D27" s="31" t="n">
+      <c r="D27" s="65" t="n">
         <v>0.0006240764395684956</v>
       </c>
       <c r="E27" s="13" t="inlineStr">
@@ -3452,10 +4704,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C28" s="30" t="n">
+      <c r="C28" s="64" t="n">
         <v>2.4</v>
       </c>
-      <c r="D28" s="31" t="n">
+      <c r="D28" s="65" t="n">
         <v>0.0006240764395684967</v>
       </c>
       <c r="E28" s="13" t="inlineStr">
@@ -3479,10 +4731,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C29" s="30" t="n">
+      <c r="C29" s="64" t="n">
         <v>2.6</v>
       </c>
-      <c r="D29" s="31" t="n">
+      <c r="D29" s="65" t="n">
         <v>0.0006240764395684967</v>
       </c>
       <c r="E29" s="13" t="inlineStr">
@@ -3506,10 +4758,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C30" s="30" t="n">
+      <c r="C30" s="64" t="n">
         <v>2.8</v>
       </c>
-      <c r="D30" s="31" t="n">
+      <c r="D30" s="65" t="n">
         <v>0.0006240764395684973</v>
       </c>
       <c r="E30" s="13" t="inlineStr">
@@ -3523,7 +4775,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="26" t="inlineStr">
+      <c r="A31" s="60" t="inlineStr">
         <is>
           <t>Cu-Al-Si-O</t>
         </is>
@@ -3533,10 +4785,10 @@
           <t>Al2O3:SiO2</t>
         </is>
       </c>
-      <c r="C31" s="32" t="n">
+      <c r="C31" s="66" t="n">
         <v>3</v>
       </c>
-      <c r="D31" s="33" t="n">
+      <c r="D31" s="67" t="n">
         <v>0.0006240764395684973</v>
       </c>
       <c r="E31" s="15" t="inlineStr">
@@ -3554,7 +4806,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3629,19 +4881,19 @@
       <c r="C2" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D2" s="34" t="n">
+      <c r="D2" s="68" t="n">
         <v>0.9</v>
       </c>
-      <c r="E2" s="34" t="n">
+      <c r="E2" s="68" t="n">
         <v>0.04</v>
       </c>
-      <c r="F2" s="34" t="n">
+      <c r="F2" s="68" t="n">
         <v>0.06</v>
       </c>
-      <c r="G2" s="29" t="n">
+      <c r="G2" s="63" t="n">
         <v>0.0006242415932771841</v>
       </c>
-      <c r="H2" s="24" t="inlineStr">
+      <c r="H2" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3661,19 +4913,19 @@
       <c r="C3" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D3" s="34" t="n">
+      <c r="D3" s="68" t="n">
         <v>0.855263</v>
       </c>
-      <c r="E3" s="34" t="n">
+      <c r="E3" s="68" t="n">
         <v>0.057895</v>
       </c>
-      <c r="F3" s="34" t="n">
+      <c r="F3" s="68" t="n">
         <v>0.086842</v>
       </c>
-      <c r="G3" s="29" t="n">
+      <c r="G3" s="63" t="n">
         <v>0.000624241593277183</v>
       </c>
-      <c r="H3" s="24" t="inlineStr">
+      <c r="H3" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3693,19 +4945,19 @@
       <c r="C4" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D4" s="34" t="n">
+      <c r="D4" s="68" t="n">
         <v>0.810526</v>
       </c>
-      <c r="E4" s="34" t="n">
+      <c r="E4" s="68" t="n">
         <v>0.075789</v>
       </c>
-      <c r="F4" s="34" t="n">
+      <c r="F4" s="68" t="n">
         <v>0.113684</v>
       </c>
-      <c r="G4" s="29" t="n">
+      <c r="G4" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H4" s="24" t="inlineStr">
+      <c r="H4" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3725,19 +4977,19 @@
       <c r="C5" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D5" s="34" t="n">
+      <c r="D5" s="68" t="n">
         <v>0.7657890000000001</v>
       </c>
-      <c r="E5" s="34" t="n">
+      <c r="E5" s="68" t="n">
         <v>0.093684</v>
       </c>
-      <c r="F5" s="34" t="n">
+      <c r="F5" s="68" t="n">
         <v>0.140526</v>
       </c>
-      <c r="G5" s="29" t="n">
+      <c r="G5" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H5" s="24" t="inlineStr">
+      <c r="H5" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3757,19 +5009,19 @@
       <c r="C6" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D6" s="34" t="n">
+      <c r="D6" s="68" t="n">
         <v>0.7210530000000001</v>
       </c>
-      <c r="E6" s="34" t="n">
+      <c r="E6" s="68" t="n">
         <v>0.111579</v>
       </c>
-      <c r="F6" s="34" t="n">
+      <c r="F6" s="68" t="n">
         <v>0.167368</v>
       </c>
-      <c r="G6" s="29" t="n">
+      <c r="G6" s="63" t="n">
         <v>0.0006242415932771846</v>
       </c>
-      <c r="H6" s="24" t="inlineStr">
+      <c r="H6" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3789,19 +5041,19 @@
       <c r="C7" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D7" s="34" t="n">
+      <c r="D7" s="68" t="n">
         <v>0.676316</v>
       </c>
-      <c r="E7" s="34" t="n">
+      <c r="E7" s="68" t="n">
         <v>0.129474</v>
       </c>
-      <c r="F7" s="34" t="n">
+      <c r="F7" s="68" t="n">
         <v>0.194211</v>
       </c>
-      <c r="G7" s="29" t="n">
+      <c r="G7" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H7" s="24" t="inlineStr">
+      <c r="H7" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3821,19 +5073,19 @@
       <c r="C8" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D8" s="34" t="n">
+      <c r="D8" s="68" t="n">
         <v>0.631579</v>
       </c>
-      <c r="E8" s="34" t="n">
+      <c r="E8" s="68" t="n">
         <v>0.147368</v>
       </c>
-      <c r="F8" s="34" t="n">
+      <c r="F8" s="68" t="n">
         <v>0.221053</v>
       </c>
-      <c r="G8" s="29" t="n">
+      <c r="G8" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H8" s="24" t="inlineStr">
+      <c r="H8" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3853,19 +5105,19 @@
       <c r="C9" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D9" s="34" t="n">
+      <c r="D9" s="68" t="n">
         <v>0.586842</v>
       </c>
-      <c r="E9" s="34" t="n">
+      <c r="E9" s="68" t="n">
         <v>0.165263</v>
       </c>
-      <c r="F9" s="34" t="n">
+      <c r="F9" s="68" t="n">
         <v>0.247895</v>
       </c>
-      <c r="G9" s="29" t="n">
+      <c r="G9" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H9" s="24" t="inlineStr">
+      <c r="H9" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3885,19 +5137,19 @@
       <c r="C10" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D10" s="34" t="n">
+      <c r="D10" s="68" t="n">
         <v>0.5421049999999999</v>
       </c>
-      <c r="E10" s="34" t="n">
+      <c r="E10" s="68" t="n">
         <v>0.183158</v>
       </c>
-      <c r="F10" s="34" t="n">
+      <c r="F10" s="68" t="n">
         <v>0.274737</v>
       </c>
-      <c r="G10" s="29" t="n">
+      <c r="G10" s="63" t="n">
         <v>0.0006242415932771825</v>
       </c>
-      <c r="H10" s="24" t="inlineStr">
+      <c r="H10" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3917,19 +5169,19 @@
       <c r="C11" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D11" s="34" t="n">
+      <c r="D11" s="68" t="n">
         <v>0.497368</v>
       </c>
-      <c r="E11" s="34" t="n">
+      <c r="E11" s="68" t="n">
         <v>0.201053</v>
       </c>
-      <c r="F11" s="34" t="n">
+      <c r="F11" s="68" t="n">
         <v>0.301579</v>
       </c>
-      <c r="G11" s="29" t="n">
+      <c r="G11" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H11" s="24" t="inlineStr">
+      <c r="H11" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3949,19 +5201,19 @@
       <c r="C12" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D12" s="34" t="n">
+      <c r="D12" s="68" t="n">
         <v>0.452632</v>
       </c>
-      <c r="E12" s="34" t="n">
+      <c r="E12" s="68" t="n">
         <v>0.218947</v>
       </c>
-      <c r="F12" s="34" t="n">
+      <c r="F12" s="68" t="n">
         <v>0.328421</v>
       </c>
-      <c r="G12" s="29" t="n">
+      <c r="G12" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H12" s="24" t="inlineStr">
+      <c r="H12" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -3981,19 +5233,19 @@
       <c r="C13" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D13" s="34" t="n">
+      <c r="D13" s="68" t="n">
         <v>0.407895</v>
       </c>
-      <c r="E13" s="34" t="n">
+      <c r="E13" s="68" t="n">
         <v>0.236842</v>
       </c>
-      <c r="F13" s="34" t="n">
+      <c r="F13" s="68" t="n">
         <v>0.355263</v>
       </c>
-      <c r="G13" s="29" t="n">
+      <c r="G13" s="63" t="n">
         <v>0.000624241593277183</v>
       </c>
-      <c r="H13" s="24" t="inlineStr">
+      <c r="H13" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4013,19 +5265,19 @@
       <c r="C14" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D14" s="34" t="n">
+      <c r="D14" s="68" t="n">
         <v>0.363158</v>
       </c>
-      <c r="E14" s="34" t="n">
+      <c r="E14" s="68" t="n">
         <v>0.254737</v>
       </c>
-      <c r="F14" s="34" t="n">
+      <c r="F14" s="68" t="n">
         <v>0.382105</v>
       </c>
-      <c r="G14" s="29" t="n">
+      <c r="G14" s="63" t="n">
         <v>0.0006242415932771836</v>
       </c>
-      <c r="H14" s="24" t="inlineStr">
+      <c r="H14" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4045,19 +5297,19 @@
       <c r="C15" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D15" s="34" t="n">
+      <c r="D15" s="68" t="n">
         <v>0.318421</v>
       </c>
-      <c r="E15" s="34" t="n">
+      <c r="E15" s="68" t="n">
         <v>0.272632</v>
       </c>
-      <c r="F15" s="34" t="n">
+      <c r="F15" s="68" t="n">
         <v>0.408947</v>
       </c>
-      <c r="G15" s="29" t="n">
+      <c r="G15" s="63" t="n">
         <v>0.0006242415932771846</v>
       </c>
-      <c r="H15" s="24" t="inlineStr">
+      <c r="H15" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4077,19 +5329,19 @@
       <c r="C16" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D16" s="34" t="n">
+      <c r="D16" s="68" t="n">
         <v>0.273684</v>
       </c>
-      <c r="E16" s="34" t="n">
+      <c r="E16" s="68" t="n">
         <v>0.290526</v>
       </c>
-      <c r="F16" s="34" t="n">
+      <c r="F16" s="68" t="n">
         <v>0.435789</v>
       </c>
-      <c r="G16" s="29" t="n">
+      <c r="G16" s="63" t="n">
         <v>0.000624241593277183</v>
       </c>
-      <c r="H16" s="24" t="inlineStr">
+      <c r="H16" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4109,19 +5361,19 @@
       <c r="C17" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D17" s="34" t="n">
+      <c r="D17" s="68" t="n">
         <v>0.228947</v>
       </c>
-      <c r="E17" s="34" t="n">
+      <c r="E17" s="68" t="n">
         <v>0.308421</v>
       </c>
-      <c r="F17" s="34" t="n">
+      <c r="F17" s="68" t="n">
         <v>0.462632</v>
       </c>
-      <c r="G17" s="29" t="n">
+      <c r="G17" s="63" t="n">
         <v>0.0006242415932771825</v>
       </c>
-      <c r="H17" s="24" t="inlineStr">
+      <c r="H17" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4141,19 +5393,19 @@
       <c r="C18" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D18" s="34" t="n">
+      <c r="D18" s="68" t="n">
         <v>0.184211</v>
       </c>
-      <c r="E18" s="34" t="n">
+      <c r="E18" s="68" t="n">
         <v>0.326316</v>
       </c>
-      <c r="F18" s="34" t="n">
+      <c r="F18" s="68" t="n">
         <v>0.489474</v>
       </c>
-      <c r="G18" s="29" t="n">
+      <c r="G18" s="63" t="n">
         <v>0.0006242415932771825</v>
       </c>
-      <c r="H18" s="24" t="inlineStr">
+      <c r="H18" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4173,19 +5425,19 @@
       <c r="C19" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D19" s="34" t="n">
+      <c r="D19" s="68" t="n">
         <v>0.139474</v>
       </c>
-      <c r="E19" s="34" t="n">
+      <c r="E19" s="68" t="n">
         <v>0.344211</v>
       </c>
-      <c r="F19" s="34" t="n">
+      <c r="F19" s="68" t="n">
         <v>0.516316</v>
       </c>
-      <c r="G19" s="29" t="n">
+      <c r="G19" s="63" t="n">
         <v>0.000624241593277183</v>
       </c>
-      <c r="H19" s="24" t="inlineStr">
+      <c r="H19" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4205,19 +5457,19 @@
       <c r="C20" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D20" s="34" t="n">
+      <c r="D20" s="68" t="n">
         <v>0.094737</v>
       </c>
-      <c r="E20" s="34" t="n">
+      <c r="E20" s="68" t="n">
         <v>0.362105</v>
       </c>
-      <c r="F20" s="34" t="n">
+      <c r="F20" s="68" t="n">
         <v>0.543158</v>
       </c>
-      <c r="G20" s="29" t="n">
+      <c r="G20" s="63" t="n">
         <v>0.0006242415932771825</v>
       </c>
-      <c r="H20" s="24" t="inlineStr">
+      <c r="H20" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4237,19 +5489,19 @@
       <c r="C21" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D21" s="34" t="n">
+      <c r="D21" s="68" t="n">
         <v>0.05</v>
       </c>
-      <c r="E21" s="34" t="n">
+      <c r="E21" s="68" t="n">
         <v>0.38</v>
       </c>
-      <c r="F21" s="34" t="n">
+      <c r="F21" s="68" t="n">
         <v>0.57</v>
       </c>
-      <c r="G21" s="29" t="n">
+      <c r="G21" s="63" t="n">
         <v>0.0006242415932771841</v>
       </c>
-      <c r="H21" s="24" t="inlineStr">
+      <c r="H21" s="58" t="inlineStr">
         <is>
           <t>CORUNDUM#1; IONIC_LIQ#1</t>
         </is>
@@ -4269,19 +5521,19 @@
       <c r="C22" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D22" s="35" t="n">
+      <c r="D22" s="69" t="n">
         <v>0.9</v>
       </c>
-      <c r="E22" s="35" t="n">
+      <c r="E22" s="69" t="n">
         <v>0.05</v>
       </c>
-      <c r="F22" s="35" t="n">
+      <c r="F22" s="69" t="n">
         <v>0.05</v>
       </c>
-      <c r="G22" s="31" t="n">
+      <c r="G22" s="65" t="n">
         <v>0.0006234486982757811</v>
       </c>
-      <c r="H22" s="25" t="inlineStr">
+      <c r="H22" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4301,19 +5553,19 @@
       <c r="C23" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D23" s="35" t="n">
+      <c r="D23" s="69" t="n">
         <v>0.855263</v>
       </c>
-      <c r="E23" s="35" t="n">
+      <c r="E23" s="69" t="n">
         <v>0.072368</v>
       </c>
-      <c r="F23" s="35" t="n">
+      <c r="F23" s="69" t="n">
         <v>0.072368</v>
       </c>
-      <c r="G23" s="31" t="n">
+      <c r="G23" s="65" t="n">
         <v>0.0006234240698697985</v>
       </c>
-      <c r="H23" s="25" t="inlineStr">
+      <c r="H23" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4333,19 +5585,19 @@
       <c r="C24" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D24" s="35" t="n">
+      <c r="D24" s="69" t="n">
         <v>0.810526</v>
       </c>
-      <c r="E24" s="35" t="n">
+      <c r="E24" s="69" t="n">
         <v>0.094737</v>
       </c>
-      <c r="F24" s="35" t="n">
+      <c r="F24" s="69" t="n">
         <v>0.094737</v>
       </c>
-      <c r="G24" s="31" t="n">
+      <c r="G24" s="65" t="n">
         <v>0.000623390113702764</v>
       </c>
-      <c r="H24" s="25" t="inlineStr">
+      <c r="H24" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4365,19 +5617,19 @@
       <c r="C25" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D25" s="35" t="n">
+      <c r="D25" s="69" t="n">
         <v>0.7657890000000001</v>
       </c>
-      <c r="E25" s="35" t="n">
+      <c r="E25" s="69" t="n">
         <v>0.117105</v>
       </c>
-      <c r="F25" s="35" t="n">
+      <c r="F25" s="69" t="n">
         <v>0.117105</v>
       </c>
-      <c r="G25" s="31" t="n">
+      <c r="G25" s="65" t="n">
         <v>0.0006233465051459715</v>
       </c>
-      <c r="H25" s="25" t="inlineStr">
+      <c r="H25" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4397,19 +5649,19 @@
       <c r="C26" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D26" s="35" t="n">
+      <c r="D26" s="69" t="n">
         <v>0.7210530000000001</v>
       </c>
-      <c r="E26" s="35" t="n">
+      <c r="E26" s="69" t="n">
         <v>0.139474</v>
       </c>
-      <c r="F26" s="35" t="n">
+      <c r="F26" s="69" t="n">
         <v>0.139474</v>
       </c>
-      <c r="G26" s="31" t="n">
+      <c r="G26" s="65" t="n">
         <v>0.0006232927260585453</v>
       </c>
-      <c r="H26" s="25" t="inlineStr">
+      <c r="H26" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4429,19 +5681,19 @@
       <c r="C27" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D27" s="35" t="n">
+      <c r="D27" s="69" t="n">
         <v>0.676316</v>
       </c>
-      <c r="E27" s="35" t="n">
+      <c r="E27" s="69" t="n">
         <v>0.161842</v>
       </c>
-      <c r="F27" s="35" t="n">
+      <c r="F27" s="69" t="n">
         <v>0.161842</v>
       </c>
-      <c r="G27" s="31" t="n">
+      <c r="G27" s="65" t="n">
         <v>0.0006232279909242769</v>
       </c>
-      <c r="H27" s="25" t="inlineStr">
+      <c r="H27" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4461,19 +5713,19 @@
       <c r="C28" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D28" s="35" t="n">
+      <c r="D28" s="69" t="n">
         <v>0.631579</v>
       </c>
-      <c r="E28" s="35" t="n">
+      <c r="E28" s="69" t="n">
         <v>0.184211</v>
       </c>
-      <c r="F28" s="35" t="n">
+      <c r="F28" s="69" t="n">
         <v>0.184211</v>
       </c>
-      <c r="G28" s="31" t="n">
+      <c r="G28" s="65" t="n">
         <v>0.0006231511590811589</v>
       </c>
-      <c r="H28" s="25" t="inlineStr">
+      <c r="H28" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4493,19 +5745,19 @@
       <c r="C29" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D29" s="35" t="n">
+      <c r="D29" s="69" t="n">
         <v>0.586842</v>
       </c>
-      <c r="E29" s="35" t="n">
+      <c r="E29" s="69" t="n">
         <v>0.206579</v>
       </c>
-      <c r="F29" s="35" t="n">
+      <c r="F29" s="69" t="n">
         <v>0.206579</v>
       </c>
-      <c r="G29" s="31" t="n">
+      <c r="G29" s="65" t="n">
         <v>0.0006230606192890642</v>
       </c>
-      <c r="H29" s="25" t="inlineStr">
+      <c r="H29" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4525,19 +5777,19 @@
       <c r="C30" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D30" s="35" t="n">
+      <c r="D30" s="69" t="n">
         <v>0.5421049999999999</v>
       </c>
-      <c r="E30" s="35" t="n">
+      <c r="E30" s="69" t="n">
         <v>0.228947</v>
       </c>
-      <c r="F30" s="35" t="n">
+      <c r="F30" s="69" t="n">
         <v>0.228947</v>
       </c>
-      <c r="G30" s="31" t="n">
+      <c r="G30" s="65" t="n">
         <v>0.0006229541258469519</v>
       </c>
-      <c r="H30" s="25" t="inlineStr">
+      <c r="H30" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4557,19 +5809,19 @@
       <c r="C31" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D31" s="35" t="n">
+      <c r="D31" s="69" t="n">
         <v>0.497368</v>
       </c>
-      <c r="E31" s="35" t="n">
+      <c r="E31" s="69" t="n">
         <v>0.251316</v>
       </c>
-      <c r="F31" s="35" t="n">
+      <c r="F31" s="69" t="n">
         <v>0.251316</v>
       </c>
-      <c r="G31" s="31" t="n">
+      <c r="G31" s="65" t="n">
         <v>0.0006228285531386366</v>
       </c>
-      <c r="H31" s="25" t="inlineStr">
+      <c r="H31" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4589,19 +5841,19 @@
       <c r="C32" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D32" s="35" t="n">
+      <c r="D32" s="69" t="n">
         <v>0.452632</v>
       </c>
-      <c r="E32" s="35" t="n">
+      <c r="E32" s="69" t="n">
         <v>0.273684</v>
       </c>
-      <c r="F32" s="35" t="n">
+      <c r="F32" s="69" t="n">
         <v>0.273684</v>
       </c>
-      <c r="G32" s="31" t="n">
+      <c r="G32" s="65" t="n">
         <v>0.0006226795122556773</v>
       </c>
-      <c r="H32" s="25" t="inlineStr">
+      <c r="H32" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4621,19 +5873,19 @@
       <c r="C33" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D33" s="35" t="n">
+      <c r="D33" s="69" t="n">
         <v>0.407895</v>
       </c>
-      <c r="E33" s="35" t="n">
+      <c r="E33" s="69" t="n">
         <v>0.296053</v>
       </c>
-      <c r="F33" s="35" t="n">
+      <c r="F33" s="69" t="n">
         <v>0.296053</v>
       </c>
-      <c r="G33" s="31" t="n">
+      <c r="G33" s="65" t="n">
         <v>0.000622500727556083</v>
       </c>
-      <c r="H33" s="25" t="inlineStr">
+      <c r="H33" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4653,19 +5905,19 @@
       <c r="C34" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D34" s="35" t="n">
+      <c r="D34" s="69" t="n">
         <v>0.363158</v>
       </c>
-      <c r="E34" s="35" t="n">
+      <c r="E34" s="69" t="n">
         <v>0.318421</v>
       </c>
-      <c r="F34" s="35" t="n">
+      <c r="F34" s="69" t="n">
         <v>0.318421</v>
       </c>
-      <c r="G34" s="31" t="n">
+      <c r="G34" s="65" t="n">
         <v>0.0006222829760272391</v>
       </c>
-      <c r="H34" s="25" t="inlineStr">
+      <c r="H34" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4685,19 +5937,19 @@
       <c r="C35" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D35" s="35" t="n">
+      <c r="D35" s="69" t="n">
         <v>0.318421</v>
       </c>
-      <c r="E35" s="35" t="n">
+      <c r="E35" s="69" t="n">
         <v>0.340789</v>
       </c>
-      <c r="F35" s="35" t="n">
+      <c r="F35" s="69" t="n">
         <v>0.340789</v>
       </c>
-      <c r="G35" s="31" t="n">
+      <c r="G35" s="65" t="n">
         <v>0.0006220121819606671</v>
       </c>
-      <c r="H35" s="25" t="inlineStr">
+      <c r="H35" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4717,19 +5969,19 @@
       <c r="C36" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D36" s="35" t="n">
+      <c r="D36" s="69" t="n">
         <v>0.273684</v>
       </c>
-      <c r="E36" s="35" t="n">
+      <c r="E36" s="69" t="n">
         <v>0.363158</v>
       </c>
-      <c r="F36" s="35" t="n">
+      <c r="F36" s="69" t="n">
         <v>0.363158</v>
       </c>
-      <c r="G36" s="31" t="n">
+      <c r="G36" s="65" t="n">
         <v>0.0006216657532754782</v>
       </c>
-      <c r="H36" s="25" t="inlineStr">
+      <c r="H36" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4749,19 +6001,19 @@
       <c r="C37" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D37" s="35" t="n">
+      <c r="D37" s="69" t="n">
         <v>0.228947</v>
       </c>
-      <c r="E37" s="35" t="n">
+      <c r="E37" s="69" t="n">
         <v>0.385526</v>
       </c>
-      <c r="F37" s="35" t="n">
+      <c r="F37" s="69" t="n">
         <v>0.385526</v>
       </c>
-      <c r="G37" s="31" t="n">
+      <c r="G37" s="65" t="n">
         <v>0.0006212048918444731</v>
       </c>
-      <c r="H37" s="25" t="inlineStr">
+      <c r="H37" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4781,19 +6033,19 @@
       <c r="C38" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D38" s="35" t="n">
+      <c r="D38" s="69" t="n">
         <v>0.184211</v>
       </c>
-      <c r="E38" s="35" t="n">
+      <c r="E38" s="69" t="n">
         <v>0.407895</v>
       </c>
-      <c r="F38" s="35" t="n">
+      <c r="F38" s="69" t="n">
         <v>0.407895</v>
       </c>
-      <c r="G38" s="31" t="n">
+      <c r="G38" s="65" t="n">
         <v>0.0006205564490138872</v>
       </c>
-      <c r="H38" s="25" t="inlineStr">
+      <c r="H38" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4813,19 +6065,19 @@
       <c r="C39" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D39" s="35" t="n">
+      <c r="D39" s="69" t="n">
         <v>0.139474</v>
       </c>
-      <c r="E39" s="35" t="n">
+      <c r="E39" s="69" t="n">
         <v>0.430263</v>
       </c>
-      <c r="F39" s="35" t="n">
+      <c r="F39" s="69" t="n">
         <v>0.430263</v>
       </c>
-      <c r="G39" s="31" t="n">
+      <c r="G39" s="65" t="n">
         <v>0.0006195624103164132</v>
       </c>
-      <c r="H39" s="25" t="inlineStr">
+      <c r="H39" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4845,19 +6097,19 @@
       <c r="C40" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D40" s="35" t="n">
+      <c r="D40" s="69" t="n">
         <v>0.094737</v>
       </c>
-      <c r="E40" s="35" t="n">
+      <c r="E40" s="69" t="n">
         <v>0.452632</v>
       </c>
-      <c r="F40" s="35" t="n">
+      <c r="F40" s="69" t="n">
         <v>0.452632</v>
       </c>
-      <c r="G40" s="31" t="n">
+      <c r="G40" s="65" t="n">
         <v>0.0006177982099275926</v>
       </c>
-      <c r="H40" s="25" t="inlineStr">
+      <c r="H40" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4877,19 +6129,19 @@
       <c r="C41" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D41" s="35" t="n">
+      <c r="D41" s="69" t="n">
         <v>0.05</v>
       </c>
-      <c r="E41" s="35" t="n">
+      <c r="E41" s="69" t="n">
         <v>0.475</v>
       </c>
-      <c r="F41" s="35" t="n">
+      <c r="F41" s="69" t="n">
         <v>0.475</v>
       </c>
-      <c r="G41" s="31" t="n">
+      <c r="G41" s="65" t="n">
         <v>0.0006135214100988033</v>
       </c>
-      <c r="H41" s="25" t="inlineStr">
+      <c r="H41" s="59" t="inlineStr">
         <is>
           <t>HALITE#1; IONIC_LIQ#1</t>
         </is>
@@ -4909,19 +6161,19 @@
       <c r="C42" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D42" s="34" t="n">
+      <c r="D42" s="68" t="n">
         <v>0.9</v>
       </c>
-      <c r="E42" s="34" t="n">
+      <c r="E42" s="68" t="n">
         <v>0.05</v>
       </c>
-      <c r="F42" s="34" t="n">
+      <c r="F42" s="68" t="n">
         <v>0.05</v>
       </c>
-      <c r="G42" s="29" t="n">
+      <c r="G42" s="63" t="n">
         <v>0.0006192201975493238</v>
       </c>
-      <c r="H42" s="24" t="inlineStr">
+      <c r="H42" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -4941,19 +6193,19 @@
       <c r="C43" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D43" s="34" t="n">
+      <c r="D43" s="68" t="n">
         <v>0.855263</v>
       </c>
-      <c r="E43" s="34" t="n">
+      <c r="E43" s="68" t="n">
         <v>0.072368</v>
       </c>
-      <c r="F43" s="34" t="n">
+      <c r="F43" s="68" t="n">
         <v>0.072368</v>
       </c>
-      <c r="G43" s="29" t="n">
+      <c r="G43" s="63" t="n">
         <v>0.0006178389962257873</v>
       </c>
-      <c r="H43" s="24" t="inlineStr">
+      <c r="H43" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -4973,19 +6225,19 @@
       <c r="C44" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D44" s="34" t="n">
+      <c r="D44" s="68" t="n">
         <v>0.810526</v>
       </c>
-      <c r="E44" s="34" t="n">
+      <c r="E44" s="68" t="n">
         <v>0.094737</v>
       </c>
-      <c r="F44" s="34" t="n">
+      <c r="F44" s="68" t="n">
         <v>0.094737</v>
       </c>
-      <c r="G44" s="29" t="n">
+      <c r="G44" s="63" t="n">
         <v>0.0006164156519341792</v>
       </c>
-      <c r="H44" s="24" t="inlineStr">
+      <c r="H44" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5005,19 +6257,19 @@
       <c r="C45" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D45" s="34" t="n">
+      <c r="D45" s="68" t="n">
         <v>0.7657890000000001</v>
       </c>
-      <c r="E45" s="34" t="n">
+      <c r="E45" s="68" t="n">
         <v>0.117105</v>
       </c>
-      <c r="F45" s="34" t="n">
+      <c r="F45" s="68" t="n">
         <v>0.117105</v>
       </c>
-      <c r="G45" s="29" t="n">
+      <c r="G45" s="63" t="n">
         <v>0.0006149434371808388</v>
       </c>
-      <c r="H45" s="24" t="inlineStr">
+      <c r="H45" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5037,19 +6289,19 @@
       <c r="C46" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D46" s="34" t="n">
+      <c r="D46" s="68" t="n">
         <v>0.7210530000000001</v>
       </c>
-      <c r="E46" s="34" t="n">
+      <c r="E46" s="68" t="n">
         <v>0.139474</v>
       </c>
-      <c r="F46" s="34" t="n">
+      <c r="F46" s="68" t="n">
         <v>0.139474</v>
       </c>
-      <c r="G46" s="29" t="n">
+      <c r="G46" s="63" t="n">
         <v>0.0006134086362605692</v>
       </c>
-      <c r="H46" s="24" t="inlineStr">
+      <c r="H46" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5069,19 +6321,19 @@
       <c r="C47" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D47" s="34" t="n">
+      <c r="D47" s="68" t="n">
         <v>0.676316</v>
       </c>
-      <c r="E47" s="34" t="n">
+      <c r="E47" s="68" t="n">
         <v>0.161842</v>
       </c>
-      <c r="F47" s="34" t="n">
+      <c r="F47" s="68" t="n">
         <v>0.161842</v>
       </c>
-      <c r="G47" s="29" t="n">
+      <c r="G47" s="63" t="n">
         <v>0.000611794507683605</v>
       </c>
-      <c r="H47" s="24" t="inlineStr">
+      <c r="H47" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5101,19 +6353,19 @@
       <c r="C48" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D48" s="34" t="n">
+      <c r="D48" s="68" t="n">
         <v>0.631579</v>
       </c>
-      <c r="E48" s="34" t="n">
+      <c r="E48" s="68" t="n">
         <v>0.184211</v>
       </c>
-      <c r="F48" s="34" t="n">
+      <c r="F48" s="68" t="n">
         <v>0.184211</v>
       </c>
-      <c r="G48" s="29" t="n">
+      <c r="G48" s="63" t="n">
         <v>0.0006100815926117644</v>
       </c>
-      <c r="H48" s="24" t="inlineStr">
+      <c r="H48" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5133,19 +6385,19 @@
       <c r="C49" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D49" s="34" t="n">
+      <c r="D49" s="68" t="n">
         <v>0.586842</v>
       </c>
-      <c r="E49" s="34" t="n">
+      <c r="E49" s="68" t="n">
         <v>0.206579</v>
       </c>
-      <c r="F49" s="34" t="n">
+      <c r="F49" s="68" t="n">
         <v>0.206579</v>
       </c>
-      <c r="G49" s="29" t="n">
+      <c r="G49" s="63" t="n">
         <v>0.0006082469669095847</v>
       </c>
-      <c r="H49" s="24" t="inlineStr">
+      <c r="H49" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5165,19 +6417,19 @@
       <c r="C50" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D50" s="34" t="n">
+      <c r="D50" s="68" t="n">
         <v>0.5421049999999999</v>
       </c>
-      <c r="E50" s="34" t="n">
+      <c r="E50" s="68" t="n">
         <v>0.228947</v>
       </c>
-      <c r="F50" s="34" t="n">
+      <c r="F50" s="68" t="n">
         <v>0.228947</v>
       </c>
-      <c r="G50" s="29" t="n">
+      <c r="G50" s="63" t="n">
         <v>0.0006062629201632612</v>
       </c>
-      <c r="H50" s="24" t="inlineStr">
+      <c r="H50" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5197,19 +6449,19 @@
       <c r="C51" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D51" s="34" t="n">
+      <c r="D51" s="68" t="n">
         <v>0.497368</v>
       </c>
-      <c r="E51" s="34" t="n">
+      <c r="E51" s="68" t="n">
         <v>0.251316</v>
       </c>
-      <c r="F51" s="34" t="n">
+      <c r="F51" s="68" t="n">
         <v>0.251316</v>
       </c>
-      <c r="G51" s="29" t="n">
+      <c r="G51" s="63" t="n">
         <v>0.0006040950268609877</v>
       </c>
-      <c r="H51" s="24" t="inlineStr">
+      <c r="H51" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5229,19 +6481,19 @@
       <c r="C52" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D52" s="34" t="n">
+      <c r="D52" s="68" t="n">
         <v>0.452632</v>
       </c>
-      <c r="E52" s="34" t="n">
+      <c r="E52" s="68" t="n">
         <v>0.273684</v>
       </c>
-      <c r="F52" s="34" t="n">
+      <c r="F52" s="68" t="n">
         <v>0.273684</v>
       </c>
-      <c r="G52" s="29" t="n">
+      <c r="G52" s="63" t="n">
         <v>0.00060169933822934</v>
       </c>
-      <c r="H52" s="24" t="inlineStr">
+      <c r="H52" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5261,19 +6513,19 @@
       <c r="C53" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D53" s="34" t="n">
+      <c r="D53" s="68" t="n">
         <v>0.407895</v>
       </c>
-      <c r="E53" s="34" t="n">
+      <c r="E53" s="68" t="n">
         <v>0.296053</v>
       </c>
-      <c r="F53" s="34" t="n">
+      <c r="F53" s="68" t="n">
         <v>0.296053</v>
       </c>
-      <c r="G53" s="29" t="n">
+      <c r="G53" s="63" t="n">
         <v>0.0005990181736125742</v>
       </c>
-      <c r="H53" s="24" t="inlineStr">
+      <c r="H53" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5293,19 +6545,19 @@
       <c r="C54" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D54" s="34" t="n">
+      <c r="D54" s="68" t="n">
         <v>0.363158</v>
       </c>
-      <c r="E54" s="34" t="n">
+      <c r="E54" s="68" t="n">
         <v>0.318421</v>
       </c>
-      <c r="F54" s="34" t="n">
+      <c r="F54" s="68" t="n">
         <v>0.318421</v>
       </c>
-      <c r="G54" s="29" t="n">
+      <c r="G54" s="63" t="n">
         <v>0.0005959735807338218</v>
       </c>
-      <c r="H54" s="24" t="inlineStr">
+      <c r="H54" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5325,19 +6577,19 @@
       <c r="C55" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D55" s="34" t="n">
+      <c r="D55" s="68" t="n">
         <v>0.318421</v>
       </c>
-      <c r="E55" s="34" t="n">
+      <c r="E55" s="68" t="n">
         <v>0.340789</v>
       </c>
-      <c r="F55" s="34" t="n">
+      <c r="F55" s="68" t="n">
         <v>0.340789</v>
       </c>
-      <c r="G55" s="29" t="n">
+      <c r="G55" s="63" t="n">
         <v>0.0005924567681126914</v>
       </c>
-      <c r="H55" s="24" t="inlineStr">
+      <c r="H55" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5357,19 +6609,19 @@
       <c r="C56" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D56" s="34" t="n">
+      <c r="D56" s="68" t="n">
         <v>0.273684</v>
       </c>
-      <c r="E56" s="34" t="n">
+      <c r="E56" s="68" t="n">
         <v>0.363158</v>
       </c>
-      <c r="F56" s="34" t="n">
+      <c r="F56" s="68" t="n">
         <v>0.363158</v>
       </c>
-      <c r="G56" s="29" t="n">
+      <c r="G56" s="63" t="n">
         <v>0.0005883103133506319</v>
       </c>
-      <c r="H56" s="24" t="inlineStr">
+      <c r="H56" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5389,19 +6641,19 @@
       <c r="C57" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D57" s="34" t="n">
+      <c r="D57" s="68" t="n">
         <v>0.228947</v>
       </c>
-      <c r="E57" s="34" t="n">
+      <c r="E57" s="68" t="n">
         <v>0.385526</v>
       </c>
-      <c r="F57" s="34" t="n">
+      <c r="F57" s="68" t="n">
         <v>0.385526</v>
       </c>
-      <c r="G57" s="29" t="n">
+      <c r="G57" s="63" t="n">
         <v>0.0005832970131890047</v>
       </c>
-      <c r="H57" s="24" t="inlineStr">
+      <c r="H57" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5421,19 +6673,19 @@
       <c r="C58" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D58" s="34" t="n">
+      <c r="D58" s="68" t="n">
         <v>0.184211</v>
       </c>
-      <c r="E58" s="34" t="n">
+      <c r="E58" s="68" t="n">
         <v>0.407895</v>
       </c>
-      <c r="F58" s="34" t="n">
+      <c r="F58" s="68" t="n">
         <v>0.407895</v>
       </c>
-      <c r="G58" s="29" t="n">
+      <c r="G58" s="63" t="n">
         <v>0.0005770442311225281</v>
       </c>
-      <c r="H58" s="24" t="inlineStr">
+      <c r="H58" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5453,19 +6705,19 @@
       <c r="C59" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D59" s="34" t="n">
+      <c r="D59" s="68" t="n">
         <v>0.139474</v>
       </c>
-      <c r="E59" s="34" t="n">
+      <c r="E59" s="68" t="n">
         <v>0.430263</v>
       </c>
-      <c r="F59" s="34" t="n">
+      <c r="F59" s="68" t="n">
         <v>0.430263</v>
       </c>
-      <c r="G59" s="29" t="n">
+      <c r="G59" s="63" t="n">
         <v>0.0005689524243180519</v>
       </c>
-      <c r="H59" s="24" t="inlineStr">
+      <c r="H59" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5485,19 +6737,19 @@
       <c r="C60" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D60" s="34" t="n">
+      <c r="D60" s="68" t="n">
         <v>0.094737</v>
       </c>
-      <c r="E60" s="34" t="n">
+      <c r="E60" s="68" t="n">
         <v>0.452632</v>
       </c>
-      <c r="F60" s="34" t="n">
+      <c r="F60" s="68" t="n">
         <v>0.452632</v>
       </c>
-      <c r="G60" s="29" t="n">
+      <c r="G60" s="63" t="n">
         <v>0.0005581573496582796</v>
       </c>
-      <c r="H60" s="24" t="inlineStr">
+      <c r="H60" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5517,19 +6769,19 @@
       <c r="C61" s="12" t="n">
         <v>1800</v>
       </c>
-      <c r="D61" s="34" t="n">
+      <c r="D61" s="68" t="n">
         <v>0.05</v>
       </c>
-      <c r="E61" s="34" t="n">
+      <c r="E61" s="68" t="n">
         <v>0.475</v>
       </c>
-      <c r="F61" s="34" t="n">
+      <c r="F61" s="68" t="n">
         <v>0.475</v>
       </c>
-      <c r="G61" s="29" t="n">
+      <c r="G61" s="63" t="n">
         <v>0.0005441813023263959</v>
       </c>
-      <c r="H61" s="24" t="inlineStr">
+      <c r="H61" s="58" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#3</t>
         </is>
@@ -5549,19 +6801,19 @@
       <c r="C62" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D62" s="35" t="n">
+      <c r="D62" s="69" t="n">
         <v>0.9</v>
       </c>
-      <c r="E62" s="35" t="n">
+      <c r="E62" s="69" t="n">
         <v>0.028571</v>
       </c>
-      <c r="F62" s="35" t="n">
+      <c r="F62" s="69" t="n">
         <v>0.07142900000000001</v>
       </c>
-      <c r="G62" s="31" t="n">
+      <c r="G62" s="65" t="n">
         <v>0.0006089752639324707</v>
       </c>
-      <c r="H62" s="25" t="inlineStr">
+      <c r="H62" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2; V3O5_HT#1</t>
         </is>
@@ -5581,19 +6833,19 @@
       <c r="C63" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D63" s="35" t="n">
+      <c r="D63" s="69" t="n">
         <v>0.855263</v>
       </c>
-      <c r="E63" s="35" t="n">
+      <c r="E63" s="69" t="n">
         <v>0.041353</v>
       </c>
-      <c r="F63" s="35" t="n">
+      <c r="F63" s="69" t="n">
         <v>0.103383</v>
       </c>
-      <c r="G63" s="31" t="n">
+      <c r="G63" s="65" t="n">
         <v>0.0006089752639324707</v>
       </c>
-      <c r="H63" s="25" t="inlineStr">
+      <c r="H63" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2; V3O5_HT#1</t>
         </is>
@@ -5613,19 +6865,19 @@
       <c r="C64" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D64" s="35" t="n">
+      <c r="D64" s="69" t="n">
         <v>0.810526</v>
       </c>
-      <c r="E64" s="35" t="n">
+      <c r="E64" s="69" t="n">
         <v>0.054135</v>
       </c>
-      <c r="F64" s="35" t="n">
+      <c r="F64" s="69" t="n">
         <v>0.135338</v>
       </c>
-      <c r="G64" s="31" t="n">
+      <c r="G64" s="65" t="n">
         <v>0.000608975263932468</v>
       </c>
-      <c r="H64" s="25" t="inlineStr">
+      <c r="H64" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2; V3O5_HT#1</t>
         </is>
@@ -5645,19 +6897,19 @@
       <c r="C65" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D65" s="35" t="n">
+      <c r="D65" s="69" t="n">
         <v>0.7657890000000001</v>
       </c>
-      <c r="E65" s="35" t="n">
+      <c r="E65" s="69" t="n">
         <v>0.066917</v>
       </c>
-      <c r="F65" s="35" t="n">
+      <c r="F65" s="69" t="n">
         <v>0.167293</v>
       </c>
-      <c r="G65" s="31" t="n">
+      <c r="G65" s="65" t="n">
         <v>0.0006089752639324696</v>
       </c>
-      <c r="H65" s="25" t="inlineStr">
+      <c r="H65" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2; V3O5_HT#1</t>
         </is>
@@ -5677,19 +6929,19 @@
       <c r="C66" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D66" s="35" t="n">
+      <c r="D66" s="69" t="n">
         <v>0.7210530000000001</v>
       </c>
-      <c r="E66" s="35" t="n">
+      <c r="E66" s="69" t="n">
         <v>0.07969900000000001</v>
       </c>
-      <c r="F66" s="35" t="n">
+      <c r="F66" s="69" t="n">
         <v>0.199248</v>
       </c>
-      <c r="G66" s="31" t="n">
+      <c r="G66" s="65" t="n">
         <v>0.0006086989931423054</v>
       </c>
-      <c r="H66" s="25" t="inlineStr">
+      <c r="H66" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5709,19 +6961,19 @@
       <c r="C67" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D67" s="35" t="n">
+      <c r="D67" s="69" t="n">
         <v>0.676316</v>
       </c>
-      <c r="E67" s="35" t="n">
+      <c r="E67" s="69" t="n">
         <v>0.09248099999999999</v>
       </c>
-      <c r="F67" s="35" t="n">
+      <c r="F67" s="69" t="n">
         <v>0.231203</v>
       </c>
-      <c r="G67" s="31" t="n">
+      <c r="G67" s="65" t="n">
         <v>0.0006075806595837329</v>
       </c>
-      <c r="H67" s="25" t="inlineStr">
+      <c r="H67" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5741,19 +6993,19 @@
       <c r="C68" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D68" s="35" t="n">
+      <c r="D68" s="69" t="n">
         <v>0.631579</v>
       </c>
-      <c r="E68" s="35" t="n">
+      <c r="E68" s="69" t="n">
         <v>0.105263</v>
       </c>
-      <c r="F68" s="35" t="n">
+      <c r="F68" s="69" t="n">
         <v>0.263158</v>
       </c>
-      <c r="G68" s="31" t="n">
+      <c r="G68" s="65" t="n">
         <v>0.0006066170076563114</v>
       </c>
-      <c r="H68" s="25" t="inlineStr">
+      <c r="H68" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5773,19 +7025,19 @@
       <c r="C69" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D69" s="35" t="n">
+      <c r="D69" s="69" t="n">
         <v>0.586842</v>
       </c>
-      <c r="E69" s="35" t="n">
+      <c r="E69" s="69" t="n">
         <v>0.118045</v>
       </c>
-      <c r="F69" s="35" t="n">
+      <c r="F69" s="69" t="n">
         <v>0.295113</v>
       </c>
-      <c r="G69" s="31" t="n">
+      <c r="G69" s="65" t="n">
         <v>0.0006057789423692359</v>
       </c>
-      <c r="H69" s="25" t="inlineStr">
+      <c r="H69" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5805,19 +7057,19 @@
       <c r="C70" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D70" s="35" t="n">
+      <c r="D70" s="69" t="n">
         <v>0.5421049999999999</v>
       </c>
-      <c r="E70" s="35" t="n">
+      <c r="E70" s="69" t="n">
         <v>0.130827</v>
       </c>
-      <c r="F70" s="35" t="n">
+      <c r="F70" s="69" t="n">
         <v>0.327068</v>
       </c>
-      <c r="G70" s="31" t="n">
+      <c r="G70" s="65" t="n">
         <v>0.0006050440821113034</v>
       </c>
-      <c r="H70" s="25" t="inlineStr">
+      <c r="H70" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5837,19 +7089,19 @@
       <c r="C71" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D71" s="35" t="n">
+      <c r="D71" s="69" t="n">
         <v>0.497368</v>
       </c>
-      <c r="E71" s="35" t="n">
+      <c r="E71" s="69" t="n">
         <v>0.143609</v>
       </c>
-      <c r="F71" s="35" t="n">
+      <c r="F71" s="69" t="n">
         <v>0.359023</v>
       </c>
-      <c r="G71" s="31" t="n">
+      <c r="G71" s="65" t="n">
         <v>0.0006043949529175177</v>
       </c>
-      <c r="H71" s="25" t="inlineStr">
+      <c r="H71" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5869,19 +7121,19 @@
       <c r="C72" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D72" s="35" t="n">
+      <c r="D72" s="69" t="n">
         <v>0.452632</v>
       </c>
-      <c r="E72" s="35" t="n">
+      <c r="E72" s="69" t="n">
         <v>0.156391</v>
       </c>
-      <c r="F72" s="35" t="n">
+      <c r="F72" s="69" t="n">
         <v>0.390977</v>
       </c>
-      <c r="G72" s="31" t="n">
+      <c r="G72" s="65" t="n">
         <v>0.0006038177336590362</v>
       </c>
-      <c r="H72" s="25" t="inlineStr">
+      <c r="H72" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5901,19 +7153,19 @@
       <c r="C73" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D73" s="35" t="n">
+      <c r="D73" s="69" t="n">
         <v>0.407895</v>
       </c>
-      <c r="E73" s="35" t="n">
+      <c r="E73" s="69" t="n">
         <v>0.169173</v>
       </c>
-      <c r="F73" s="35" t="n">
+      <c r="F73" s="69" t="n">
         <v>0.422932</v>
       </c>
-      <c r="G73" s="31" t="n">
+      <c r="G73" s="65" t="n">
         <v>0.0006033013642003349</v>
       </c>
-      <c r="H73" s="25" t="inlineStr">
+      <c r="H73" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5933,19 +7185,19 @@
       <c r="C74" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D74" s="35" t="n">
+      <c r="D74" s="69" t="n">
         <v>0.363158</v>
       </c>
-      <c r="E74" s="35" t="n">
+      <c r="E74" s="69" t="n">
         <v>0.181955</v>
       </c>
-      <c r="F74" s="35" t="n">
+      <c r="F74" s="69" t="n">
         <v>0.454887</v>
       </c>
-      <c r="G74" s="31" t="n">
+      <c r="G74" s="65" t="n">
         <v>0.0006028368997837505</v>
       </c>
-      <c r="H74" s="25" t="inlineStr">
+      <c r="H74" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5965,19 +7217,19 @@
       <c r="C75" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D75" s="35" t="n">
+      <c r="D75" s="69" t="n">
         <v>0.318421</v>
       </c>
-      <c r="E75" s="35" t="n">
+      <c r="E75" s="69" t="n">
         <v>0.194737</v>
       </c>
-      <c r="F75" s="35" t="n">
+      <c r="F75" s="69" t="n">
         <v>0.486842</v>
       </c>
-      <c r="G75" s="31" t="n">
+      <c r="G75" s="65" t="n">
         <v>0.0006024170362593856</v>
       </c>
-      <c r="H75" s="25" t="inlineStr">
+      <c r="H75" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -5997,19 +7249,19 @@
       <c r="C76" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D76" s="35" t="n">
+      <c r="D76" s="69" t="n">
         <v>0.273684</v>
       </c>
-      <c r="E76" s="35" t="n">
+      <c r="E76" s="69" t="n">
         <v>0.207519</v>
       </c>
-      <c r="F76" s="35" t="n">
+      <c r="F76" s="69" t="n">
         <v>0.518797</v>
       </c>
-      <c r="G76" s="31" t="n">
+      <c r="G76" s="65" t="n">
         <v>0.0006020357560719341</v>
       </c>
-      <c r="H76" s="25" t="inlineStr">
+      <c r="H76" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6029,19 +7281,19 @@
       <c r="C77" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D77" s="35" t="n">
+      <c r="D77" s="69" t="n">
         <v>0.228947</v>
       </c>
-      <c r="E77" s="35" t="n">
+      <c r="E77" s="69" t="n">
         <v>0.220301</v>
       </c>
-      <c r="F77" s="35" t="n">
+      <c r="F77" s="69" t="n">
         <v>0.550752</v>
       </c>
-      <c r="G77" s="31" t="n">
+      <c r="G77" s="65" t="n">
         <v>0.0006016880609681081</v>
       </c>
-      <c r="H77" s="25" t="inlineStr">
+      <c r="H77" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#1; IONIC_LIQ#2</t>
         </is>
@@ -6061,19 +7313,19 @@
       <c r="C78" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D78" s="35" t="n">
+      <c r="D78" s="69" t="n">
         <v>0.184211</v>
       </c>
-      <c r="E78" s="35" t="n">
+      <c r="E78" s="69" t="n">
         <v>0.233083</v>
       </c>
-      <c r="F78" s="35" t="n">
+      <c r="F78" s="69" t="n">
         <v>0.582707</v>
       </c>
-      <c r="G78" s="31" t="n">
+      <c r="G78" s="65" t="n">
         <v>0.0003420427646720472</v>
       </c>
-      <c r="H78" s="25" t="inlineStr">
+      <c r="H78" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#2</t>
         </is>
@@ -6093,19 +7345,19 @@
       <c r="C79" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D79" s="35" t="n">
+      <c r="D79" s="69" t="n">
         <v>0.139474</v>
       </c>
-      <c r="E79" s="35" t="n">
+      <c r="E79" s="69" t="n">
         <v>0.245865</v>
       </c>
-      <c r="F79" s="35" t="n">
+      <c r="F79" s="69" t="n">
         <v>0.614662</v>
       </c>
-      <c r="G79" s="31" t="n">
+      <c r="G79" s="65" t="n">
         <v>0.0001478601310591977</v>
       </c>
-      <c r="H79" s="25" t="inlineStr">
+      <c r="H79" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#2</t>
         </is>
@@ -6125,26 +7377,26 @@
       <c r="C80" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="D80" s="35" t="n">
+      <c r="D80" s="69" t="n">
         <v>0.094737</v>
       </c>
-      <c r="E80" s="35" t="n">
+      <c r="E80" s="69" t="n">
         <v>0.258647</v>
       </c>
-      <c r="F80" s="35" t="n">
+      <c r="F80" s="69" t="n">
         <v>0.646617</v>
       </c>
-      <c r="G80" s="31" t="n">
+      <c r="G80" s="65" t="n">
         <v>6.016951044280985e-05</v>
       </c>
-      <c r="H80" s="25" t="inlineStr">
+      <c r="H80" s="59" t="inlineStr">
         <is>
           <t>IONIC_LIQ#2</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="26" t="inlineStr">
+      <c r="A81" s="60" t="inlineStr">
         <is>
           <t>Cu-V-O</t>
         </is>
@@ -6157,19 +7409,19 @@
       <c r="C81" s="15" t="n">
         <v>1800</v>
       </c>
-      <c r="D81" s="36" t="n">
+      <c r="D81" s="70" t="n">
         <v>0.05</v>
       </c>
-      <c r="E81" s="36" t="n">
+      <c r="E81" s="70" t="n">
         <v>0.271429</v>
       </c>
-      <c r="F81" s="36" t="n">
+      <c r="F81" s="70" t="n">
         <v>0.678571</v>
       </c>
-      <c r="G81" s="33" t="n">
+      <c r="G81" s="67" t="n">
         <v>3.304376173394248e-05</v>
       </c>
-      <c r="H81" s="27" t="inlineStr">
+      <c r="H81" s="61" t="inlineStr">
         <is>
           <t>GAS#1; IONIC_LIQ#2</t>
         </is>
@@ -6180,7 +7432,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6244,7 +7496,7 @@
           <t>Fine-resolution dG vs T for top 6 ternary candidates (25 K steps, 800-1900 K)</t>
         </is>
       </c>
-      <c r="E2" s="24" t="inlineStr">
+      <c r="E2" s="58" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
@@ -6271,7 +7523,7 @@
           <t>CuFe2O4 formation decomposed into Cu-capture vs Fe-oxidation components (50 K steps, 800-1900 K)</t>
         </is>
       </c>
-      <c r="E3" s="25" t="inlineStr">
+      <c r="E3" s="59" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
@@ -6298,7 +7550,7 @@
           <t>Pre-computed Fe-oxidation and Cu-capture percentages</t>
         </is>
       </c>
-      <c r="E4" s="24" t="inlineStr">
+      <c r="E4" s="58" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
@@ -6325,7 +7577,7 @@
           <t>Cu activity in quaternary slag systems (Cu-Mn-Si-O, Cu-Al-Si-O) vs basicity ratio at 1800 K</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="59" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
@@ -6337,22 +7589,22 @@
           <t>cu_activity_vs_oxide.csv</t>
         </is>
       </c>
-      <c r="B6" s="37" t="inlineStr">
+      <c r="B6" s="45" t="inlineStr">
         <is>
           <t>simulations/tcpython/cu_activity_vs_oxide.py</t>
         </is>
       </c>
-      <c r="C6" s="37" t="inlineStr">
+      <c r="C6" s="45" t="inlineStr">
         <is>
           <t>TCOX14</t>
         </is>
       </c>
-      <c r="D6" s="37" t="inlineStr">
+      <c r="D6" s="45" t="inlineStr">
         <is>
           <t>Cu activity sweep at 1800 K across 4 ternary systems (Cu-Al-O, Cu-Mn-O, Cu-Fe-O, Cu-V-O), 20 compositions each</t>
         </is>
       </c>
-      <c r="E6" s="38" t="inlineStr">
+      <c r="E6" s="71" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>

</xml_diff>